<commit_message>
[FIX] - Bracket tab fully functionnal for solo generation except sort button | [ADD] - progress bar when generating files
</commit_message>
<xml_diff>
--- a/resources/template/rififi_bracket_solo_16.xlsx
+++ b/resources/template/rififi_bracket_solo_16.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hugor\GitHub\Asso\AssetsGenerator\resources\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7171D925-5790-4AC4-BB9A-DC09D2AB080F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71B8F226-4FFF-4343-82C4-8948BF67118F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="5250" windowWidth="29040" windowHeight="16440" xr2:uid="{2F0D60C5-63AA-4767-A59B-0FBF4FA7B0CE}"/>
   </bookViews>
@@ -1121,7 +1121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="176">
+  <cellXfs count="175">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1339,6 +1339,222 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="15" fillId="4" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1366,12 +1582,6 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="13" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1381,42 +1591,6 @@
     <xf numFmtId="0" fontId="3" fillId="13" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1434,183 +1608,6 @@
     </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="15" fillId="4" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2340,64 +2337,64 @@
       <c r="A1" s="84" t="s">
         <v>133</v>
       </c>
-      <c r="B1" s="174"/>
-      <c r="C1" s="157"/>
-      <c r="D1" s="157"/>
-      <c r="E1" s="157"/>
-      <c r="F1" s="157"/>
-      <c r="G1" s="157"/>
-      <c r="H1" s="157"/>
-      <c r="I1" s="157"/>
-      <c r="J1" s="157"/>
-      <c r="K1" s="157"/>
-      <c r="L1" s="157"/>
-      <c r="M1" s="157"/>
-      <c r="N1" s="157"/>
-      <c r="O1" s="157"/>
-      <c r="P1" s="157"/>
-      <c r="Q1" s="157"/>
-      <c r="R1" s="157"/>
-      <c r="S1" s="157"/>
-      <c r="T1" s="157"/>
-      <c r="U1" s="157"/>
-      <c r="V1" s="157"/>
-      <c r="W1" s="157"/>
-      <c r="X1" s="157"/>
-      <c r="Y1" s="157"/>
-      <c r="Z1" s="157"/>
-      <c r="AA1" s="157"/>
-      <c r="AB1" s="157"/>
-      <c r="AC1" s="157"/>
-      <c r="AD1" s="157"/>
-      <c r="AE1" s="157"/>
-      <c r="AF1" s="157"/>
-      <c r="AG1" s="157"/>
-      <c r="AH1" s="157"/>
-      <c r="AI1" s="157"/>
-      <c r="AJ1" s="157"/>
-      <c r="AK1" s="157"/>
-      <c r="AL1" s="157"/>
-      <c r="AM1" s="157"/>
-      <c r="AN1" s="157"/>
-      <c r="AO1" s="153"/>
+      <c r="B1" s="94"/>
+      <c r="C1" s="116"/>
+      <c r="D1" s="116"/>
+      <c r="E1" s="116"/>
+      <c r="F1" s="116"/>
+      <c r="G1" s="116"/>
+      <c r="H1" s="116"/>
+      <c r="I1" s="116"/>
+      <c r="J1" s="116"/>
+      <c r="K1" s="116"/>
+      <c r="L1" s="116"/>
+      <c r="M1" s="116"/>
+      <c r="N1" s="116"/>
+      <c r="O1" s="116"/>
+      <c r="P1" s="116"/>
+      <c r="Q1" s="116"/>
+      <c r="R1" s="116"/>
+      <c r="S1" s="116"/>
+      <c r="T1" s="116"/>
+      <c r="U1" s="116"/>
+      <c r="V1" s="116"/>
+      <c r="W1" s="116"/>
+      <c r="X1" s="116"/>
+      <c r="Y1" s="116"/>
+      <c r="Z1" s="116"/>
+      <c r="AA1" s="116"/>
+      <c r="AB1" s="116"/>
+      <c r="AC1" s="116"/>
+      <c r="AD1" s="116"/>
+      <c r="AE1" s="116"/>
+      <c r="AF1" s="116"/>
+      <c r="AG1" s="116"/>
+      <c r="AH1" s="116"/>
+      <c r="AI1" s="116"/>
+      <c r="AJ1" s="116"/>
+      <c r="AK1" s="116"/>
+      <c r="AL1" s="116"/>
+      <c r="AM1" s="116"/>
+      <c r="AN1" s="116"/>
+      <c r="AO1" s="112"/>
     </row>
     <row r="2" spans="1:41" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="84" t="s">
         <v>134</v>
       </c>
-      <c r="B2" s="175"/>
-      <c r="C2" s="111" t="s">
+      <c r="B2" s="95"/>
+      <c r="C2" s="169" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="112"/>
-      <c r="E2" s="112"/>
-      <c r="F2" s="112"/>
-      <c r="G2" s="112"/>
-      <c r="H2" s="112"/>
-      <c r="I2" s="112"/>
-      <c r="J2" s="112"/>
-      <c r="K2" s="112"/>
-      <c r="L2" s="161"/>
+      <c r="D2" s="170"/>
+      <c r="E2" s="170"/>
+      <c r="F2" s="170"/>
+      <c r="G2" s="170"/>
+      <c r="H2" s="170"/>
+      <c r="I2" s="170"/>
+      <c r="J2" s="170"/>
+      <c r="K2" s="170"/>
+      <c r="L2" s="117"/>
       <c r="M2" s="37"/>
       <c r="N2" s="37"/>
       <c r="O2" s="37"/>
@@ -2417,7 +2414,7 @@
       <c r="AC2" s="38"/>
       <c r="AD2" s="38"/>
       <c r="AE2" s="38"/>
-      <c r="AF2" s="96"/>
+      <c r="AF2" s="166"/>
       <c r="AG2" s="38"/>
       <c r="AH2" s="38"/>
       <c r="AI2" s="38"/>
@@ -2426,23 +2423,23 @@
       <c r="AL2" s="38"/>
       <c r="AM2" s="38"/>
       <c r="AN2" s="39"/>
-      <c r="AO2" s="154"/>
+      <c r="AO2" s="113"/>
     </row>
     <row r="3" spans="1:41" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="84" t="s">
         <v>131</v>
       </c>
-      <c r="B3" s="175"/>
-      <c r="C3" s="113"/>
-      <c r="D3" s="114"/>
-      <c r="E3" s="114"/>
-      <c r="F3" s="114"/>
-      <c r="G3" s="114"/>
-      <c r="H3" s="114"/>
-      <c r="I3" s="114"/>
-      <c r="J3" s="114"/>
-      <c r="K3" s="114"/>
-      <c r="L3" s="162"/>
+      <c r="B3" s="95"/>
+      <c r="C3" s="171"/>
+      <c r="D3" s="172"/>
+      <c r="E3" s="172"/>
+      <c r="F3" s="172"/>
+      <c r="G3" s="172"/>
+      <c r="H3" s="172"/>
+      <c r="I3" s="172"/>
+      <c r="J3" s="172"/>
+      <c r="K3" s="172"/>
+      <c r="L3" s="118"/>
       <c r="M3" s="70"/>
       <c r="N3" s="70"/>
       <c r="O3" s="70"/>
@@ -2462,7 +2459,7 @@
       <c r="AC3" s="71"/>
       <c r="AD3" s="71"/>
       <c r="AE3" s="71"/>
-      <c r="AF3" s="97"/>
+      <c r="AF3" s="167"/>
       <c r="AG3" s="71"/>
       <c r="AH3" s="71"/>
       <c r="AI3" s="71"/>
@@ -2471,23 +2468,23 @@
       <c r="AL3" s="71"/>
       <c r="AM3" s="71"/>
       <c r="AN3" s="40"/>
-      <c r="AO3" s="154"/>
+      <c r="AO3" s="113"/>
     </row>
     <row r="4" spans="1:41" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="84" t="s">
         <v>130</v>
       </c>
-      <c r="B4" s="175"/>
-      <c r="C4" s="113"/>
-      <c r="D4" s="114"/>
-      <c r="E4" s="114"/>
-      <c r="F4" s="114"/>
-      <c r="G4" s="114"/>
-      <c r="H4" s="114"/>
-      <c r="I4" s="114"/>
-      <c r="J4" s="114"/>
-      <c r="K4" s="114"/>
-      <c r="L4" s="162"/>
+      <c r="B4" s="95"/>
+      <c r="C4" s="171"/>
+      <c r="D4" s="172"/>
+      <c r="E4" s="172"/>
+      <c r="F4" s="172"/>
+      <c r="G4" s="172"/>
+      <c r="H4" s="172"/>
+      <c r="I4" s="172"/>
+      <c r="J4" s="172"/>
+      <c r="K4" s="172"/>
+      <c r="L4" s="118"/>
       <c r="M4" s="71"/>
       <c r="N4" s="71"/>
       <c r="O4" s="71"/>
@@ -2507,7 +2504,7 @@
       <c r="AC4" s="71"/>
       <c r="AD4" s="71"/>
       <c r="AE4" s="71"/>
-      <c r="AF4" s="97"/>
+      <c r="AF4" s="167"/>
       <c r="AG4" s="71"/>
       <c r="AH4" s="71"/>
       <c r="AI4" s="71"/>
@@ -2516,167 +2513,166 @@
       <c r="AL4" s="71"/>
       <c r="AM4" s="71"/>
       <c r="AN4" s="40"/>
-      <c r="AO4" s="154"/>
+      <c r="AO4" s="113"/>
     </row>
     <row r="5" spans="1:41" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="84" t="s">
         <v>132</v>
       </c>
-      <c r="B5" s="175"/>
-      <c r="C5" s="113"/>
-      <c r="D5" s="114"/>
-      <c r="E5" s="114"/>
-      <c r="F5" s="114"/>
-      <c r="G5" s="114"/>
-      <c r="H5" s="114"/>
-      <c r="I5" s="114"/>
-      <c r="J5" s="114"/>
-      <c r="K5" s="114"/>
-      <c r="L5" s="162"/>
-      <c r="M5" s="123" t="s">
+      <c r="B5" s="95"/>
+      <c r="C5" s="171"/>
+      <c r="D5" s="172"/>
+      <c r="E5" s="172"/>
+      <c r="F5" s="172"/>
+      <c r="G5" s="172"/>
+      <c r="H5" s="172"/>
+      <c r="I5" s="172"/>
+      <c r="J5" s="172"/>
+      <c r="K5" s="172"/>
+      <c r="L5" s="118"/>
+      <c r="M5" s="143" t="s">
         <v>42</v>
       </c>
-      <c r="N5" s="124"/>
-      <c r="O5" s="124"/>
-      <c r="P5" s="124"/>
-      <c r="Q5" s="124"/>
-      <c r="R5" s="124"/>
-      <c r="S5" s="124"/>
-      <c r="T5" s="124"/>
-      <c r="U5" s="124"/>
-      <c r="V5" s="124"/>
-      <c r="W5" s="124"/>
-      <c r="X5" s="124"/>
-      <c r="Y5" s="124"/>
-      <c r="Z5" s="124"/>
-      <c r="AA5" s="124"/>
-      <c r="AB5" s="124"/>
-      <c r="AC5" s="124"/>
-      <c r="AD5" s="124"/>
-      <c r="AE5" s="125"/>
-      <c r="AF5" s="97"/>
-      <c r="AG5" s="165" t="s">
+      <c r="N5" s="144"/>
+      <c r="O5" s="144"/>
+      <c r="P5" s="144"/>
+      <c r="Q5" s="144"/>
+      <c r="R5" s="144"/>
+      <c r="S5" s="144"/>
+      <c r="T5" s="144"/>
+      <c r="U5" s="144"/>
+      <c r="V5" s="144"/>
+      <c r="W5" s="144"/>
+      <c r="X5" s="144"/>
+      <c r="Y5" s="144"/>
+      <c r="Z5" s="144"/>
+      <c r="AA5" s="144"/>
+      <c r="AB5" s="144"/>
+      <c r="AC5" s="144"/>
+      <c r="AD5" s="144"/>
+      <c r="AE5" s="145"/>
+      <c r="AF5" s="167"/>
+      <c r="AG5" s="85" t="s">
         <v>140</v>
       </c>
-      <c r="AH5" s="166"/>
-      <c r="AI5" s="166"/>
-      <c r="AJ5" s="166"/>
-      <c r="AK5" s="166"/>
-      <c r="AL5" s="166"/>
-      <c r="AM5" s="166"/>
-      <c r="AN5" s="167"/>
-      <c r="AO5" s="154"/>
+      <c r="AH5" s="86"/>
+      <c r="AI5" s="86"/>
+      <c r="AJ5" s="86"/>
+      <c r="AK5" s="86"/>
+      <c r="AL5" s="86"/>
+      <c r="AM5" s="86"/>
+      <c r="AN5" s="87"/>
+      <c r="AO5" s="113"/>
     </row>
     <row r="6" spans="1:41" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="84" t="s">
         <v>162</v>
       </c>
-      <c r="B6" s="175"/>
-      <c r="C6" s="115"/>
-      <c r="D6" s="116"/>
-      <c r="E6" s="116"/>
-      <c r="F6" s="116"/>
-      <c r="G6" s="116"/>
-      <c r="H6" s="116"/>
-      <c r="I6" s="116"/>
-      <c r="J6" s="116"/>
-      <c r="K6" s="116"/>
-      <c r="L6" s="162"/>
-      <c r="M6" s="126"/>
-      <c r="N6" s="127"/>
-      <c r="O6" s="127"/>
-      <c r="P6" s="127"/>
-      <c r="Q6" s="127"/>
-      <c r="R6" s="127"/>
-      <c r="S6" s="127"/>
-      <c r="T6" s="127"/>
-      <c r="U6" s="127"/>
-      <c r="V6" s="127"/>
-      <c r="W6" s="127"/>
-      <c r="X6" s="127"/>
-      <c r="Y6" s="127"/>
-      <c r="Z6" s="127"/>
-      <c r="AA6" s="127"/>
-      <c r="AB6" s="127"/>
-      <c r="AC6" s="127"/>
-      <c r="AD6" s="127"/>
-      <c r="AE6" s="128"/>
-      <c r="AF6" s="97"/>
-      <c r="AG6" s="168"/>
-      <c r="AH6" s="169"/>
-      <c r="AI6" s="169"/>
-      <c r="AJ6" s="169"/>
-      <c r="AK6" s="169"/>
-      <c r="AL6" s="169"/>
-      <c r="AM6" s="169"/>
-      <c r="AN6" s="170"/>
-      <c r="AO6" s="154"/>
+      <c r="B6" s="95"/>
+      <c r="C6" s="173"/>
+      <c r="D6" s="174"/>
+      <c r="E6" s="174"/>
+      <c r="F6" s="174"/>
+      <c r="G6" s="174"/>
+      <c r="H6" s="174"/>
+      <c r="I6" s="174"/>
+      <c r="J6" s="174"/>
+      <c r="K6" s="174"/>
+      <c r="L6" s="118"/>
+      <c r="M6" s="146"/>
+      <c r="N6" s="147"/>
+      <c r="O6" s="147"/>
+      <c r="P6" s="147"/>
+      <c r="Q6" s="147"/>
+      <c r="R6" s="147"/>
+      <c r="S6" s="147"/>
+      <c r="T6" s="147"/>
+      <c r="U6" s="147"/>
+      <c r="V6" s="147"/>
+      <c r="W6" s="147"/>
+      <c r="X6" s="147"/>
+      <c r="Y6" s="147"/>
+      <c r="Z6" s="147"/>
+      <c r="AA6" s="147"/>
+      <c r="AB6" s="147"/>
+      <c r="AC6" s="147"/>
+      <c r="AD6" s="147"/>
+      <c r="AE6" s="148"/>
+      <c r="AF6" s="167"/>
+      <c r="AG6" s="88"/>
+      <c r="AH6" s="89"/>
+      <c r="AI6" s="89"/>
+      <c r="AJ6" s="89"/>
+      <c r="AK6" s="89"/>
+      <c r="AL6" s="89"/>
+      <c r="AM6" s="89"/>
+      <c r="AN6" s="90"/>
+      <c r="AO6" s="113"/>
     </row>
     <row r="7" spans="1:41" ht="39.950000000000003" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="84" t="s">
         <v>112</v>
       </c>
-      <c r="B7" s="175"/>
+      <c r="B7" s="95"/>
       <c r="C7" s="68"/>
-      <c r="D7" s="122" t="s">
+      <c r="D7" s="156" t="s">
         <v>141</v>
       </c>
-      <c r="E7" s="122"/>
-      <c r="F7" s="122"/>
-      <c r="G7" s="122"/>
-      <c r="H7" s="122"/>
-      <c r="I7" s="120" t="str">
-        <f>"01/01/2025"</f>
-        <v>01/01/2025</v>
-      </c>
-      <c r="J7" s="121"/>
+      <c r="E7" s="156"/>
+      <c r="F7" s="156"/>
+      <c r="G7" s="156"/>
+      <c r="H7" s="156"/>
+      <c r="I7" s="155">
+        <v>45658</v>
+      </c>
+      <c r="J7" s="155"/>
       <c r="K7" s="69"/>
-      <c r="L7" s="162"/>
-      <c r="M7" s="129"/>
-      <c r="N7" s="130"/>
-      <c r="O7" s="130"/>
-      <c r="P7" s="130"/>
-      <c r="Q7" s="130"/>
-      <c r="R7" s="130"/>
-      <c r="S7" s="130"/>
-      <c r="T7" s="130"/>
-      <c r="U7" s="130"/>
-      <c r="V7" s="130"/>
-      <c r="W7" s="130"/>
-      <c r="X7" s="130"/>
-      <c r="Y7" s="130"/>
-      <c r="Z7" s="130"/>
-      <c r="AA7" s="130"/>
-      <c r="AB7" s="130"/>
-      <c r="AC7" s="130"/>
-      <c r="AD7" s="130"/>
-      <c r="AE7" s="131"/>
-      <c r="AF7" s="97"/>
-      <c r="AG7" s="171"/>
-      <c r="AH7" s="172"/>
-      <c r="AI7" s="172"/>
-      <c r="AJ7" s="172"/>
-      <c r="AK7" s="172"/>
-      <c r="AL7" s="172"/>
-      <c r="AM7" s="172"/>
-      <c r="AN7" s="173"/>
-      <c r="AO7" s="154"/>
+      <c r="L7" s="118"/>
+      <c r="M7" s="149"/>
+      <c r="N7" s="150"/>
+      <c r="O7" s="150"/>
+      <c r="P7" s="150"/>
+      <c r="Q7" s="150"/>
+      <c r="R7" s="150"/>
+      <c r="S7" s="150"/>
+      <c r="T7" s="150"/>
+      <c r="U7" s="150"/>
+      <c r="V7" s="150"/>
+      <c r="W7" s="150"/>
+      <c r="X7" s="150"/>
+      <c r="Y7" s="150"/>
+      <c r="Z7" s="150"/>
+      <c r="AA7" s="150"/>
+      <c r="AB7" s="150"/>
+      <c r="AC7" s="150"/>
+      <c r="AD7" s="150"/>
+      <c r="AE7" s="151"/>
+      <c r="AF7" s="167"/>
+      <c r="AG7" s="91"/>
+      <c r="AH7" s="92"/>
+      <c r="AI7" s="92"/>
+      <c r="AJ7" s="92"/>
+      <c r="AK7" s="92"/>
+      <c r="AL7" s="92"/>
+      <c r="AM7" s="92"/>
+      <c r="AN7" s="93"/>
+      <c r="AO7" s="113"/>
     </row>
     <row r="8" spans="1:41" ht="5.0999999999999996" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A8" s="84" t="s">
         <v>119</v>
       </c>
-      <c r="B8" s="175"/>
-      <c r="C8" s="118"/>
-      <c r="D8" s="119"/>
-      <c r="E8" s="119"/>
-      <c r="F8" s="119"/>
-      <c r="G8" s="119"/>
-      <c r="H8" s="119"/>
-      <c r="I8" s="119"/>
-      <c r="J8" s="119"/>
-      <c r="K8" s="119"/>
-      <c r="L8" s="162"/>
+      <c r="B8" s="95"/>
+      <c r="C8" s="153"/>
+      <c r="D8" s="154"/>
+      <c r="E8" s="154"/>
+      <c r="F8" s="154"/>
+      <c r="G8" s="154"/>
+      <c r="H8" s="154"/>
+      <c r="I8" s="154"/>
+      <c r="J8" s="154"/>
+      <c r="K8" s="154"/>
+      <c r="L8" s="118"/>
       <c r="M8" s="71"/>
       <c r="N8" s="71"/>
       <c r="O8" s="71"/>
@@ -2696,7 +2692,7 @@
       <c r="AC8" s="71"/>
       <c r="AD8" s="71"/>
       <c r="AE8" s="71"/>
-      <c r="AF8" s="97"/>
+      <c r="AF8" s="167"/>
       <c r="AG8" s="71"/>
       <c r="AH8" s="71"/>
       <c r="AI8" s="71"/>
@@ -2705,23 +2701,23 @@
       <c r="AL8" s="71"/>
       <c r="AM8" s="71"/>
       <c r="AN8" s="40"/>
-      <c r="AO8" s="154"/>
+      <c r="AO8" s="113"/>
     </row>
     <row r="9" spans="1:41" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="84" t="s">
         <v>115</v>
       </c>
-      <c r="B9" s="175"/>
+      <c r="B9" s="95"/>
       <c r="C9" s="41"/>
-      <c r="D9" s="117"/>
-      <c r="E9" s="117"/>
+      <c r="D9" s="152"/>
+      <c r="E9" s="152"/>
       <c r="F9" s="72"/>
       <c r="G9" s="73"/>
-      <c r="H9" s="117"/>
-      <c r="I9" s="117"/>
-      <c r="J9" s="117"/>
+      <c r="H9" s="152"/>
+      <c r="I9" s="152"/>
+      <c r="J9" s="152"/>
       <c r="K9" s="71"/>
-      <c r="L9" s="162"/>
+      <c r="L9" s="118"/>
       <c r="M9" s="71"/>
       <c r="N9" s="71"/>
       <c r="O9" s="71"/>
@@ -2741,7 +2737,7 @@
       <c r="AC9" s="71"/>
       <c r="AD9" s="71"/>
       <c r="AE9" s="71"/>
-      <c r="AF9" s="97"/>
+      <c r="AF9" s="167"/>
       <c r="AG9" s="71"/>
       <c r="AH9" s="71"/>
       <c r="AI9" s="71"/>
@@ -2750,13 +2746,13 @@
       <c r="AL9" s="71"/>
       <c r="AM9" s="71"/>
       <c r="AN9" s="40"/>
-      <c r="AO9" s="154"/>
+      <c r="AO9" s="113"/>
     </row>
     <row r="10" spans="1:41" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="84" t="s">
         <v>114</v>
       </c>
-      <c r="B10" s="175"/>
+      <c r="B10" s="95"/>
       <c r="C10" s="41"/>
       <c r="D10" s="71"/>
       <c r="E10" s="73"/>
@@ -2766,7 +2762,7 @@
       <c r="I10" s="71"/>
       <c r="J10" s="71"/>
       <c r="K10" s="71"/>
-      <c r="L10" s="162"/>
+      <c r="L10" s="118"/>
       <c r="M10" s="71"/>
       <c r="N10" s="71"/>
       <c r="O10" s="71"/>
@@ -2786,7 +2782,7 @@
       <c r="AC10" s="71"/>
       <c r="AD10" s="71"/>
       <c r="AE10" s="71"/>
-      <c r="AF10" s="97"/>
+      <c r="AF10" s="167"/>
       <c r="AG10" s="71"/>
       <c r="AH10" s="71"/>
       <c r="AI10" s="71"/>
@@ -2795,13 +2791,13 @@
       <c r="AL10" s="71"/>
       <c r="AM10" s="71"/>
       <c r="AN10" s="40"/>
-      <c r="AO10" s="154"/>
+      <c r="AO10" s="113"/>
     </row>
     <row r="11" spans="1:41" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="84" t="s">
         <v>116</v>
       </c>
-      <c r="B11" s="175"/>
+      <c r="B11" s="95"/>
       <c r="C11" s="41"/>
       <c r="D11" s="71"/>
       <c r="E11" s="73"/>
@@ -2811,50 +2807,50 @@
       <c r="I11" s="71"/>
       <c r="J11" s="71"/>
       <c r="K11" s="71"/>
-      <c r="L11" s="162"/>
-      <c r="M11" s="103" t="s">
+      <c r="L11" s="118"/>
+      <c r="M11" s="121" t="s">
         <v>38</v>
       </c>
-      <c r="N11" s="103"/>
-      <c r="O11" s="103"/>
-      <c r="P11" s="103"/>
-      <c r="Q11" s="103"/>
-      <c r="R11" s="103"/>
-      <c r="S11" s="104"/>
+      <c r="N11" s="121"/>
+      <c r="O11" s="121"/>
+      <c r="P11" s="121"/>
+      <c r="Q11" s="121"/>
+      <c r="R11" s="121"/>
+      <c r="S11" s="122"/>
       <c r="T11" s="71"/>
-      <c r="U11" s="102" t="s">
+      <c r="U11" s="120" t="s">
         <v>45</v>
       </c>
-      <c r="V11" s="103"/>
-      <c r="W11" s="103"/>
-      <c r="X11" s="103"/>
-      <c r="Y11" s="104"/>
+      <c r="V11" s="121"/>
+      <c r="W11" s="121"/>
+      <c r="X11" s="121"/>
+      <c r="Y11" s="122"/>
       <c r="Z11" s="71"/>
-      <c r="AA11" s="102" t="s">
+      <c r="AA11" s="120" t="s">
         <v>41</v>
       </c>
-      <c r="AB11" s="103"/>
-      <c r="AC11" s="103"/>
-      <c r="AD11" s="103"/>
-      <c r="AE11" s="103"/>
-      <c r="AF11" s="97"/>
+      <c r="AB11" s="121"/>
+      <c r="AC11" s="121"/>
+      <c r="AD11" s="121"/>
+      <c r="AE11" s="121"/>
+      <c r="AF11" s="167"/>
       <c r="AG11" s="71"/>
-      <c r="AH11" s="102" t="s">
+      <c r="AH11" s="120" t="s">
         <v>54</v>
       </c>
-      <c r="AI11" s="103"/>
-      <c r="AJ11" s="103"/>
-      <c r="AK11" s="103"/>
-      <c r="AL11" s="103"/>
-      <c r="AM11" s="104"/>
+      <c r="AI11" s="121"/>
+      <c r="AJ11" s="121"/>
+      <c r="AK11" s="121"/>
+      <c r="AL11" s="121"/>
+      <c r="AM11" s="122"/>
       <c r="AN11" s="40"/>
-      <c r="AO11" s="154"/>
+      <c r="AO11" s="113"/>
     </row>
     <row r="12" spans="1:41" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="84" t="s">
         <v>118</v>
       </c>
-      <c r="B12" s="175"/>
+      <c r="B12" s="95"/>
       <c r="C12" s="41"/>
       <c r="D12" s="71"/>
       <c r="E12" s="73"/>
@@ -2864,101 +2860,101 @@
       <c r="I12" s="71"/>
       <c r="J12" s="71"/>
       <c r="K12" s="71"/>
-      <c r="L12" s="162"/>
-      <c r="M12" s="106"/>
-      <c r="N12" s="106"/>
-      <c r="O12" s="106"/>
-      <c r="P12" s="106"/>
-      <c r="Q12" s="106"/>
-      <c r="R12" s="106"/>
-      <c r="S12" s="107"/>
+      <c r="L12" s="118"/>
+      <c r="M12" s="124"/>
+      <c r="N12" s="124"/>
+      <c r="O12" s="124"/>
+      <c r="P12" s="124"/>
+      <c r="Q12" s="124"/>
+      <c r="R12" s="124"/>
+      <c r="S12" s="125"/>
       <c r="T12" s="71"/>
-      <c r="U12" s="105"/>
-      <c r="V12" s="106"/>
-      <c r="W12" s="106"/>
-      <c r="X12" s="106"/>
-      <c r="Y12" s="107"/>
+      <c r="U12" s="123"/>
+      <c r="V12" s="124"/>
+      <c r="W12" s="124"/>
+      <c r="X12" s="124"/>
+      <c r="Y12" s="125"/>
       <c r="Z12" s="71"/>
-      <c r="AA12" s="105"/>
-      <c r="AB12" s="106"/>
-      <c r="AC12" s="106"/>
-      <c r="AD12" s="106"/>
-      <c r="AE12" s="106"/>
-      <c r="AF12" s="97"/>
+      <c r="AA12" s="123"/>
+      <c r="AB12" s="124"/>
+      <c r="AC12" s="124"/>
+      <c r="AD12" s="124"/>
+      <c r="AE12" s="124"/>
+      <c r="AF12" s="167"/>
       <c r="AG12" s="71"/>
-      <c r="AH12" s="105"/>
-      <c r="AI12" s="106"/>
-      <c r="AJ12" s="106"/>
-      <c r="AK12" s="106"/>
-      <c r="AL12" s="106"/>
-      <c r="AM12" s="107"/>
+      <c r="AH12" s="123"/>
+      <c r="AI12" s="124"/>
+      <c r="AJ12" s="124"/>
+      <c r="AK12" s="124"/>
+      <c r="AL12" s="124"/>
+      <c r="AM12" s="125"/>
       <c r="AN12" s="40"/>
-      <c r="AO12" s="154"/>
+      <c r="AO12" s="113"/>
     </row>
     <row r="13" spans="1:41" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="84" t="s">
         <v>120</v>
       </c>
-      <c r="B13" s="175"/>
+      <c r="B13" s="95"/>
       <c r="C13" s="41"/>
-      <c r="D13" s="85" t="s">
+      <c r="D13" s="157" t="s">
         <v>2</v>
       </c>
-      <c r="E13" s="87"/>
+      <c r="E13" s="159"/>
       <c r="F13" s="72"/>
       <c r="G13" s="73"/>
-      <c r="H13" s="85" t="s">
+      <c r="H13" s="157" t="s">
         <v>139</v>
       </c>
-      <c r="I13" s="86"/>
-      <c r="J13" s="87"/>
+      <c r="I13" s="158"/>
+      <c r="J13" s="159"/>
       <c r="K13" s="71"/>
-      <c r="L13" s="162"/>
-      <c r="M13" s="109"/>
-      <c r="N13" s="109"/>
-      <c r="O13" s="109"/>
-      <c r="P13" s="109"/>
-      <c r="Q13" s="109"/>
-      <c r="R13" s="109"/>
-      <c r="S13" s="110"/>
+      <c r="L13" s="118"/>
+      <c r="M13" s="127"/>
+      <c r="N13" s="127"/>
+      <c r="O13" s="127"/>
+      <c r="P13" s="127"/>
+      <c r="Q13" s="127"/>
+      <c r="R13" s="127"/>
+      <c r="S13" s="128"/>
       <c r="T13" s="71"/>
-      <c r="U13" s="108"/>
-      <c r="V13" s="109"/>
-      <c r="W13" s="109"/>
-      <c r="X13" s="109"/>
-      <c r="Y13" s="110"/>
+      <c r="U13" s="126"/>
+      <c r="V13" s="127"/>
+      <c r="W13" s="127"/>
+      <c r="X13" s="127"/>
+      <c r="Y13" s="128"/>
       <c r="Z13" s="71"/>
-      <c r="AA13" s="108"/>
-      <c r="AB13" s="109"/>
-      <c r="AC13" s="109"/>
-      <c r="AD13" s="109"/>
-      <c r="AE13" s="109"/>
-      <c r="AF13" s="97"/>
+      <c r="AA13" s="126"/>
+      <c r="AB13" s="127"/>
+      <c r="AC13" s="127"/>
+      <c r="AD13" s="127"/>
+      <c r="AE13" s="127"/>
+      <c r="AF13" s="167"/>
       <c r="AG13" s="71"/>
-      <c r="AH13" s="108"/>
-      <c r="AI13" s="109"/>
-      <c r="AJ13" s="109"/>
-      <c r="AK13" s="109"/>
-      <c r="AL13" s="109"/>
-      <c r="AM13" s="110"/>
+      <c r="AH13" s="126"/>
+      <c r="AI13" s="127"/>
+      <c r="AJ13" s="127"/>
+      <c r="AK13" s="127"/>
+      <c r="AL13" s="127"/>
+      <c r="AM13" s="128"/>
       <c r="AN13" s="40"/>
-      <c r="AO13" s="154"/>
+      <c r="AO13" s="113"/>
     </row>
     <row r="14" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="84" t="s">
         <v>113</v>
       </c>
-      <c r="B14" s="175"/>
+      <c r="B14" s="95"/>
       <c r="C14" s="41"/>
-      <c r="D14" s="88"/>
-      <c r="E14" s="91"/>
+      <c r="D14" s="160"/>
+      <c r="E14" s="163"/>
       <c r="F14" s="72"/>
       <c r="G14" s="73"/>
-      <c r="H14" s="88"/>
-      <c r="I14" s="89"/>
-      <c r="J14" s="90"/>
+      <c r="H14" s="160"/>
+      <c r="I14" s="161"/>
+      <c r="J14" s="162"/>
       <c r="K14" s="71"/>
-      <c r="L14" s="162"/>
+      <c r="L14" s="118"/>
       <c r="M14" s="74"/>
       <c r="N14" s="74"/>
       <c r="O14" s="74"/>
@@ -2967,33 +2963,33 @@
       <c r="R14" s="74"/>
       <c r="S14" s="3"/>
       <c r="T14" s="71"/>
-      <c r="U14" s="134"/>
-      <c r="V14" s="132"/>
-      <c r="W14" s="132"/>
-      <c r="X14" s="132"/>
-      <c r="Y14" s="133"/>
+      <c r="U14" s="104"/>
+      <c r="V14" s="105"/>
+      <c r="W14" s="105"/>
+      <c r="X14" s="105"/>
+      <c r="Y14" s="107"/>
       <c r="Z14" s="71"/>
-      <c r="AA14" s="134"/>
-      <c r="AB14" s="132"/>
-      <c r="AC14" s="132"/>
-      <c r="AD14" s="132"/>
-      <c r="AE14" s="132"/>
-      <c r="AF14" s="97"/>
+      <c r="AA14" s="104"/>
+      <c r="AB14" s="105"/>
+      <c r="AC14" s="105"/>
+      <c r="AD14" s="105"/>
+      <c r="AE14" s="105"/>
+      <c r="AF14" s="167"/>
       <c r="AG14" s="71"/>
-      <c r="AH14" s="134"/>
-      <c r="AI14" s="132"/>
-      <c r="AJ14" s="132"/>
-      <c r="AK14" s="132"/>
-      <c r="AL14" s="132"/>
-      <c r="AM14" s="133"/>
+      <c r="AH14" s="104"/>
+      <c r="AI14" s="105"/>
+      <c r="AJ14" s="105"/>
+      <c r="AK14" s="105"/>
+      <c r="AL14" s="105"/>
+      <c r="AM14" s="107"/>
       <c r="AN14" s="40"/>
-      <c r="AO14" s="154"/>
+      <c r="AO14" s="113"/>
     </row>
     <row r="15" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="84" t="s">
         <v>117</v>
       </c>
-      <c r="B15" s="175"/>
+      <c r="B15" s="95"/>
       <c r="C15" s="41"/>
       <c r="D15" s="65" t="s">
         <v>3</v>
@@ -3014,58 +3010,58 @@
         <v>19</v>
       </c>
       <c r="K15" s="71"/>
-      <c r="L15" s="162"/>
-      <c r="M15" s="150"/>
+      <c r="L15" s="118"/>
+      <c r="M15" s="111"/>
       <c r="N15" s="75"/>
       <c r="O15" s="75"/>
       <c r="P15" s="5">
         <v>4</v>
       </c>
-      <c r="Q15" s="94" t="s">
+      <c r="Q15" s="138" t="s">
         <v>31</v>
       </c>
-      <c r="R15" s="95"/>
-      <c r="S15" s="147"/>
+      <c r="R15" s="139"/>
+      <c r="S15" s="96"/>
       <c r="T15" s="71"/>
-      <c r="U15" s="147"/>
+      <c r="U15" s="96"/>
       <c r="V15" s="5">
         <v>4</v>
       </c>
-      <c r="W15" s="94" t="s">
+      <c r="W15" s="138" t="s">
         <v>31</v>
       </c>
-      <c r="X15" s="95"/>
-      <c r="Y15" s="147"/>
+      <c r="X15" s="139"/>
+      <c r="Y15" s="96"/>
       <c r="Z15" s="71"/>
-      <c r="AA15" s="147"/>
+      <c r="AA15" s="96"/>
       <c r="AB15" s="5">
         <v>6</v>
       </c>
-      <c r="AC15" s="94" t="s">
+      <c r="AC15" s="138" t="s">
         <v>31</v>
       </c>
-      <c r="AD15" s="95"/>
-      <c r="AE15" s="158"/>
-      <c r="AF15" s="97"/>
+      <c r="AD15" s="139"/>
+      <c r="AE15" s="108"/>
+      <c r="AF15" s="167"/>
       <c r="AG15" s="71"/>
-      <c r="AH15" s="147"/>
+      <c r="AH15" s="96"/>
       <c r="AI15" s="5">
         <v>8</v>
       </c>
-      <c r="AJ15" s="92" t="s">
+      <c r="AJ15" s="164" t="s">
         <v>31</v>
       </c>
-      <c r="AK15" s="92"/>
-      <c r="AL15" s="93"/>
-      <c r="AM15" s="147"/>
+      <c r="AK15" s="164"/>
+      <c r="AL15" s="165"/>
+      <c r="AM15" s="96"/>
       <c r="AN15" s="40"/>
-      <c r="AO15" s="154"/>
+      <c r="AO15" s="113"/>
     </row>
     <row r="16" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="84" t="s">
         <v>163</v>
       </c>
-      <c r="B16" s="175"/>
+      <c r="B16" s="95"/>
       <c r="C16" s="41"/>
       <c r="D16" s="66" t="s">
         <v>4</v>
@@ -3086,8 +3082,8 @@
         <v>20</v>
       </c>
       <c r="K16" s="71"/>
-      <c r="L16" s="162"/>
-      <c r="M16" s="151"/>
+      <c r="L16" s="118"/>
+      <c r="M16" s="99"/>
       <c r="N16" s="75"/>
       <c r="O16" s="75">
         <f>ROW()</f>
@@ -3102,9 +3098,9 @@
       <c r="R16" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="S16" s="148"/>
+      <c r="S16" s="97"/>
       <c r="T16" s="71"/>
-      <c r="U16" s="148"/>
+      <c r="U16" s="97"/>
       <c r="V16" s="4" t="s">
         <v>32</v>
       </c>
@@ -3114,9 +3110,9 @@
       <c r="X16" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="Y16" s="148"/>
+      <c r="Y16" s="97"/>
       <c r="Z16" s="71"/>
-      <c r="AA16" s="148"/>
+      <c r="AA16" s="97"/>
       <c r="AB16" s="4" t="s">
         <v>32</v>
       </c>
@@ -3126,10 +3122,10 @@
       <c r="AD16" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="AE16" s="159"/>
-      <c r="AF16" s="97"/>
+      <c r="AE16" s="109"/>
+      <c r="AF16" s="167"/>
       <c r="AG16" s="71"/>
-      <c r="AH16" s="148"/>
+      <c r="AH16" s="97"/>
       <c r="AI16" s="4" t="s">
         <v>32</v>
       </c>
@@ -3142,15 +3138,15 @@
       <c r="AL16" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="AM16" s="148"/>
+      <c r="AM16" s="97"/>
       <c r="AN16" s="40"/>
-      <c r="AO16" s="154"/>
+      <c r="AO16" s="113"/>
     </row>
     <row r="17" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="84" t="s">
         <v>91</v>
       </c>
-      <c r="B17" s="175"/>
+      <c r="B17" s="95"/>
       <c r="C17" s="41"/>
       <c r="D17" s="66" t="s">
         <v>5</v>
@@ -3171,8 +3167,8 @@
         <v>21</v>
       </c>
       <c r="K17" s="71"/>
-      <c r="L17" s="162"/>
-      <c r="M17" s="151"/>
+      <c r="L17" s="118"/>
+      <c r="M17" s="99"/>
       <c r="N17" s="75" t="str">
         <f t="shared" ref="N17:N32" si="1">IF(E15=2,D15 &amp; "  [DQ]",D15)</f>
         <v>Participant #01</v>
@@ -3181,7 +3177,7 @@
         <f t="shared" ref="O17:O32" si="2">IF(E15&gt;=1,ROW()-$O$16,"")</f>
         <v/>
       </c>
-      <c r="P17" s="99" t="s">
+      <c r="P17" s="101" t="s">
         <v>34</v>
       </c>
       <c r="Q17" s="11" t="str" cm="1">
@@ -3189,10 +3185,10 @@
         <v>-</v>
       </c>
       <c r="R17" s="9"/>
-      <c r="S17" s="148"/>
+      <c r="S17" s="97"/>
       <c r="T17" s="71"/>
-      <c r="U17" s="148"/>
-      <c r="V17" s="99" t="s">
+      <c r="U17" s="97"/>
+      <c r="V17" s="101" t="s">
         <v>39</v>
       </c>
       <c r="W17" s="11" t="str">
@@ -3200,10 +3196,10 @@
         <v>A1</v>
       </c>
       <c r="X17" s="6"/>
-      <c r="Y17" s="148"/>
+      <c r="Y17" s="97"/>
       <c r="Z17" s="71"/>
-      <c r="AA17" s="148"/>
-      <c r="AB17" s="99" t="s">
+      <c r="AA17" s="97"/>
+      <c r="AB17" s="101" t="s">
         <v>52</v>
       </c>
       <c r="AC17" s="11" t="str">
@@ -3211,11 +3207,11 @@
         <v>E1</v>
       </c>
       <c r="AD17" s="6"/>
-      <c r="AE17" s="159"/>
-      <c r="AF17" s="97"/>
+      <c r="AE17" s="109"/>
+      <c r="AF17" s="167"/>
       <c r="AG17" s="71"/>
-      <c r="AH17" s="148"/>
-      <c r="AI17" s="99" t="s">
+      <c r="AH17" s="97"/>
+      <c r="AI17" s="101" t="s">
         <v>55</v>
       </c>
       <c r="AJ17" s="21" t="str">
@@ -3226,15 +3222,15 @@
       <c r="AL17" s="47">
         <v>0</v>
       </c>
-      <c r="AM17" s="151"/>
+      <c r="AM17" s="99"/>
       <c r="AN17" s="40"/>
-      <c r="AO17" s="154"/>
+      <c r="AO17" s="113"/>
     </row>
     <row r="18" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="84" t="s">
         <v>164</v>
       </c>
-      <c r="B18" s="175"/>
+      <c r="B18" s="95"/>
       <c r="C18" s="42"/>
       <c r="D18" s="66" t="s">
         <v>6</v>
@@ -3255,8 +3251,8 @@
         <v>22</v>
       </c>
       <c r="K18" s="71"/>
-      <c r="L18" s="162"/>
-      <c r="M18" s="151"/>
+      <c r="L18" s="118"/>
+      <c r="M18" s="99"/>
       <c r="N18" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #02</v>
@@ -3265,35 +3261,35 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P18" s="100"/>
+      <c r="P18" s="102"/>
       <c r="Q18" s="12" t="str" cm="1">
         <f t="array" ref="Q18">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B5))),"-")</f>
         <v>-</v>
       </c>
       <c r="R18" s="10"/>
-      <c r="S18" s="148"/>
+      <c r="S18" s="97"/>
       <c r="T18" s="71"/>
-      <c r="U18" s="148"/>
-      <c r="V18" s="100"/>
+      <c r="U18" s="97"/>
+      <c r="V18" s="102"/>
       <c r="W18" s="12" t="str">
         <f>IF(ISBLANK($R$25),"C1",$R$25)</f>
         <v>C1</v>
       </c>
       <c r="X18" s="14"/>
-      <c r="Y18" s="148"/>
+      <c r="Y18" s="97"/>
       <c r="Z18" s="71"/>
-      <c r="AA18" s="148"/>
-      <c r="AB18" s="100"/>
+      <c r="AA18" s="97"/>
+      <c r="AB18" s="102"/>
       <c r="AC18" s="12" t="str">
         <f>IF(ISBLANK($X$21),"F1",$X$21)</f>
         <v>F1</v>
       </c>
       <c r="AD18" s="14"/>
-      <c r="AE18" s="159"/>
-      <c r="AF18" s="97"/>
+      <c r="AE18" s="109"/>
+      <c r="AF18" s="167"/>
       <c r="AG18" s="71"/>
-      <c r="AH18" s="148"/>
-      <c r="AI18" s="100"/>
+      <c r="AH18" s="97"/>
+      <c r="AI18" s="102"/>
       <c r="AJ18" s="22" t="str">
         <f>IF(ISBLANK($AD$18),"WF2",$AD$18)</f>
         <v>WF2</v>
@@ -3302,15 +3298,15 @@
       <c r="AL18" s="48">
         <v>0</v>
       </c>
-      <c r="AM18" s="151"/>
+      <c r="AM18" s="99"/>
       <c r="AN18" s="40"/>
-      <c r="AO18" s="154"/>
+      <c r="AO18" s="113"/>
     </row>
     <row r="19" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="84" t="s">
         <v>93</v>
       </c>
-      <c r="B19" s="175"/>
+      <c r="B19" s="95"/>
       <c r="C19" s="42"/>
       <c r="D19" s="66" t="s">
         <v>7</v>
@@ -3331,8 +3327,8 @@
         <v>23</v>
       </c>
       <c r="K19" s="71"/>
-      <c r="L19" s="162"/>
-      <c r="M19" s="151"/>
+      <c r="L19" s="118"/>
+      <c r="M19" s="99"/>
       <c r="N19" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #03</v>
@@ -3341,35 +3337,35 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P19" s="100"/>
+      <c r="P19" s="102"/>
       <c r="Q19" s="12" t="str" cm="1">
         <f t="array" ref="Q19">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B9))),"-")</f>
         <v>-</v>
       </c>
       <c r="R19" s="7"/>
-      <c r="S19" s="148"/>
+      <c r="S19" s="97"/>
       <c r="T19" s="71"/>
-      <c r="U19" s="148"/>
-      <c r="V19" s="100"/>
+      <c r="U19" s="97"/>
+      <c r="V19" s="102"/>
       <c r="W19" s="12" t="str">
         <f>IF(ISBLANK($R$22),"B2",$R$22)</f>
         <v>B2</v>
       </c>
       <c r="X19" s="7"/>
-      <c r="Y19" s="148"/>
+      <c r="Y19" s="97"/>
       <c r="Z19" s="71"/>
-      <c r="AA19" s="148"/>
-      <c r="AB19" s="100"/>
+      <c r="AA19" s="97"/>
+      <c r="AB19" s="102"/>
       <c r="AC19" s="12" t="str">
         <f>IF(ISBLANK($X$18),"E2",$X$18)</f>
         <v>E2</v>
       </c>
       <c r="AD19" s="7"/>
-      <c r="AE19" s="159"/>
-      <c r="AF19" s="97"/>
+      <c r="AE19" s="109"/>
+      <c r="AF19" s="167"/>
       <c r="AG19" s="71"/>
-      <c r="AH19" s="148"/>
-      <c r="AI19" s="100"/>
+      <c r="AH19" s="97"/>
+      <c r="AI19" s="102"/>
       <c r="AJ19" s="22" t="str">
         <f>IF(ISBLANK($AD$47),"K1",$AD$47)</f>
         <v>K1</v>
@@ -3378,15 +3374,15 @@
       <c r="AL19" s="49">
         <v>0</v>
       </c>
-      <c r="AM19" s="151"/>
+      <c r="AM19" s="99"/>
       <c r="AN19" s="40"/>
-      <c r="AO19" s="154"/>
+      <c r="AO19" s="113"/>
     </row>
     <row r="20" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="84" t="s">
         <v>142</v>
       </c>
-      <c r="B20" s="175"/>
+      <c r="B20" s="95"/>
       <c r="C20" s="42"/>
       <c r="D20" s="66" t="s">
         <v>8</v>
@@ -3407,8 +3403,8 @@
         <v>24</v>
       </c>
       <c r="K20" s="71"/>
-      <c r="L20" s="162"/>
-      <c r="M20" s="151"/>
+      <c r="L20" s="118"/>
+      <c r="M20" s="99"/>
       <c r="N20" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #04</v>
@@ -3417,35 +3413,35 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P20" s="101"/>
+      <c r="P20" s="103"/>
       <c r="Q20" s="13" t="str" cm="1">
         <f t="array" ref="Q20">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B13))),"-")</f>
         <v>-</v>
       </c>
       <c r="R20" s="8"/>
-      <c r="S20" s="148"/>
+      <c r="S20" s="97"/>
       <c r="T20" s="71"/>
-      <c r="U20" s="148"/>
-      <c r="V20" s="101"/>
+      <c r="U20" s="97"/>
+      <c r="V20" s="103"/>
       <c r="W20" s="13" t="str">
         <f>IF(ISBLANK($R$30),"D2",$R$30)</f>
         <v>D2</v>
       </c>
       <c r="X20" s="8"/>
-      <c r="Y20" s="148"/>
+      <c r="Y20" s="97"/>
       <c r="Z20" s="71"/>
-      <c r="AA20" s="149"/>
-      <c r="AB20" s="101"/>
+      <c r="AA20" s="98"/>
+      <c r="AB20" s="103"/>
       <c r="AC20" s="13" t="str">
         <f>IF(ISBLANK($X$22),"F2",$X$22)</f>
         <v>F2</v>
       </c>
       <c r="AD20" s="8"/>
-      <c r="AE20" s="160"/>
-      <c r="AF20" s="97"/>
+      <c r="AE20" s="110"/>
+      <c r="AF20" s="167"/>
       <c r="AG20" s="71"/>
-      <c r="AH20" s="149"/>
-      <c r="AI20" s="101"/>
+      <c r="AH20" s="98"/>
+      <c r="AI20" s="103"/>
       <c r="AJ20" s="23" t="str">
         <f>IF(ISBLANK($AD$50),"L1",$AD$50)</f>
         <v>L1</v>
@@ -3454,15 +3450,15 @@
       <c r="AL20" s="14">
         <v>0</v>
       </c>
-      <c r="AM20" s="152"/>
+      <c r="AM20" s="100"/>
       <c r="AN20" s="40"/>
-      <c r="AO20" s="154"/>
+      <c r="AO20" s="113"/>
     </row>
     <row r="21" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="84" t="s">
         <v>143</v>
       </c>
-      <c r="B21" s="175"/>
+      <c r="B21" s="95"/>
       <c r="C21" s="42"/>
       <c r="D21" s="66" t="s">
         <v>9</v>
@@ -3483,8 +3479,8 @@
         <v>25</v>
       </c>
       <c r="K21" s="71"/>
-      <c r="L21" s="162"/>
-      <c r="M21" s="151"/>
+      <c r="L21" s="118"/>
+      <c r="M21" s="99"/>
       <c r="N21" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #05</v>
@@ -3493,7 +3489,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P21" s="99" t="s">
+      <c r="P21" s="101" t="s">
         <v>35</v>
       </c>
       <c r="Q21" s="11" t="str" cm="1">
@@ -3501,10 +3497,10 @@
         <v>-</v>
       </c>
       <c r="R21" s="9"/>
-      <c r="S21" s="148"/>
+      <c r="S21" s="97"/>
       <c r="T21" s="71"/>
-      <c r="U21" s="148"/>
-      <c r="V21" s="99" t="s">
+      <c r="U21" s="97"/>
+      <c r="V21" s="101" t="s">
         <v>40</v>
       </c>
       <c r="W21" s="12" t="str">
@@ -3512,29 +3508,29 @@
         <v>B1</v>
       </c>
       <c r="X21" s="6"/>
-      <c r="Y21" s="148"/>
+      <c r="Y21" s="97"/>
       <c r="Z21" s="71"/>
-      <c r="AA21" s="134"/>
-      <c r="AB21" s="132"/>
-      <c r="AC21" s="132"/>
-      <c r="AD21" s="132"/>
-      <c r="AE21" s="132"/>
-      <c r="AF21" s="97"/>
+      <c r="AA21" s="104"/>
+      <c r="AB21" s="105"/>
+      <c r="AC21" s="105"/>
+      <c r="AD21" s="105"/>
+      <c r="AE21" s="105"/>
+      <c r="AF21" s="167"/>
       <c r="AG21" s="71"/>
-      <c r="AH21" s="134"/>
-      <c r="AI21" s="132"/>
-      <c r="AJ21" s="164"/>
-      <c r="AK21" s="164"/>
-      <c r="AL21" s="164"/>
-      <c r="AM21" s="133"/>
+      <c r="AH21" s="104"/>
+      <c r="AI21" s="105"/>
+      <c r="AJ21" s="106"/>
+      <c r="AK21" s="106"/>
+      <c r="AL21" s="106"/>
+      <c r="AM21" s="107"/>
       <c r="AN21" s="40"/>
-      <c r="AO21" s="154"/>
+      <c r="AO21" s="113"/>
     </row>
     <row r="22" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="84" t="s">
         <v>144</v>
       </c>
-      <c r="B22" s="175"/>
+      <c r="B22" s="95"/>
       <c r="C22" s="42"/>
       <c r="D22" s="66" t="s">
         <v>10</v>
@@ -3555,8 +3551,8 @@
         <v>26</v>
       </c>
       <c r="K22" s="71"/>
-      <c r="L22" s="162"/>
-      <c r="M22" s="151"/>
+      <c r="L22" s="118"/>
+      <c r="M22" s="99"/>
       <c r="N22" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #06</v>
@@ -3565,29 +3561,29 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P22" s="100"/>
+      <c r="P22" s="102"/>
       <c r="Q22" s="12" t="str" cm="1">
         <f t="array" ref="Q22">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B6))),"-")</f>
         <v>-</v>
       </c>
       <c r="R22" s="10"/>
-      <c r="S22" s="148"/>
+      <c r="S22" s="97"/>
       <c r="T22" s="71"/>
-      <c r="U22" s="148"/>
-      <c r="V22" s="100"/>
+      <c r="U22" s="97"/>
+      <c r="V22" s="102"/>
       <c r="W22" s="12" t="str">
         <f>IF(ISBLANK($R$29),"D1",$R$29)</f>
         <v>D1</v>
       </c>
       <c r="X22" s="14"/>
-      <c r="Y22" s="148"/>
+      <c r="Y22" s="97"/>
       <c r="Z22" s="71"/>
       <c r="AA22" s="71"/>
       <c r="AB22" s="76"/>
       <c r="AC22" s="77"/>
       <c r="AD22" s="78"/>
       <c r="AE22" s="71"/>
-      <c r="AF22" s="97"/>
+      <c r="AF22" s="167"/>
       <c r="AG22" s="71"/>
       <c r="AH22" s="71"/>
       <c r="AI22" s="71"/>
@@ -3596,13 +3592,13 @@
       <c r="AL22" s="71"/>
       <c r="AM22" s="71"/>
       <c r="AN22" s="40"/>
-      <c r="AO22" s="154"/>
+      <c r="AO22" s="113"/>
     </row>
     <row r="23" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="84" t="s">
         <v>165</v>
       </c>
-      <c r="B23" s="175"/>
+      <c r="B23" s="95"/>
       <c r="C23" s="42"/>
       <c r="D23" s="66" t="s">
         <v>11</v>
@@ -3623,8 +3619,8 @@
         <v>27</v>
       </c>
       <c r="K23" s="71"/>
-      <c r="L23" s="162"/>
-      <c r="M23" s="151"/>
+      <c r="L23" s="118"/>
+      <c r="M23" s="99"/>
       <c r="N23" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #07</v>
@@ -3633,29 +3629,29 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P23" s="100"/>
+      <c r="P23" s="102"/>
       <c r="Q23" s="12" t="str" cm="1">
         <f t="array" ref="Q23">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B10))),"-")</f>
         <v>-</v>
       </c>
       <c r="R23" s="7"/>
-      <c r="S23" s="148"/>
+      <c r="S23" s="97"/>
       <c r="T23" s="71"/>
-      <c r="U23" s="148"/>
-      <c r="V23" s="100"/>
+      <c r="U23" s="97"/>
+      <c r="V23" s="102"/>
       <c r="W23" s="12" t="str">
         <f>IF(ISBLANK($R$18),"A2",$R$18)</f>
         <v>A2</v>
       </c>
       <c r="X23" s="7"/>
-      <c r="Y23" s="148"/>
+      <c r="Y23" s="97"/>
       <c r="Z23" s="71"/>
       <c r="AA23" s="71"/>
       <c r="AB23" s="76"/>
       <c r="AC23" s="77"/>
       <c r="AD23" s="78"/>
       <c r="AE23" s="71"/>
-      <c r="AF23" s="97"/>
+      <c r="AF23" s="167"/>
       <c r="AG23" s="71"/>
       <c r="AH23" s="71"/>
       <c r="AI23" s="71"/>
@@ -3664,13 +3660,13 @@
       <c r="AL23" s="71"/>
       <c r="AM23" s="71"/>
       <c r="AN23" s="40"/>
-      <c r="AO23" s="154"/>
+      <c r="AO23" s="113"/>
     </row>
     <row r="24" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="84" t="s">
         <v>145</v>
       </c>
-      <c r="B24" s="175"/>
+      <c r="B24" s="95"/>
       <c r="C24" s="42"/>
       <c r="D24" s="66" t="s">
         <v>12</v>
@@ -3691,8 +3687,8 @@
         <v>27</v>
       </c>
       <c r="K24" s="71"/>
-      <c r="L24" s="162"/>
-      <c r="M24" s="151"/>
+      <c r="L24" s="118"/>
+      <c r="M24" s="99"/>
       <c r="N24" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #08</v>
@@ -3701,29 +3697,29 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P24" s="101"/>
+      <c r="P24" s="103"/>
       <c r="Q24" s="13" t="str" cm="1">
         <f t="array" ref="Q24">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B14))),"-")</f>
         <v>-</v>
       </c>
       <c r="R24" s="8"/>
-      <c r="S24" s="148"/>
+      <c r="S24" s="97"/>
       <c r="T24" s="71"/>
-      <c r="U24" s="149"/>
-      <c r="V24" s="101"/>
+      <c r="U24" s="98"/>
+      <c r="V24" s="103"/>
       <c r="W24" s="13" t="str">
         <f>IF(ISBLANK($R$26),"C2",$R$26)</f>
         <v>C2</v>
       </c>
       <c r="X24" s="8"/>
-      <c r="Y24" s="149"/>
+      <c r="Y24" s="98"/>
       <c r="Z24" s="71"/>
       <c r="AA24" s="71"/>
       <c r="AB24" s="76"/>
       <c r="AC24" s="77"/>
       <c r="AD24" s="78"/>
       <c r="AE24" s="71"/>
-      <c r="AF24" s="97"/>
+      <c r="AF24" s="167"/>
       <c r="AG24" s="71"/>
       <c r="AH24" s="71"/>
       <c r="AI24" s="71"/>
@@ -3732,13 +3728,13 @@
       <c r="AL24" s="71"/>
       <c r="AM24" s="71"/>
       <c r="AN24" s="40"/>
-      <c r="AO24" s="154"/>
+      <c r="AO24" s="113"/>
     </row>
     <row r="25" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="84" t="s">
         <v>63</v>
       </c>
-      <c r="B25" s="175"/>
+      <c r="B25" s="95"/>
       <c r="C25" s="42"/>
       <c r="D25" s="66" t="s">
         <v>13</v>
@@ -3759,8 +3755,8 @@
         <v>28</v>
       </c>
       <c r="K25" s="71"/>
-      <c r="L25" s="162"/>
-      <c r="M25" s="151"/>
+      <c r="L25" s="118"/>
+      <c r="M25" s="99"/>
       <c r="N25" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #09</v>
@@ -3769,7 +3765,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P25" s="99" t="s">
+      <c r="P25" s="101" t="s">
         <v>36</v>
       </c>
       <c r="Q25" s="11" t="str" cm="1">
@@ -3777,37 +3773,37 @@
         <v>-</v>
       </c>
       <c r="R25" s="9"/>
-      <c r="S25" s="148"/>
+      <c r="S25" s="97"/>
       <c r="T25" s="71"/>
-      <c r="U25" s="134"/>
-      <c r="V25" s="132"/>
-      <c r="W25" s="132"/>
-      <c r="X25" s="132"/>
-      <c r="Y25" s="133"/>
+      <c r="U25" s="104"/>
+      <c r="V25" s="105"/>
+      <c r="W25" s="105"/>
+      <c r="X25" s="105"/>
+      <c r="Y25" s="107"/>
       <c r="Z25" s="71"/>
       <c r="AA25" s="71"/>
       <c r="AB25" s="71"/>
       <c r="AC25" s="71"/>
       <c r="AD25" s="71"/>
       <c r="AE25" s="71"/>
-      <c r="AF25" s="97"/>
+      <c r="AF25" s="167"/>
       <c r="AG25" s="71"/>
-      <c r="AH25" s="102" t="s">
+      <c r="AH25" s="120" t="s">
         <v>53</v>
       </c>
-      <c r="AI25" s="103"/>
-      <c r="AJ25" s="103"/>
-      <c r="AK25" s="103"/>
-      <c r="AL25" s="103"/>
-      <c r="AM25" s="104"/>
+      <c r="AI25" s="121"/>
+      <c r="AJ25" s="121"/>
+      <c r="AK25" s="121"/>
+      <c r="AL25" s="121"/>
+      <c r="AM25" s="122"/>
       <c r="AN25" s="40"/>
-      <c r="AO25" s="154"/>
+      <c r="AO25" s="113"/>
     </row>
     <row r="26" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="84" t="s">
         <v>146</v>
       </c>
-      <c r="B26" s="175"/>
+      <c r="B26" s="95"/>
       <c r="C26" s="42"/>
       <c r="D26" s="66" t="s">
         <v>14</v>
@@ -3828,8 +3824,8 @@
         <v>28</v>
       </c>
       <c r="K26" s="71"/>
-      <c r="L26" s="162"/>
-      <c r="M26" s="151"/>
+      <c r="L26" s="118"/>
+      <c r="M26" s="99"/>
       <c r="N26" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #10</v>
@@ -3838,13 +3834,13 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P26" s="100"/>
+      <c r="P26" s="102"/>
       <c r="Q26" s="12" t="str" cm="1">
         <f t="array" ref="Q26">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B7))),"-")</f>
         <v>-</v>
       </c>
       <c r="R26" s="10"/>
-      <c r="S26" s="148"/>
+      <c r="S26" s="97"/>
       <c r="T26" s="71"/>
       <c r="U26" s="71"/>
       <c r="V26" s="76"/>
@@ -3857,22 +3853,22 @@
       <c r="AC26" s="71"/>
       <c r="AD26" s="71"/>
       <c r="AE26" s="71"/>
-      <c r="AF26" s="97"/>
+      <c r="AF26" s="167"/>
       <c r="AG26" s="71"/>
-      <c r="AH26" s="105"/>
-      <c r="AI26" s="106"/>
-      <c r="AJ26" s="106"/>
-      <c r="AK26" s="106"/>
-      <c r="AL26" s="106"/>
-      <c r="AM26" s="107"/>
+      <c r="AH26" s="123"/>
+      <c r="AI26" s="124"/>
+      <c r="AJ26" s="124"/>
+      <c r="AK26" s="124"/>
+      <c r="AL26" s="124"/>
+      <c r="AM26" s="125"/>
       <c r="AN26" s="40"/>
-      <c r="AO26" s="154"/>
+      <c r="AO26" s="113"/>
     </row>
     <row r="27" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="84" t="s">
         <v>124</v>
       </c>
-      <c r="B27" s="175"/>
+      <c r="B27" s="95"/>
       <c r="C27" s="42"/>
       <c r="D27" s="66" t="s">
         <v>15</v>
@@ -3893,8 +3889,8 @@
         <v>29</v>
       </c>
       <c r="K27" s="71"/>
-      <c r="L27" s="162"/>
-      <c r="M27" s="151"/>
+      <c r="L27" s="118"/>
+      <c r="M27" s="99"/>
       <c r="N27" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #11</v>
@@ -3903,13 +3899,13 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P27" s="100"/>
+      <c r="P27" s="102"/>
       <c r="Q27" s="12" t="str" cm="1">
         <f t="array" ref="Q27">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B11))),"-")</f>
         <v>-</v>
       </c>
       <c r="R27" s="7"/>
-      <c r="S27" s="148"/>
+      <c r="S27" s="97"/>
       <c r="T27" s="71"/>
       <c r="U27" s="71"/>
       <c r="V27" s="76"/>
@@ -3922,22 +3918,22 @@
       <c r="AC27" s="71"/>
       <c r="AD27" s="71"/>
       <c r="AE27" s="71"/>
-      <c r="AF27" s="97"/>
+      <c r="AF27" s="167"/>
       <c r="AG27" s="71"/>
-      <c r="AH27" s="108"/>
-      <c r="AI27" s="109"/>
-      <c r="AJ27" s="109"/>
-      <c r="AK27" s="109"/>
-      <c r="AL27" s="109"/>
-      <c r="AM27" s="110"/>
+      <c r="AH27" s="126"/>
+      <c r="AI27" s="127"/>
+      <c r="AJ27" s="127"/>
+      <c r="AK27" s="127"/>
+      <c r="AL27" s="127"/>
+      <c r="AM27" s="128"/>
       <c r="AN27" s="40"/>
-      <c r="AO27" s="154"/>
+      <c r="AO27" s="113"/>
     </row>
     <row r="28" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="84" t="s">
         <v>90</v>
       </c>
-      <c r="B28" s="175"/>
+      <c r="B28" s="95"/>
       <c r="C28" s="42"/>
       <c r="D28" s="66" t="s">
         <v>16</v>
@@ -3958,8 +3954,8 @@
         <v>29</v>
       </c>
       <c r="K28" s="71"/>
-      <c r="L28" s="162"/>
-      <c r="M28" s="151"/>
+      <c r="L28" s="118"/>
+      <c r="M28" s="99"/>
       <c r="N28" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #12</v>
@@ -3968,13 +3964,13 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P28" s="101"/>
+      <c r="P28" s="103"/>
       <c r="Q28" s="13" t="str" cm="1">
         <f t="array" ref="Q28">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B15))),"-")</f>
         <v>-</v>
       </c>
       <c r="R28" s="8"/>
-      <c r="S28" s="148"/>
+      <c r="S28" s="97"/>
       <c r="T28" s="71"/>
       <c r="U28" s="71"/>
       <c r="V28" s="76"/>
@@ -3987,22 +3983,22 @@
       <c r="AC28" s="71"/>
       <c r="AD28" s="71"/>
       <c r="AE28" s="71"/>
-      <c r="AF28" s="97"/>
+      <c r="AF28" s="167"/>
       <c r="AG28" s="71"/>
-      <c r="AH28" s="134"/>
-      <c r="AI28" s="132"/>
-      <c r="AJ28" s="132"/>
-      <c r="AK28" s="132"/>
-      <c r="AL28" s="132"/>
-      <c r="AM28" s="133"/>
+      <c r="AH28" s="104"/>
+      <c r="AI28" s="105"/>
+      <c r="AJ28" s="105"/>
+      <c r="AK28" s="105"/>
+      <c r="AL28" s="105"/>
+      <c r="AM28" s="107"/>
       <c r="AN28" s="40"/>
-      <c r="AO28" s="154"/>
+      <c r="AO28" s="113"/>
     </row>
     <row r="29" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="84" t="s">
         <v>138</v>
       </c>
-      <c r="B29" s="175"/>
+      <c r="B29" s="95"/>
       <c r="C29" s="42"/>
       <c r="D29" s="66" t="s">
         <v>17</v>
@@ -4023,8 +4019,8 @@
         <v>30</v>
       </c>
       <c r="K29" s="71"/>
-      <c r="L29" s="162"/>
-      <c r="M29" s="151"/>
+      <c r="L29" s="118"/>
+      <c r="M29" s="99"/>
       <c r="N29" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #13</v>
@@ -4033,7 +4029,7 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P29" s="99" t="s">
+      <c r="P29" s="101" t="s">
         <v>37</v>
       </c>
       <c r="Q29" s="11" t="str" cm="1">
@@ -4041,7 +4037,7 @@
         <v>-</v>
       </c>
       <c r="R29" s="9"/>
-      <c r="S29" s="148"/>
+      <c r="S29" s="97"/>
       <c r="T29" s="71"/>
       <c r="U29" s="71"/>
       <c r="V29" s="76"/>
@@ -4054,26 +4050,26 @@
       <c r="AC29" s="71"/>
       <c r="AD29" s="71"/>
       <c r="AE29" s="71"/>
-      <c r="AF29" s="97"/>
+      <c r="AF29" s="167"/>
       <c r="AG29" s="71"/>
-      <c r="AH29" s="147"/>
+      <c r="AH29" s="96"/>
       <c r="AI29" s="5">
         <v>8</v>
       </c>
-      <c r="AJ29" s="94" t="s">
+      <c r="AJ29" s="138" t="s">
         <v>31</v>
       </c>
-      <c r="AK29" s="94"/>
-      <c r="AL29" s="95"/>
-      <c r="AM29" s="147"/>
+      <c r="AK29" s="138"/>
+      <c r="AL29" s="139"/>
+      <c r="AM29" s="96"/>
       <c r="AN29" s="40"/>
-      <c r="AO29" s="154"/>
+      <c r="AO29" s="113"/>
     </row>
     <row r="30" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="84" t="s">
         <v>166</v>
       </c>
-      <c r="B30" s="175"/>
+      <c r="B30" s="95"/>
       <c r="C30" s="42"/>
       <c r="D30" s="67" t="s">
         <v>18</v>
@@ -4094,8 +4090,8 @@
         <v>30</v>
       </c>
       <c r="K30" s="71"/>
-      <c r="L30" s="162"/>
-      <c r="M30" s="151"/>
+      <c r="L30" s="118"/>
+      <c r="M30" s="99"/>
       <c r="N30" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #14</v>
@@ -4104,13 +4100,13 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P30" s="100"/>
+      <c r="P30" s="102"/>
       <c r="Q30" s="12" t="str" cm="1">
         <f t="array" ref="Q30">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B8))),"-")</f>
         <v>-</v>
       </c>
       <c r="R30" s="10"/>
-      <c r="S30" s="148"/>
+      <c r="S30" s="97"/>
       <c r="T30" s="71"/>
       <c r="U30" s="71"/>
       <c r="V30" s="76"/>
@@ -4123,9 +4119,9 @@
       <c r="AC30" s="71"/>
       <c r="AD30" s="71"/>
       <c r="AE30" s="71"/>
-      <c r="AF30" s="97"/>
+      <c r="AF30" s="167"/>
       <c r="AG30" s="71"/>
-      <c r="AH30" s="148"/>
+      <c r="AH30" s="97"/>
       <c r="AI30" s="4" t="s">
         <v>32</v>
       </c>
@@ -4138,15 +4134,15 @@
       <c r="AL30" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="AM30" s="148"/>
+      <c r="AM30" s="97"/>
       <c r="AN30" s="40"/>
-      <c r="AO30" s="154"/>
+      <c r="AO30" s="113"/>
     </row>
     <row r="31" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="84" t="s">
         <v>125</v>
       </c>
-      <c r="B31" s="175"/>
+      <c r="B31" s="95"/>
       <c r="C31" s="42"/>
       <c r="D31" s="79"/>
       <c r="E31" s="72"/>
@@ -4156,8 +4152,8 @@
       <c r="I31" s="72"/>
       <c r="J31" s="72"/>
       <c r="K31" s="80"/>
-      <c r="L31" s="162"/>
-      <c r="M31" s="151"/>
+      <c r="L31" s="118"/>
+      <c r="M31" s="99"/>
       <c r="N31" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #15</v>
@@ -4166,13 +4162,13 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P31" s="100"/>
+      <c r="P31" s="102"/>
       <c r="Q31" s="12" t="str" cm="1">
         <f t="array" ref="Q31">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B12))),"-")</f>
         <v>-</v>
       </c>
       <c r="R31" s="7"/>
-      <c r="S31" s="148"/>
+      <c r="S31" s="97"/>
       <c r="T31" s="71"/>
       <c r="U31" s="71"/>
       <c r="V31" s="76"/>
@@ -4185,10 +4181,10 @@
       <c r="AC31" s="71"/>
       <c r="AD31" s="71"/>
       <c r="AE31" s="71"/>
-      <c r="AF31" s="97"/>
+      <c r="AF31" s="167"/>
       <c r="AG31" s="71"/>
-      <c r="AH31" s="148"/>
-      <c r="AI31" s="99" t="s">
+      <c r="AH31" s="97"/>
+      <c r="AI31" s="101" t="s">
         <v>56</v>
       </c>
       <c r="AJ31" s="21" t="str">
@@ -4199,15 +4195,15 @@
       <c r="AL31" s="47">
         <v>0</v>
       </c>
-      <c r="AM31" s="151"/>
+      <c r="AM31" s="99"/>
       <c r="AN31" s="40"/>
-      <c r="AO31" s="154"/>
+      <c r="AO31" s="113"/>
     </row>
     <row r="32" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="84" t="s">
         <v>147</v>
       </c>
-      <c r="B32" s="175"/>
+      <c r="B32" s="95"/>
       <c r="C32" s="42"/>
       <c r="D32" s="79"/>
       <c r="E32" s="72"/>
@@ -4217,8 +4213,8 @@
       <c r="I32" s="72"/>
       <c r="J32" s="72"/>
       <c r="K32" s="80"/>
-      <c r="L32" s="162"/>
-      <c r="M32" s="152"/>
+      <c r="L32" s="118"/>
+      <c r="M32" s="100"/>
       <c r="N32" s="60" t="str">
         <f t="shared" si="1"/>
         <v>Participant #16</v>
@@ -4227,13 +4223,13 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P32" s="101"/>
+      <c r="P32" s="103"/>
       <c r="Q32" s="13" t="str" cm="1">
         <f t="array" ref="Q32">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B16))),"-")</f>
         <v>-</v>
       </c>
       <c r="R32" s="8"/>
-      <c r="S32" s="149"/>
+      <c r="S32" s="98"/>
       <c r="T32" s="71"/>
       <c r="U32" s="71"/>
       <c r="V32" s="76"/>
@@ -4246,10 +4242,10 @@
       <c r="AC32" s="71"/>
       <c r="AD32" s="71"/>
       <c r="AE32" s="71"/>
-      <c r="AF32" s="97"/>
+      <c r="AF32" s="167"/>
       <c r="AG32" s="71"/>
-      <c r="AH32" s="148"/>
-      <c r="AI32" s="100"/>
+      <c r="AH32" s="97"/>
+      <c r="AI32" s="102"/>
       <c r="AJ32" s="22" t="str">
         <f>IF(ISBLANK($AD$51),"L2",$AD$51)</f>
         <v>L2</v>
@@ -4258,15 +4254,15 @@
       <c r="AL32" s="48">
         <v>0</v>
       </c>
-      <c r="AM32" s="151"/>
+      <c r="AM32" s="99"/>
       <c r="AN32" s="40"/>
-      <c r="AO32" s="154"/>
+      <c r="AO32" s="113"/>
     </row>
     <row r="33" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="B33" s="175"/>
+      <c r="B33" s="95"/>
       <c r="C33" s="42"/>
       <c r="D33" s="79"/>
       <c r="E33" s="72"/>
@@ -4276,17 +4272,17 @@
       <c r="I33" s="72"/>
       <c r="J33" s="72"/>
       <c r="K33" s="80"/>
-      <c r="L33" s="162"/>
-      <c r="M33" s="132" t="str">
+      <c r="L33" s="118"/>
+      <c r="M33" s="105" t="str">
         <f>IF(E31&gt;=1,ROW()-$O$16,"")</f>
         <v/>
       </c>
-      <c r="N33" s="132"/>
-      <c r="O33" s="132"/>
-      <c r="P33" s="132"/>
-      <c r="Q33" s="132"/>
-      <c r="R33" s="132"/>
-      <c r="S33" s="133"/>
+      <c r="N33" s="105"/>
+      <c r="O33" s="105"/>
+      <c r="P33" s="105"/>
+      <c r="Q33" s="105"/>
+      <c r="R33" s="105"/>
+      <c r="S33" s="107"/>
       <c r="T33" s="71"/>
       <c r="U33" s="71"/>
       <c r="V33" s="71"/>
@@ -4299,10 +4295,10 @@
       <c r="AC33" s="71"/>
       <c r="AD33" s="71"/>
       <c r="AE33" s="71"/>
-      <c r="AF33" s="97"/>
+      <c r="AF33" s="167"/>
       <c r="AG33" s="71"/>
-      <c r="AH33" s="148"/>
-      <c r="AI33" s="100"/>
+      <c r="AH33" s="97"/>
+      <c r="AI33" s="102"/>
       <c r="AJ33" s="22" t="str">
         <f>IF(ISBLANK($AD$49),"K3",$AD$49)</f>
         <v>K3</v>
@@ -4311,15 +4307,15 @@
       <c r="AL33" s="49">
         <v>0</v>
       </c>
-      <c r="AM33" s="151"/>
+      <c r="AM33" s="99"/>
       <c r="AN33" s="40"/>
-      <c r="AO33" s="154"/>
+      <c r="AO33" s="113"/>
     </row>
     <row r="34" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="84" t="s">
         <v>98</v>
       </c>
-      <c r="B34" s="175"/>
+      <c r="B34" s="95"/>
       <c r="C34" s="42"/>
       <c r="D34" s="79"/>
       <c r="E34" s="72"/>
@@ -4329,7 +4325,7 @@
       <c r="I34" s="72"/>
       <c r="J34" s="72"/>
       <c r="K34" s="80"/>
-      <c r="L34" s="162"/>
+      <c r="L34" s="118"/>
       <c r="M34" s="71"/>
       <c r="N34" s="71"/>
       <c r="O34" s="71" t="str">
@@ -4352,10 +4348,10 @@
       <c r="AC34" s="71"/>
       <c r="AD34" s="71"/>
       <c r="AE34" s="71"/>
-      <c r="AF34" s="97"/>
+      <c r="AF34" s="167"/>
       <c r="AG34" s="71"/>
-      <c r="AH34" s="149"/>
-      <c r="AI34" s="101"/>
+      <c r="AH34" s="98"/>
+      <c r="AI34" s="103"/>
       <c r="AJ34" s="23" t="str">
         <f>IF(ISBLANK($AD$52),"L3",$AD$52)</f>
         <v>L3</v>
@@ -4364,15 +4360,15 @@
       <c r="AL34" s="14">
         <v>0</v>
       </c>
-      <c r="AM34" s="152"/>
+      <c r="AM34" s="100"/>
       <c r="AN34" s="40"/>
-      <c r="AO34" s="154"/>
+      <c r="AO34" s="113"/>
     </row>
     <row r="35" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="84" t="s">
         <v>104</v>
       </c>
-      <c r="B35" s="175"/>
+      <c r="B35" s="95"/>
       <c r="C35" s="42"/>
       <c r="D35" s="79"/>
       <c r="E35" s="72"/>
@@ -4382,7 +4378,7 @@
       <c r="I35" s="72"/>
       <c r="J35" s="72"/>
       <c r="K35" s="80"/>
-      <c r="L35" s="162"/>
+      <c r="L35" s="118"/>
       <c r="M35" s="71"/>
       <c r="N35" s="82"/>
       <c r="O35" s="82"/>
@@ -4402,22 +4398,22 @@
       <c r="AC35" s="82"/>
       <c r="AD35" s="82"/>
       <c r="AE35" s="82"/>
-      <c r="AF35" s="97"/>
+      <c r="AF35" s="167"/>
       <c r="AG35" s="71"/>
-      <c r="AH35" s="134"/>
-      <c r="AI35" s="132"/>
-      <c r="AJ35" s="164"/>
-      <c r="AK35" s="164"/>
-      <c r="AL35" s="164"/>
-      <c r="AM35" s="133"/>
+      <c r="AH35" s="104"/>
+      <c r="AI35" s="105"/>
+      <c r="AJ35" s="106"/>
+      <c r="AK35" s="106"/>
+      <c r="AL35" s="106"/>
+      <c r="AM35" s="107"/>
       <c r="AN35" s="40"/>
-      <c r="AO35" s="154"/>
+      <c r="AO35" s="113"/>
     </row>
     <row r="36" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="84" t="s">
         <v>106</v>
       </c>
-      <c r="B36" s="175"/>
+      <c r="B36" s="95"/>
       <c r="C36" s="42"/>
       <c r="D36" s="79"/>
       <c r="E36" s="72"/>
@@ -4427,29 +4423,29 @@
       <c r="I36" s="72"/>
       <c r="J36" s="72"/>
       <c r="K36" s="80"/>
-      <c r="L36" s="162"/>
-      <c r="M36" s="135" t="s">
+      <c r="L36" s="118"/>
+      <c r="M36" s="129" t="s">
         <v>43</v>
       </c>
-      <c r="N36" s="136"/>
-      <c r="O36" s="136"/>
-      <c r="P36" s="136"/>
-      <c r="Q36" s="136"/>
-      <c r="R36" s="136"/>
-      <c r="S36" s="136"/>
-      <c r="T36" s="136"/>
-      <c r="U36" s="136"/>
-      <c r="V36" s="136"/>
-      <c r="W36" s="136"/>
-      <c r="X36" s="136"/>
-      <c r="Y36" s="136"/>
-      <c r="Z36" s="136"/>
-      <c r="AA36" s="136"/>
-      <c r="AB36" s="136"/>
-      <c r="AC36" s="136"/>
-      <c r="AD36" s="136"/>
-      <c r="AE36" s="137"/>
-      <c r="AF36" s="97"/>
+      <c r="N36" s="130"/>
+      <c r="O36" s="130"/>
+      <c r="P36" s="130"/>
+      <c r="Q36" s="130"/>
+      <c r="R36" s="130"/>
+      <c r="S36" s="130"/>
+      <c r="T36" s="130"/>
+      <c r="U36" s="130"/>
+      <c r="V36" s="130"/>
+      <c r="W36" s="130"/>
+      <c r="X36" s="130"/>
+      <c r="Y36" s="130"/>
+      <c r="Z36" s="130"/>
+      <c r="AA36" s="130"/>
+      <c r="AB36" s="130"/>
+      <c r="AC36" s="130"/>
+      <c r="AD36" s="130"/>
+      <c r="AE36" s="131"/>
+      <c r="AF36" s="167"/>
       <c r="AG36" s="71"/>
       <c r="AH36" s="71"/>
       <c r="AI36" s="71"/>
@@ -4458,13 +4454,13 @@
       <c r="AL36" s="71"/>
       <c r="AM36" s="71"/>
       <c r="AN36" s="40"/>
-      <c r="AO36" s="154"/>
+      <c r="AO36" s="113"/>
     </row>
     <row r="37" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="84" t="s">
         <v>105</v>
       </c>
-      <c r="B37" s="175"/>
+      <c r="B37" s="95"/>
       <c r="C37" s="42"/>
       <c r="D37" s="79"/>
       <c r="E37" s="72"/>
@@ -4474,27 +4470,27 @@
       <c r="I37" s="72"/>
       <c r="J37" s="72"/>
       <c r="K37" s="80"/>
-      <c r="L37" s="162"/>
-      <c r="M37" s="138"/>
-      <c r="N37" s="139"/>
-      <c r="O37" s="139"/>
-      <c r="P37" s="139"/>
-      <c r="Q37" s="139"/>
-      <c r="R37" s="139"/>
-      <c r="S37" s="139"/>
-      <c r="T37" s="139"/>
-      <c r="U37" s="139"/>
-      <c r="V37" s="139"/>
-      <c r="W37" s="139"/>
-      <c r="X37" s="139"/>
-      <c r="Y37" s="139"/>
-      <c r="Z37" s="139"/>
-      <c r="AA37" s="139"/>
-      <c r="AB37" s="139"/>
-      <c r="AC37" s="139"/>
-      <c r="AD37" s="139"/>
-      <c r="AE37" s="140"/>
-      <c r="AF37" s="97"/>
+      <c r="L37" s="118"/>
+      <c r="M37" s="132"/>
+      <c r="N37" s="133"/>
+      <c r="O37" s="133"/>
+      <c r="P37" s="133"/>
+      <c r="Q37" s="133"/>
+      <c r="R37" s="133"/>
+      <c r="S37" s="133"/>
+      <c r="T37" s="133"/>
+      <c r="U37" s="133"/>
+      <c r="V37" s="133"/>
+      <c r="W37" s="133"/>
+      <c r="X37" s="133"/>
+      <c r="Y37" s="133"/>
+      <c r="Z37" s="133"/>
+      <c r="AA37" s="133"/>
+      <c r="AB37" s="133"/>
+      <c r="AC37" s="133"/>
+      <c r="AD37" s="133"/>
+      <c r="AE37" s="134"/>
+      <c r="AF37" s="167"/>
       <c r="AG37" s="71"/>
       <c r="AH37" s="71"/>
       <c r="AI37" s="71"/>
@@ -4503,13 +4499,13 @@
       <c r="AL37" s="71"/>
       <c r="AM37" s="71"/>
       <c r="AN37" s="40"/>
-      <c r="AO37" s="154"/>
+      <c r="AO37" s="113"/>
     </row>
     <row r="38" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="84" t="s">
         <v>101</v>
       </c>
-      <c r="B38" s="175"/>
+      <c r="B38" s="95"/>
       <c r="C38" s="42"/>
       <c r="D38" s="79"/>
       <c r="E38" s="72"/>
@@ -4519,27 +4515,27 @@
       <c r="I38" s="72"/>
       <c r="J38" s="72"/>
       <c r="K38" s="80"/>
-      <c r="L38" s="162"/>
-      <c r="M38" s="141"/>
-      <c r="N38" s="142"/>
-      <c r="O38" s="142"/>
-      <c r="P38" s="142"/>
-      <c r="Q38" s="142"/>
-      <c r="R38" s="142"/>
-      <c r="S38" s="142"/>
-      <c r="T38" s="142"/>
-      <c r="U38" s="142"/>
-      <c r="V38" s="142"/>
-      <c r="W38" s="142"/>
-      <c r="X38" s="142"/>
-      <c r="Y38" s="142"/>
-      <c r="Z38" s="142"/>
-      <c r="AA38" s="142"/>
-      <c r="AB38" s="142"/>
-      <c r="AC38" s="142"/>
-      <c r="AD38" s="142"/>
-      <c r="AE38" s="143"/>
-      <c r="AF38" s="97"/>
+      <c r="L38" s="118"/>
+      <c r="M38" s="135"/>
+      <c r="N38" s="136"/>
+      <c r="O38" s="136"/>
+      <c r="P38" s="136"/>
+      <c r="Q38" s="136"/>
+      <c r="R38" s="136"/>
+      <c r="S38" s="136"/>
+      <c r="T38" s="136"/>
+      <c r="U38" s="136"/>
+      <c r="V38" s="136"/>
+      <c r="W38" s="136"/>
+      <c r="X38" s="136"/>
+      <c r="Y38" s="136"/>
+      <c r="Z38" s="136"/>
+      <c r="AA38" s="136"/>
+      <c r="AB38" s="136"/>
+      <c r="AC38" s="136"/>
+      <c r="AD38" s="136"/>
+      <c r="AE38" s="137"/>
+      <c r="AF38" s="167"/>
       <c r="AG38" s="71"/>
       <c r="AH38" s="71"/>
       <c r="AI38" s="71"/>
@@ -4548,13 +4544,13 @@
       <c r="AL38" s="71"/>
       <c r="AM38" s="71"/>
       <c r="AN38" s="40"/>
-      <c r="AO38" s="154"/>
+      <c r="AO38" s="113"/>
     </row>
     <row r="39" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="84" t="s">
         <v>103</v>
       </c>
-      <c r="B39" s="175"/>
+      <c r="B39" s="95"/>
       <c r="C39" s="42"/>
       <c r="D39" s="79"/>
       <c r="E39" s="72"/>
@@ -4564,7 +4560,7 @@
       <c r="I39" s="72"/>
       <c r="J39" s="72"/>
       <c r="K39" s="80"/>
-      <c r="L39" s="162"/>
+      <c r="L39" s="118"/>
       <c r="M39" s="71"/>
       <c r="N39" s="71"/>
       <c r="O39" s="71"/>
@@ -4584,7 +4580,7 @@
       <c r="AC39" s="71"/>
       <c r="AD39" s="71"/>
       <c r="AE39" s="71"/>
-      <c r="AF39" s="97"/>
+      <c r="AF39" s="167"/>
       <c r="AG39" s="71"/>
       <c r="AH39" s="71"/>
       <c r="AI39" s="71"/>
@@ -4593,13 +4589,13 @@
       <c r="AL39" s="71"/>
       <c r="AM39" s="71"/>
       <c r="AN39" s="40"/>
-      <c r="AO39" s="154"/>
+      <c r="AO39" s="113"/>
     </row>
     <row r="40" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="84" t="s">
         <v>102</v>
       </c>
-      <c r="B40" s="175"/>
+      <c r="B40" s="95"/>
       <c r="C40" s="42"/>
       <c r="D40" s="79"/>
       <c r="E40" s="72"/>
@@ -4609,7 +4605,7 @@
       <c r="I40" s="72"/>
       <c r="J40" s="72"/>
       <c r="K40" s="80"/>
-      <c r="L40" s="162"/>
+      <c r="L40" s="118"/>
       <c r="M40" s="71"/>
       <c r="N40" s="71"/>
       <c r="O40" s="71"/>
@@ -4629,7 +4625,7 @@
       <c r="AC40" s="71"/>
       <c r="AD40" s="71"/>
       <c r="AE40" s="71"/>
-      <c r="AF40" s="97"/>
+      <c r="AF40" s="167"/>
       <c r="AG40" s="71"/>
       <c r="AH40" s="71"/>
       <c r="AI40" s="71"/>
@@ -4638,13 +4634,13 @@
       <c r="AL40" s="71"/>
       <c r="AM40" s="71"/>
       <c r="AN40" s="40"/>
-      <c r="AO40" s="154"/>
+      <c r="AO40" s="113"/>
     </row>
     <row r="41" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="84" t="s">
         <v>122</v>
       </c>
-      <c r="B41" s="175"/>
+      <c r="B41" s="95"/>
       <c r="C41" s="42"/>
       <c r="D41" s="79"/>
       <c r="E41" s="72"/>
@@ -4654,33 +4650,33 @@
       <c r="I41" s="72"/>
       <c r="J41" s="72"/>
       <c r="K41" s="80"/>
-      <c r="L41" s="162"/>
-      <c r="M41" s="103" t="s">
+      <c r="L41" s="118"/>
+      <c r="M41" s="121" t="s">
         <v>44</v>
       </c>
-      <c r="N41" s="103"/>
-      <c r="O41" s="103"/>
-      <c r="P41" s="103"/>
-      <c r="Q41" s="103"/>
-      <c r="R41" s="103"/>
-      <c r="S41" s="104"/>
+      <c r="N41" s="121"/>
+      <c r="O41" s="121"/>
+      <c r="P41" s="121"/>
+      <c r="Q41" s="121"/>
+      <c r="R41" s="121"/>
+      <c r="S41" s="122"/>
       <c r="T41" s="70"/>
-      <c r="U41" s="102" t="s">
+      <c r="U41" s="120" t="s">
         <v>48</v>
       </c>
-      <c r="V41" s="103"/>
-      <c r="W41" s="103"/>
-      <c r="X41" s="103"/>
-      <c r="Y41" s="104"/>
+      <c r="V41" s="121"/>
+      <c r="W41" s="121"/>
+      <c r="X41" s="121"/>
+      <c r="Y41" s="122"/>
       <c r="Z41" s="70"/>
-      <c r="AA41" s="102" t="s">
+      <c r="AA41" s="120" t="s">
         <v>51</v>
       </c>
-      <c r="AB41" s="103"/>
-      <c r="AC41" s="103"/>
-      <c r="AD41" s="103"/>
-      <c r="AE41" s="103"/>
-      <c r="AF41" s="97"/>
+      <c r="AB41" s="121"/>
+      <c r="AC41" s="121"/>
+      <c r="AD41" s="121"/>
+      <c r="AE41" s="121"/>
+      <c r="AF41" s="167"/>
       <c r="AG41" s="71"/>
       <c r="AH41" s="71"/>
       <c r="AI41" s="71"/>
@@ -4689,13 +4685,13 @@
       <c r="AL41" s="71"/>
       <c r="AM41" s="71"/>
       <c r="AN41" s="40"/>
-      <c r="AO41" s="154"/>
+      <c r="AO41" s="113"/>
     </row>
     <row r="42" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="84" t="s">
         <v>77</v>
       </c>
-      <c r="B42" s="175"/>
+      <c r="B42" s="95"/>
       <c r="C42" s="42"/>
       <c r="D42" s="79"/>
       <c r="E42" s="72"/>
@@ -4705,27 +4701,27 @@
       <c r="I42" s="72"/>
       <c r="J42" s="72"/>
       <c r="K42" s="80"/>
-      <c r="L42" s="162"/>
-      <c r="M42" s="106"/>
-      <c r="N42" s="106"/>
-      <c r="O42" s="106"/>
-      <c r="P42" s="106"/>
-      <c r="Q42" s="106"/>
-      <c r="R42" s="106"/>
-      <c r="S42" s="107"/>
+      <c r="L42" s="118"/>
+      <c r="M42" s="124"/>
+      <c r="N42" s="124"/>
+      <c r="O42" s="124"/>
+      <c r="P42" s="124"/>
+      <c r="Q42" s="124"/>
+      <c r="R42" s="124"/>
+      <c r="S42" s="125"/>
       <c r="T42" s="70"/>
-      <c r="U42" s="105"/>
-      <c r="V42" s="106"/>
-      <c r="W42" s="106"/>
-      <c r="X42" s="106"/>
-      <c r="Y42" s="107"/>
+      <c r="U42" s="123"/>
+      <c r="V42" s="124"/>
+      <c r="W42" s="124"/>
+      <c r="X42" s="124"/>
+      <c r="Y42" s="125"/>
       <c r="Z42" s="70"/>
-      <c r="AA42" s="105"/>
-      <c r="AB42" s="106"/>
-      <c r="AC42" s="106"/>
-      <c r="AD42" s="106"/>
-      <c r="AE42" s="106"/>
-      <c r="AF42" s="97"/>
+      <c r="AA42" s="123"/>
+      <c r="AB42" s="124"/>
+      <c r="AC42" s="124"/>
+      <c r="AD42" s="124"/>
+      <c r="AE42" s="124"/>
+      <c r="AF42" s="167"/>
       <c r="AG42" s="71"/>
       <c r="AH42" s="71"/>
       <c r="AI42" s="71"/>
@@ -4734,13 +4730,13 @@
       <c r="AL42" s="71"/>
       <c r="AM42" s="71"/>
       <c r="AN42" s="40"/>
-      <c r="AO42" s="154"/>
+      <c r="AO42" s="113"/>
     </row>
     <row r="43" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="84" t="s">
         <v>86</v>
       </c>
-      <c r="B43" s="175"/>
+      <c r="B43" s="95"/>
       <c r="C43" s="42"/>
       <c r="D43" s="79"/>
       <c r="E43" s="72"/>
@@ -4750,27 +4746,27 @@
       <c r="I43" s="72"/>
       <c r="J43" s="72"/>
       <c r="K43" s="80"/>
-      <c r="L43" s="162"/>
-      <c r="M43" s="109"/>
-      <c r="N43" s="109"/>
-      <c r="O43" s="109"/>
-      <c r="P43" s="109"/>
-      <c r="Q43" s="109"/>
-      <c r="R43" s="109"/>
-      <c r="S43" s="110"/>
+      <c r="L43" s="118"/>
+      <c r="M43" s="127"/>
+      <c r="N43" s="127"/>
+      <c r="O43" s="127"/>
+      <c r="P43" s="127"/>
+      <c r="Q43" s="127"/>
+      <c r="R43" s="127"/>
+      <c r="S43" s="128"/>
       <c r="T43" s="70"/>
-      <c r="U43" s="108"/>
-      <c r="V43" s="109"/>
-      <c r="W43" s="109"/>
-      <c r="X43" s="109"/>
-      <c r="Y43" s="110"/>
+      <c r="U43" s="126"/>
+      <c r="V43" s="127"/>
+      <c r="W43" s="127"/>
+      <c r="X43" s="127"/>
+      <c r="Y43" s="128"/>
       <c r="Z43" s="70"/>
-      <c r="AA43" s="108"/>
-      <c r="AB43" s="109"/>
-      <c r="AC43" s="109"/>
-      <c r="AD43" s="109"/>
-      <c r="AE43" s="109"/>
-      <c r="AF43" s="97"/>
+      <c r="AA43" s="126"/>
+      <c r="AB43" s="127"/>
+      <c r="AC43" s="127"/>
+      <c r="AD43" s="127"/>
+      <c r="AE43" s="127"/>
+      <c r="AF43" s="167"/>
       <c r="AG43" s="71"/>
       <c r="AH43" s="71"/>
       <c r="AI43" s="71"/>
@@ -4779,13 +4775,13 @@
       <c r="AL43" s="71"/>
       <c r="AM43" s="71"/>
       <c r="AN43" s="40"/>
-      <c r="AO43" s="154"/>
+      <c r="AO43" s="113"/>
     </row>
     <row r="44" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="84" t="s">
         <v>95</v>
       </c>
-      <c r="B44" s="175"/>
+      <c r="B44" s="95"/>
       <c r="C44" s="42"/>
       <c r="D44" s="79"/>
       <c r="E44" s="72"/>
@@ -4795,27 +4791,27 @@
       <c r="I44" s="72"/>
       <c r="J44" s="72"/>
       <c r="K44" s="80"/>
-      <c r="L44" s="162"/>
-      <c r="M44" s="132"/>
-      <c r="N44" s="132"/>
-      <c r="O44" s="132"/>
-      <c r="P44" s="132"/>
-      <c r="Q44" s="132"/>
-      <c r="R44" s="132"/>
-      <c r="S44" s="133"/>
+      <c r="L44" s="118"/>
+      <c r="M44" s="105"/>
+      <c r="N44" s="105"/>
+      <c r="O44" s="105"/>
+      <c r="P44" s="105"/>
+      <c r="Q44" s="105"/>
+      <c r="R44" s="105"/>
+      <c r="S44" s="107"/>
       <c r="T44" s="71"/>
-      <c r="U44" s="134"/>
-      <c r="V44" s="132"/>
-      <c r="W44" s="132"/>
-      <c r="X44" s="132"/>
-      <c r="Y44" s="133"/>
+      <c r="U44" s="104"/>
+      <c r="V44" s="105"/>
+      <c r="W44" s="105"/>
+      <c r="X44" s="105"/>
+      <c r="Y44" s="107"/>
       <c r="Z44" s="71"/>
-      <c r="AA44" s="134"/>
-      <c r="AB44" s="132"/>
-      <c r="AC44" s="132"/>
-      <c r="AD44" s="132"/>
-      <c r="AE44" s="132"/>
-      <c r="AF44" s="97"/>
+      <c r="AA44" s="104"/>
+      <c r="AB44" s="105"/>
+      <c r="AC44" s="105"/>
+      <c r="AD44" s="105"/>
+      <c r="AE44" s="105"/>
+      <c r="AF44" s="167"/>
       <c r="AG44" s="71"/>
       <c r="AH44" s="71"/>
       <c r="AI44" s="71"/>
@@ -4824,13 +4820,13 @@
       <c r="AL44" s="71"/>
       <c r="AM44" s="71"/>
       <c r="AN44" s="40"/>
-      <c r="AO44" s="154"/>
+      <c r="AO44" s="113"/>
     </row>
     <row r="45" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="84" t="s">
         <v>94</v>
       </c>
-      <c r="B45" s="175"/>
+      <c r="B45" s="95"/>
       <c r="C45" s="42"/>
       <c r="D45" s="79"/>
       <c r="E45" s="72"/>
@@ -4840,8 +4836,8 @@
       <c r="I45" s="72"/>
       <c r="J45" s="72"/>
       <c r="K45" s="80"/>
-      <c r="L45" s="162"/>
-      <c r="M45" s="150"/>
+      <c r="L45" s="118"/>
+      <c r="M45" s="111"/>
       <c r="P45" s="18">
         <v>4</v>
       </c>
@@ -4849,28 +4845,28 @@
         <v>31</v>
       </c>
       <c r="R45" s="20"/>
-      <c r="S45" s="147"/>
+      <c r="S45" s="96"/>
       <c r="T45" s="71"/>
-      <c r="U45" s="147"/>
+      <c r="U45" s="96"/>
       <c r="V45" s="5">
         <v>4</v>
       </c>
-      <c r="W45" s="94" t="s">
+      <c r="W45" s="138" t="s">
         <v>31</v>
       </c>
-      <c r="X45" s="95"/>
-      <c r="Y45" s="147"/>
+      <c r="X45" s="139"/>
+      <c r="Y45" s="96"/>
       <c r="Z45" s="83"/>
-      <c r="AA45" s="147"/>
+      <c r="AA45" s="96"/>
       <c r="AB45" s="5">
         <v>6</v>
       </c>
-      <c r="AC45" s="94" t="s">
+      <c r="AC45" s="138" t="s">
         <v>31</v>
       </c>
-      <c r="AD45" s="95"/>
-      <c r="AE45" s="158"/>
-      <c r="AF45" s="97"/>
+      <c r="AD45" s="139"/>
+      <c r="AE45" s="108"/>
+      <c r="AF45" s="167"/>
       <c r="AG45" s="71"/>
       <c r="AH45" s="71"/>
       <c r="AI45" s="71"/>
@@ -4879,13 +4875,13 @@
       <c r="AL45" s="71"/>
       <c r="AM45" s="71"/>
       <c r="AN45" s="40"/>
-      <c r="AO45" s="154"/>
+      <c r="AO45" s="113"/>
     </row>
     <row r="46" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="84" t="s">
         <v>107</v>
       </c>
-      <c r="B46" s="175"/>
+      <c r="B46" s="95"/>
       <c r="C46" s="42"/>
       <c r="D46" s="79"/>
       <c r="E46" s="72"/>
@@ -4895,8 +4891,8 @@
       <c r="I46" s="72"/>
       <c r="J46" s="72"/>
       <c r="K46" s="80"/>
-      <c r="L46" s="162"/>
-      <c r="M46" s="151"/>
+      <c r="L46" s="118"/>
+      <c r="M46" s="99"/>
       <c r="P46" s="4" t="s">
         <v>32</v>
       </c>
@@ -4906,9 +4902,9 @@
       <c r="R46" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="S46" s="148"/>
+      <c r="S46" s="97"/>
       <c r="T46" s="71"/>
-      <c r="U46" s="148"/>
+      <c r="U46" s="97"/>
       <c r="V46" s="4" t="s">
         <v>32</v>
       </c>
@@ -4918,9 +4914,9 @@
       <c r="X46" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="Y46" s="148"/>
+      <c r="Y46" s="97"/>
       <c r="Z46" s="72"/>
-      <c r="AA46" s="148"/>
+      <c r="AA46" s="97"/>
       <c r="AB46" s="4" t="s">
         <v>32</v>
       </c>
@@ -4930,8 +4926,8 @@
       <c r="AD46" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="AE46" s="159"/>
-      <c r="AF46" s="97"/>
+      <c r="AE46" s="109"/>
+      <c r="AF46" s="167"/>
       <c r="AG46" s="71"/>
       <c r="AH46" s="71"/>
       <c r="AI46" s="71"/>
@@ -4940,13 +4936,13 @@
       <c r="AL46" s="71"/>
       <c r="AM46" s="71"/>
       <c r="AN46" s="40"/>
-      <c r="AO46" s="154"/>
+      <c r="AO46" s="113"/>
     </row>
     <row r="47" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="84" t="s">
         <v>108</v>
       </c>
-      <c r="B47" s="175"/>
+      <c r="B47" s="95"/>
       <c r="C47" s="42"/>
       <c r="D47" s="79"/>
       <c r="E47" s="72"/>
@@ -4956,9 +4952,9 @@
       <c r="I47" s="72"/>
       <c r="J47" s="72"/>
       <c r="K47" s="80"/>
-      <c r="L47" s="162"/>
-      <c r="M47" s="151"/>
-      <c r="P47" s="144" t="s">
+      <c r="L47" s="118"/>
+      <c r="M47" s="99"/>
+      <c r="P47" s="140" t="s">
         <v>46</v>
       </c>
       <c r="Q47" s="11" t="str">
@@ -4966,10 +4962,10 @@
         <v>A3</v>
       </c>
       <c r="R47" s="6"/>
-      <c r="S47" s="148"/>
+      <c r="S47" s="97"/>
       <c r="T47" s="71"/>
-      <c r="U47" s="148"/>
-      <c r="V47" s="99" t="s">
+      <c r="U47" s="97"/>
+      <c r="V47" s="101" t="s">
         <v>50</v>
       </c>
       <c r="W47" s="11" t="str">
@@ -4977,10 +4973,10 @@
         <v>G1</v>
       </c>
       <c r="X47" s="6"/>
-      <c r="Y47" s="148"/>
+      <c r="Y47" s="97"/>
       <c r="Z47" s="77"/>
-      <c r="AA47" s="148"/>
-      <c r="AB47" s="144" t="s">
+      <c r="AA47" s="97"/>
+      <c r="AB47" s="140" t="s">
         <v>57</v>
       </c>
       <c r="AC47" s="21" t="str">
@@ -4988,8 +4984,8 @@
         <v>WF3</v>
       </c>
       <c r="AD47" s="26"/>
-      <c r="AE47" s="159"/>
-      <c r="AF47" s="97"/>
+      <c r="AE47" s="109"/>
+      <c r="AF47" s="167"/>
       <c r="AG47" s="71"/>
       <c r="AH47" s="71"/>
       <c r="AI47" s="71"/>
@@ -4998,13 +4994,13 @@
       <c r="AL47" s="71"/>
       <c r="AM47" s="71"/>
       <c r="AN47" s="40"/>
-      <c r="AO47" s="154"/>
+      <c r="AO47" s="113"/>
     </row>
     <row r="48" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="84" t="s">
         <v>97</v>
       </c>
-      <c r="B48" s="175"/>
+      <c r="B48" s="95"/>
       <c r="C48" s="42"/>
       <c r="D48" s="79"/>
       <c r="E48" s="72"/>
@@ -5014,34 +5010,34 @@
       <c r="I48" s="72"/>
       <c r="J48" s="72"/>
       <c r="K48" s="80"/>
-      <c r="L48" s="162"/>
-      <c r="M48" s="151"/>
-      <c r="P48" s="145"/>
+      <c r="L48" s="118"/>
+      <c r="M48" s="99"/>
+      <c r="P48" s="141"/>
       <c r="Q48" s="12" t="str">
         <f>IF(ISBLANK($R$27),"C3",$R$27)</f>
         <v>C3</v>
       </c>
       <c r="R48" s="14"/>
-      <c r="S48" s="148"/>
+      <c r="S48" s="97"/>
       <c r="T48" s="71"/>
-      <c r="U48" s="148"/>
-      <c r="V48" s="100"/>
+      <c r="U48" s="97"/>
+      <c r="V48" s="102"/>
       <c r="W48" s="12" t="str">
         <f>IF(ISBLANK($R$52),"H2",$R$52)</f>
         <v>H2</v>
       </c>
       <c r="X48" s="14"/>
-      <c r="Y48" s="148"/>
+      <c r="Y48" s="97"/>
       <c r="Z48" s="77"/>
-      <c r="AA48" s="148"/>
-      <c r="AB48" s="145"/>
+      <c r="AA48" s="97"/>
+      <c r="AB48" s="141"/>
       <c r="AC48" s="22" t="str">
         <f>IF(ISBLANK($X$47),"I1",$X$47)</f>
         <v>I1</v>
       </c>
       <c r="AD48" s="25"/>
-      <c r="AE48" s="159"/>
-      <c r="AF48" s="97"/>
+      <c r="AE48" s="109"/>
+      <c r="AF48" s="167"/>
       <c r="AG48" s="71"/>
       <c r="AH48" s="71"/>
       <c r="AI48" s="71"/>
@@ -5050,13 +5046,13 @@
       <c r="AL48" s="71"/>
       <c r="AM48" s="71"/>
       <c r="AN48" s="40"/>
-      <c r="AO48" s="154"/>
+      <c r="AO48" s="113"/>
     </row>
     <row r="49" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="84" t="s">
         <v>61</v>
       </c>
-      <c r="B49" s="175"/>
+      <c r="B49" s="95"/>
       <c r="C49" s="42"/>
       <c r="D49" s="79"/>
       <c r="E49" s="72"/>
@@ -5066,34 +5062,34 @@
       <c r="I49" s="72"/>
       <c r="J49" s="72"/>
       <c r="K49" s="80"/>
-      <c r="L49" s="162"/>
-      <c r="M49" s="151"/>
-      <c r="P49" s="145"/>
+      <c r="L49" s="118"/>
+      <c r="M49" s="99"/>
+      <c r="P49" s="141"/>
       <c r="Q49" s="12" t="str">
         <f>IF(ISBLANK($R$24),"B4",$R$24)</f>
         <v>B4</v>
       </c>
       <c r="R49" s="7"/>
-      <c r="S49" s="148"/>
+      <c r="S49" s="97"/>
       <c r="T49" s="71"/>
-      <c r="U49" s="148"/>
-      <c r="V49" s="100"/>
+      <c r="U49" s="97"/>
+      <c r="V49" s="102"/>
       <c r="W49" s="12" t="str">
         <f>IF(ISBLANK($X$19),"E3",$X$19)</f>
         <v>E3</v>
       </c>
       <c r="X49" s="7"/>
-      <c r="Y49" s="148"/>
+      <c r="Y49" s="97"/>
       <c r="Z49" s="77"/>
-      <c r="AA49" s="148"/>
-      <c r="AB49" s="146"/>
+      <c r="AA49" s="97"/>
+      <c r="AB49" s="142"/>
       <c r="AC49" s="22" t="str">
         <f>IF(ISBLANK($X$52),"J2",$X$52)</f>
         <v>J2</v>
       </c>
       <c r="AD49" s="24"/>
-      <c r="AE49" s="159"/>
-      <c r="AF49" s="97"/>
+      <c r="AE49" s="109"/>
+      <c r="AF49" s="167"/>
       <c r="AG49" s="71"/>
       <c r="AH49" s="71"/>
       <c r="AI49" s="71"/>
@@ -5102,13 +5098,13 @@
       <c r="AL49" s="71"/>
       <c r="AM49" s="71"/>
       <c r="AN49" s="40"/>
-      <c r="AO49" s="154"/>
+      <c r="AO49" s="113"/>
     </row>
     <row r="50" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="84" t="s">
         <v>111</v>
       </c>
-      <c r="B50" s="175"/>
+      <c r="B50" s="95"/>
       <c r="C50" s="41"/>
       <c r="D50" s="71"/>
       <c r="E50" s="73"/>
@@ -5118,27 +5114,27 @@
       <c r="I50" s="72"/>
       <c r="J50" s="72"/>
       <c r="K50" s="71"/>
-      <c r="L50" s="162"/>
-      <c r="M50" s="151"/>
-      <c r="P50" s="146"/>
+      <c r="L50" s="118"/>
+      <c r="M50" s="99"/>
+      <c r="P50" s="142"/>
       <c r="Q50" s="12" t="str">
         <f>IF(ISBLANK($R$32),"D4",$R$32)</f>
         <v>D4</v>
       </c>
       <c r="R50" s="8"/>
-      <c r="S50" s="148"/>
+      <c r="S50" s="97"/>
       <c r="T50" s="71"/>
-      <c r="U50" s="148"/>
-      <c r="V50" s="101"/>
+      <c r="U50" s="97"/>
+      <c r="V50" s="103"/>
       <c r="W50" s="12" t="str">
         <f>IF(ISBLANK($X$24),"F4",$X$24)</f>
         <v>F4</v>
       </c>
       <c r="X50" s="8"/>
-      <c r="Y50" s="148"/>
+      <c r="Y50" s="97"/>
       <c r="Z50" s="77"/>
-      <c r="AA50" s="148"/>
-      <c r="AB50" s="100" t="s">
+      <c r="AA50" s="97"/>
+      <c r="AB50" s="102" t="s">
         <v>58</v>
       </c>
       <c r="AC50" s="21" t="str">
@@ -5146,8 +5142,8 @@
         <v>WF4</v>
       </c>
       <c r="AD50" s="26"/>
-      <c r="AE50" s="159"/>
-      <c r="AF50" s="97"/>
+      <c r="AE50" s="109"/>
+      <c r="AF50" s="167"/>
       <c r="AG50" s="71"/>
       <c r="AH50" s="71"/>
       <c r="AI50" s="71"/>
@@ -5156,13 +5152,13 @@
       <c r="AL50" s="71"/>
       <c r="AM50" s="71"/>
       <c r="AN50" s="40"/>
-      <c r="AO50" s="154"/>
+      <c r="AO50" s="113"/>
     </row>
     <row r="51" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="84" t="s">
         <v>60</v>
       </c>
-      <c r="B51" s="175"/>
+      <c r="B51" s="95"/>
       <c r="C51" s="41"/>
       <c r="D51" s="71"/>
       <c r="E51" s="73"/>
@@ -5172,9 +5168,9 @@
       <c r="I51" s="72"/>
       <c r="J51" s="72"/>
       <c r="K51" s="71"/>
-      <c r="L51" s="162"/>
-      <c r="M51" s="151"/>
-      <c r="P51" s="144" t="s">
+      <c r="L51" s="118"/>
+      <c r="M51" s="99"/>
+      <c r="P51" s="140" t="s">
         <v>47</v>
       </c>
       <c r="Q51" s="11" t="str">
@@ -5182,10 +5178,10 @@
         <v>B3</v>
       </c>
       <c r="R51" s="6"/>
-      <c r="S51" s="148"/>
+      <c r="S51" s="97"/>
       <c r="T51" s="71"/>
-      <c r="U51" s="148"/>
-      <c r="V51" s="99" t="s">
+      <c r="U51" s="97"/>
+      <c r="V51" s="101" t="s">
         <v>49</v>
       </c>
       <c r="W51" s="11" t="str">
@@ -5193,17 +5189,17 @@
         <v>H1</v>
       </c>
       <c r="X51" s="6"/>
-      <c r="Y51" s="148"/>
+      <c r="Y51" s="97"/>
       <c r="Z51" s="77"/>
-      <c r="AA51" s="148"/>
-      <c r="AB51" s="100"/>
+      <c r="AA51" s="97"/>
+      <c r="AB51" s="102"/>
       <c r="AC51" s="22" t="str">
         <f>IF(ISBLANK($X$51),"J1",$X$51)</f>
         <v>J1</v>
       </c>
       <c r="AD51" s="25"/>
-      <c r="AE51" s="159"/>
-      <c r="AF51" s="97"/>
+      <c r="AE51" s="109"/>
+      <c r="AF51" s="167"/>
       <c r="AG51" s="71"/>
       <c r="AH51" s="71"/>
       <c r="AI51" s="71"/>
@@ -5212,13 +5208,13 @@
       <c r="AL51" s="71"/>
       <c r="AM51" s="71"/>
       <c r="AN51" s="40"/>
-      <c r="AO51" s="154"/>
+      <c r="AO51" s="113"/>
     </row>
     <row r="52" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="84" t="s">
         <v>136</v>
       </c>
-      <c r="B52" s="175"/>
+      <c r="B52" s="95"/>
       <c r="C52" s="41"/>
       <c r="D52" s="71"/>
       <c r="E52" s="73"/>
@@ -5228,34 +5224,34 @@
       <c r="I52" s="72"/>
       <c r="J52" s="72"/>
       <c r="K52" s="71"/>
-      <c r="L52" s="162"/>
-      <c r="M52" s="151"/>
-      <c r="P52" s="145"/>
+      <c r="L52" s="118"/>
+      <c r="M52" s="99"/>
+      <c r="P52" s="141"/>
       <c r="Q52" s="12" t="str">
         <f>IF(ISBLANK($R$31),"D3",$R$31)</f>
         <v>D3</v>
       </c>
       <c r="R52" s="14"/>
-      <c r="S52" s="148"/>
+      <c r="S52" s="97"/>
       <c r="T52" s="71"/>
-      <c r="U52" s="148"/>
-      <c r="V52" s="100"/>
+      <c r="U52" s="97"/>
+      <c r="V52" s="102"/>
       <c r="W52" s="12" t="str">
         <f>IF(ISBLANK($R$48),"G2",$R$48)</f>
         <v>G2</v>
       </c>
       <c r="X52" s="14"/>
-      <c r="Y52" s="148"/>
+      <c r="Y52" s="97"/>
       <c r="Z52" s="77"/>
-      <c r="AA52" s="149"/>
-      <c r="AB52" s="100"/>
+      <c r="AA52" s="98"/>
+      <c r="AB52" s="102"/>
       <c r="AC52" s="22" t="str">
         <f>IF(ISBLANK($X$48),"I2",$X$48)</f>
         <v>I2</v>
       </c>
       <c r="AD52" s="25"/>
-      <c r="AE52" s="160"/>
-      <c r="AF52" s="97"/>
+      <c r="AE52" s="110"/>
+      <c r="AF52" s="167"/>
       <c r="AG52" s="71"/>
       <c r="AH52" s="71"/>
       <c r="AI52" s="71"/>
@@ -5264,13 +5260,13 @@
       <c r="AL52" s="71"/>
       <c r="AM52" s="71"/>
       <c r="AN52" s="40"/>
-      <c r="AO52" s="154"/>
+      <c r="AO52" s="113"/>
     </row>
     <row r="53" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="84" t="s">
         <v>65</v>
       </c>
-      <c r="B53" s="175"/>
+      <c r="B53" s="95"/>
       <c r="C53" s="41"/>
       <c r="D53" s="71"/>
       <c r="E53" s="73"/>
@@ -5280,31 +5276,31 @@
       <c r="I53" s="72"/>
       <c r="J53" s="72"/>
       <c r="K53" s="71"/>
-      <c r="L53" s="162"/>
-      <c r="M53" s="151"/>
-      <c r="P53" s="145"/>
+      <c r="L53" s="118"/>
+      <c r="M53" s="99"/>
+      <c r="P53" s="141"/>
       <c r="Q53" s="12" t="str">
         <f>IF(ISBLANK($R$20),"A4",$R$20)</f>
         <v>A4</v>
       </c>
       <c r="R53" s="7"/>
-      <c r="S53" s="148"/>
+      <c r="S53" s="97"/>
       <c r="T53" s="71"/>
-      <c r="U53" s="148"/>
-      <c r="V53" s="100"/>
+      <c r="U53" s="97"/>
+      <c r="V53" s="102"/>
       <c r="W53" s="12" t="str">
         <f>IF(ISBLANK($X$23),"F3",$X$23)</f>
         <v>F3</v>
       </c>
       <c r="X53" s="7"/>
-      <c r="Y53" s="148"/>
+      <c r="Y53" s="97"/>
       <c r="Z53" s="77"/>
-      <c r="AA53" s="134"/>
-      <c r="AB53" s="132"/>
-      <c r="AC53" s="132"/>
-      <c r="AD53" s="132"/>
-      <c r="AE53" s="132"/>
-      <c r="AF53" s="97"/>
+      <c r="AA53" s="104"/>
+      <c r="AB53" s="105"/>
+      <c r="AC53" s="105"/>
+      <c r="AD53" s="105"/>
+      <c r="AE53" s="105"/>
+      <c r="AF53" s="167"/>
       <c r="AG53" s="71"/>
       <c r="AH53" s="71"/>
       <c r="AI53" s="71"/>
@@ -5313,13 +5309,13 @@
       <c r="AL53" s="71"/>
       <c r="AM53" s="71"/>
       <c r="AN53" s="40"/>
-      <c r="AO53" s="154"/>
+      <c r="AO53" s="113"/>
     </row>
     <row r="54" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="84" t="s">
         <v>78</v>
       </c>
-      <c r="B54" s="175"/>
+      <c r="B54" s="95"/>
       <c r="C54" s="41"/>
       <c r="D54" s="71"/>
       <c r="E54" s="73"/>
@@ -5329,31 +5325,31 @@
       <c r="I54" s="72"/>
       <c r="J54" s="72"/>
       <c r="K54" s="71"/>
-      <c r="L54" s="162"/>
-      <c r="M54" s="152"/>
-      <c r="P54" s="146"/>
+      <c r="L54" s="118"/>
+      <c r="M54" s="100"/>
+      <c r="P54" s="142"/>
       <c r="Q54" s="12" t="str">
         <f>IF(ISBLANK($R$28),"C4",$R$28)</f>
         <v>C4</v>
       </c>
       <c r="R54" s="7"/>
-      <c r="S54" s="149"/>
+      <c r="S54" s="98"/>
       <c r="T54" s="71"/>
-      <c r="U54" s="149"/>
-      <c r="V54" s="101"/>
+      <c r="U54" s="98"/>
+      <c r="V54" s="103"/>
       <c r="W54" s="13" t="str">
         <f>IF(ISBLANK($X$20),"E4",$X$20)</f>
         <v>E4</v>
       </c>
       <c r="X54" s="8"/>
-      <c r="Y54" s="149"/>
+      <c r="Y54" s="98"/>
       <c r="Z54" s="77"/>
       <c r="AA54" s="71"/>
       <c r="AB54" s="71"/>
       <c r="AC54" s="71"/>
       <c r="AD54" s="71"/>
       <c r="AE54" s="71"/>
-      <c r="AF54" s="97"/>
+      <c r="AF54" s="167"/>
       <c r="AG54" s="71"/>
       <c r="AH54" s="71"/>
       <c r="AI54" s="71"/>
@@ -5362,13 +5358,13 @@
       <c r="AL54" s="71"/>
       <c r="AM54" s="71"/>
       <c r="AN54" s="40"/>
-      <c r="AO54" s="154"/>
+      <c r="AO54" s="113"/>
     </row>
     <row r="55" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="84" t="s">
         <v>85</v>
       </c>
-      <c r="B55" s="175"/>
+      <c r="B55" s="95"/>
       <c r="C55" s="41"/>
       <c r="D55" s="71"/>
       <c r="E55" s="73"/>
@@ -5378,27 +5374,27 @@
       <c r="I55" s="72"/>
       <c r="J55" s="72"/>
       <c r="K55" s="71"/>
-      <c r="L55" s="162"/>
-      <c r="M55" s="132"/>
-      <c r="N55" s="132"/>
-      <c r="O55" s="132"/>
-      <c r="P55" s="132"/>
-      <c r="Q55" s="132"/>
-      <c r="R55" s="132"/>
-      <c r="S55" s="133"/>
+      <c r="L55" s="118"/>
+      <c r="M55" s="105"/>
+      <c r="N55" s="105"/>
+      <c r="O55" s="105"/>
+      <c r="P55" s="105"/>
+      <c r="Q55" s="105"/>
+      <c r="R55" s="105"/>
+      <c r="S55" s="107"/>
       <c r="T55" s="71"/>
-      <c r="U55" s="134"/>
-      <c r="V55" s="132"/>
-      <c r="W55" s="164"/>
-      <c r="X55" s="132"/>
-      <c r="Y55" s="133"/>
+      <c r="U55" s="104"/>
+      <c r="V55" s="105"/>
+      <c r="W55" s="106"/>
+      <c r="X55" s="105"/>
+      <c r="Y55" s="107"/>
       <c r="Z55" s="71"/>
       <c r="AA55" s="71"/>
       <c r="AB55" s="71"/>
       <c r="AC55" s="71"/>
       <c r="AD55" s="71"/>
       <c r="AE55" s="71"/>
-      <c r="AF55" s="97"/>
+      <c r="AF55" s="167"/>
       <c r="AG55" s="71"/>
       <c r="AH55" s="71"/>
       <c r="AI55" s="71"/>
@@ -5407,13 +5403,13 @@
       <c r="AL55" s="71"/>
       <c r="AM55" s="71"/>
       <c r="AN55" s="40"/>
-      <c r="AO55" s="154"/>
+      <c r="AO55" s="113"/>
     </row>
     <row r="56" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="84" t="s">
         <v>81</v>
       </c>
-      <c r="B56" s="175"/>
+      <c r="B56" s="95"/>
       <c r="C56" s="41"/>
       <c r="D56" s="71"/>
       <c r="E56" s="73"/>
@@ -5423,7 +5419,7 @@
       <c r="I56" s="72"/>
       <c r="J56" s="72"/>
       <c r="K56" s="71"/>
-      <c r="L56" s="162"/>
+      <c r="L56" s="118"/>
       <c r="M56" s="71"/>
       <c r="N56" s="71"/>
       <c r="O56" s="71"/>
@@ -5442,7 +5438,7 @@
       <c r="AB56" s="71"/>
       <c r="AD56" s="71"/>
       <c r="AE56" s="71"/>
-      <c r="AF56" s="97"/>
+      <c r="AF56" s="167"/>
       <c r="AG56" s="71"/>
       <c r="AH56" s="71"/>
       <c r="AI56" s="71"/>
@@ -5451,13 +5447,13 @@
       <c r="AL56" s="71"/>
       <c r="AM56" s="71"/>
       <c r="AN56" s="40"/>
-      <c r="AO56" s="154"/>
+      <c r="AO56" s="113"/>
     </row>
     <row r="57" spans="1:41" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A57" s="84" t="s">
         <v>80</v>
       </c>
-      <c r="B57" s="175"/>
+      <c r="B57" s="95"/>
       <c r="C57" s="43"/>
       <c r="D57" s="44"/>
       <c r="E57" s="45"/>
@@ -5467,7 +5463,7 @@
       <c r="I57" s="54"/>
       <c r="J57" s="54"/>
       <c r="K57" s="44"/>
-      <c r="L57" s="163"/>
+      <c r="L57" s="119"/>
       <c r="M57" s="44"/>
       <c r="N57" s="44"/>
       <c r="O57" s="44"/>
@@ -5487,7 +5483,7 @@
       <c r="AC57" s="44"/>
       <c r="AD57" s="44"/>
       <c r="AE57" s="44"/>
-      <c r="AF57" s="98"/>
+      <c r="AF57" s="168"/>
       <c r="AG57" s="44"/>
       <c r="AH57" s="44"/>
       <c r="AI57" s="44"/>
@@ -5496,52 +5492,52 @@
       <c r="AL57" s="44"/>
       <c r="AM57" s="44"/>
       <c r="AN57" s="46"/>
-      <c r="AO57" s="154"/>
+      <c r="AO57" s="113"/>
     </row>
     <row r="58" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="84" t="s">
         <v>82</v>
       </c>
-      <c r="B58" s="175"/>
-      <c r="C58" s="156"/>
-      <c r="D58" s="156"/>
-      <c r="E58" s="156"/>
-      <c r="F58" s="156"/>
-      <c r="G58" s="156"/>
-      <c r="H58" s="156"/>
-      <c r="I58" s="156"/>
-      <c r="J58" s="156"/>
-      <c r="K58" s="156"/>
-      <c r="L58" s="156"/>
-      <c r="M58" s="156"/>
-      <c r="N58" s="156"/>
-      <c r="O58" s="156"/>
-      <c r="P58" s="156"/>
-      <c r="Q58" s="156"/>
-      <c r="R58" s="156"/>
-      <c r="S58" s="156"/>
-      <c r="T58" s="156"/>
-      <c r="U58" s="156"/>
-      <c r="V58" s="156"/>
-      <c r="W58" s="156"/>
-      <c r="X58" s="156"/>
-      <c r="Y58" s="156"/>
-      <c r="Z58" s="156"/>
-      <c r="AA58" s="156"/>
-      <c r="AB58" s="156"/>
-      <c r="AC58" s="156"/>
-      <c r="AD58" s="156"/>
-      <c r="AE58" s="156"/>
-      <c r="AF58" s="156"/>
-      <c r="AG58" s="156"/>
-      <c r="AH58" s="156"/>
-      <c r="AI58" s="156"/>
-      <c r="AJ58" s="156"/>
-      <c r="AK58" s="156"/>
-      <c r="AL58" s="156"/>
-      <c r="AM58" s="156"/>
-      <c r="AN58" s="156"/>
-      <c r="AO58" s="154"/>
+      <c r="B58" s="95"/>
+      <c r="C58" s="115"/>
+      <c r="D58" s="115"/>
+      <c r="E58" s="115"/>
+      <c r="F58" s="115"/>
+      <c r="G58" s="115"/>
+      <c r="H58" s="115"/>
+      <c r="I58" s="115"/>
+      <c r="J58" s="115"/>
+      <c r="K58" s="115"/>
+      <c r="L58" s="115"/>
+      <c r="M58" s="115"/>
+      <c r="N58" s="115"/>
+      <c r="O58" s="115"/>
+      <c r="P58" s="115"/>
+      <c r="Q58" s="115"/>
+      <c r="R58" s="115"/>
+      <c r="S58" s="115"/>
+      <c r="T58" s="115"/>
+      <c r="U58" s="115"/>
+      <c r="V58" s="115"/>
+      <c r="W58" s="115"/>
+      <c r="X58" s="115"/>
+      <c r="Y58" s="115"/>
+      <c r="Z58" s="115"/>
+      <c r="AA58" s="115"/>
+      <c r="AB58" s="115"/>
+      <c r="AC58" s="115"/>
+      <c r="AD58" s="115"/>
+      <c r="AE58" s="115"/>
+      <c r="AF58" s="115"/>
+      <c r="AG58" s="115"/>
+      <c r="AH58" s="115"/>
+      <c r="AI58" s="115"/>
+      <c r="AJ58" s="115"/>
+      <c r="AK58" s="115"/>
+      <c r="AL58" s="115"/>
+      <c r="AM58" s="115"/>
+      <c r="AN58" s="115"/>
+      <c r="AO58" s="113"/>
     </row>
     <row r="59" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="84" t="s">
@@ -5586,7 +5582,7 @@
       <c r="AL59" s="55"/>
       <c r="AM59" s="55"/>
       <c r="AN59" s="55"/>
-      <c r="AO59" s="154"/>
+      <c r="AO59" s="113"/>
     </row>
     <row r="60" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="84" t="s">
@@ -5631,7 +5627,7 @@
       <c r="AL60" s="55"/>
       <c r="AM60" s="55"/>
       <c r="AN60" s="55"/>
-      <c r="AO60" s="154"/>
+      <c r="AO60" s="113"/>
     </row>
     <row r="61" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="84" t="s">
@@ -5676,7 +5672,7 @@
       <c r="AL61" s="55"/>
       <c r="AM61" s="55"/>
       <c r="AN61" s="55"/>
-      <c r="AO61" s="154"/>
+      <c r="AO61" s="113"/>
     </row>
     <row r="62" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="84" t="s">
@@ -5721,7 +5717,7 @@
       <c r="AL62" s="55"/>
       <c r="AM62" s="55"/>
       <c r="AN62" s="55"/>
-      <c r="AO62" s="154"/>
+      <c r="AO62" s="113"/>
     </row>
     <row r="63" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="84" t="s">
@@ -5766,7 +5762,7 @@
       <c r="AL63" s="55"/>
       <c r="AM63" s="55"/>
       <c r="AN63" s="55"/>
-      <c r="AO63" s="154"/>
+      <c r="AO63" s="113"/>
     </row>
     <row r="64" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="84" t="s">
@@ -5811,7 +5807,7 @@
       <c r="AL64" s="55"/>
       <c r="AM64" s="55"/>
       <c r="AN64" s="55"/>
-      <c r="AO64" s="154"/>
+      <c r="AO64" s="113"/>
     </row>
     <row r="65" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="84" t="s">
@@ -5856,7 +5852,7 @@
       <c r="AL65" s="55"/>
       <c r="AM65" s="55"/>
       <c r="AN65" s="55"/>
-      <c r="AO65" s="154"/>
+      <c r="AO65" s="113"/>
     </row>
     <row r="66" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="84" t="s">
@@ -5901,7 +5897,7 @@
       <c r="AL66" s="55"/>
       <c r="AM66" s="55"/>
       <c r="AN66" s="55"/>
-      <c r="AO66" s="154"/>
+      <c r="AO66" s="113"/>
     </row>
     <row r="67" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="84" t="s">
@@ -5946,7 +5942,7 @@
       <c r="AL67" s="55"/>
       <c r="AM67" s="55"/>
       <c r="AN67" s="55"/>
-      <c r="AO67" s="154"/>
+      <c r="AO67" s="113"/>
     </row>
     <row r="68" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="84" t="s">
@@ -5991,7 +5987,7 @@
       <c r="AL68" s="55"/>
       <c r="AM68" s="55"/>
       <c r="AN68" s="55"/>
-      <c r="AO68" s="154"/>
+      <c r="AO68" s="113"/>
     </row>
     <row r="69" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="84" t="s">
@@ -6036,7 +6032,7 @@
       <c r="AL69" s="55"/>
       <c r="AM69" s="55"/>
       <c r="AN69" s="55"/>
-      <c r="AO69" s="154"/>
+      <c r="AO69" s="113"/>
     </row>
     <row r="70" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="84" t="s">
@@ -6081,7 +6077,7 @@
       <c r="AL70" s="55"/>
       <c r="AM70" s="55"/>
       <c r="AN70" s="55"/>
-      <c r="AO70" s="154"/>
+      <c r="AO70" s="113"/>
     </row>
     <row r="71" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="84" t="s">
@@ -6126,7 +6122,7 @@
       <c r="AL71" s="55"/>
       <c r="AM71" s="55"/>
       <c r="AN71" s="55"/>
-      <c r="AO71" s="154"/>
+      <c r="AO71" s="113"/>
     </row>
     <row r="72" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="84" t="s">
@@ -6171,7 +6167,7 @@
       <c r="AL72" s="55"/>
       <c r="AM72" s="55"/>
       <c r="AN72" s="55"/>
-      <c r="AO72" s="154"/>
+      <c r="AO72" s="113"/>
     </row>
     <row r="73" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="84" t="s">
@@ -6216,7 +6212,7 @@
       <c r="AL73" s="55"/>
       <c r="AM73" s="55"/>
       <c r="AN73" s="55"/>
-      <c r="AO73" s="154"/>
+      <c r="AO73" s="113"/>
     </row>
     <row r="74" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="84" t="s">
@@ -6261,7 +6257,7 @@
       <c r="AL74" s="55"/>
       <c r="AM74" s="55"/>
       <c r="AN74" s="55"/>
-      <c r="AO74" s="154"/>
+      <c r="AO74" s="113"/>
     </row>
     <row r="75" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="84" t="s">
@@ -6306,7 +6302,7 @@
       <c r="AL75" s="55"/>
       <c r="AM75" s="55"/>
       <c r="AN75" s="55"/>
-      <c r="AO75" s="154"/>
+      <c r="AO75" s="113"/>
     </row>
     <row r="76" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="84" t="s">
@@ -6351,7 +6347,7 @@
       <c r="AL76" s="55"/>
       <c r="AM76" s="55"/>
       <c r="AN76" s="55"/>
-      <c r="AO76" s="154"/>
+      <c r="AO76" s="113"/>
     </row>
     <row r="77" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="84" t="s">
@@ -6396,7 +6392,7 @@
       <c r="AL77" s="55"/>
       <c r="AM77" s="55"/>
       <c r="AN77" s="55"/>
-      <c r="AO77" s="154"/>
+      <c r="AO77" s="113"/>
     </row>
     <row r="78" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="84" t="s">
@@ -6441,7 +6437,7 @@
       <c r="AL78" s="55"/>
       <c r="AM78" s="55"/>
       <c r="AN78" s="55"/>
-      <c r="AO78" s="154"/>
+      <c r="AO78" s="113"/>
     </row>
     <row r="79" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="84" t="s">
@@ -6486,14 +6482,14 @@
       <c r="AL79" s="55"/>
       <c r="AM79" s="55"/>
       <c r="AN79" s="55"/>
-      <c r="AO79" s="154"/>
+      <c r="AO79" s="113"/>
     </row>
     <row r="80" spans="1:41" s="64" customFormat="1" ht="30" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A80" s="84" t="s">
         <v>99</v>
       </c>
       <c r="B80" s="63"/>
-      <c r="AO80" s="155"/>
+      <c r="AO80" s="114"/>
     </row>
     <row r="81" spans="1:1" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="84" t="s">
@@ -6617,6 +6613,68 @@
     </row>
   </sheetData>
   <mergeCells count="78">
+    <mergeCell ref="H13:J14"/>
+    <mergeCell ref="D13:E14"/>
+    <mergeCell ref="AJ15:AL15"/>
+    <mergeCell ref="AJ29:AL29"/>
+    <mergeCell ref="AF2:AF57"/>
+    <mergeCell ref="P17:P20"/>
+    <mergeCell ref="P21:P24"/>
+    <mergeCell ref="P25:P28"/>
+    <mergeCell ref="P29:P32"/>
+    <mergeCell ref="U11:Y13"/>
+    <mergeCell ref="W15:X15"/>
+    <mergeCell ref="V17:V20"/>
+    <mergeCell ref="V21:V24"/>
+    <mergeCell ref="M11:S13"/>
+    <mergeCell ref="Q15:R15"/>
+    <mergeCell ref="C2:K6"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="C8:K8"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="M5:AE7"/>
+    <mergeCell ref="AA11:AE13"/>
+    <mergeCell ref="AC15:AD15"/>
+    <mergeCell ref="AB17:AB20"/>
+    <mergeCell ref="M33:S33"/>
+    <mergeCell ref="U25:Y25"/>
+    <mergeCell ref="AA21:AE21"/>
+    <mergeCell ref="AA14:AE14"/>
+    <mergeCell ref="U14:Y14"/>
+    <mergeCell ref="M55:S55"/>
+    <mergeCell ref="M36:AE38"/>
+    <mergeCell ref="U41:Y43"/>
+    <mergeCell ref="W45:X45"/>
+    <mergeCell ref="V47:V50"/>
+    <mergeCell ref="V51:V54"/>
+    <mergeCell ref="AA41:AE43"/>
+    <mergeCell ref="AC45:AD45"/>
+    <mergeCell ref="M44:S44"/>
+    <mergeCell ref="P47:P50"/>
+    <mergeCell ref="P51:P54"/>
+    <mergeCell ref="M41:S43"/>
+    <mergeCell ref="U45:U54"/>
+    <mergeCell ref="AB47:AB49"/>
+    <mergeCell ref="AB50:AB52"/>
+    <mergeCell ref="AA44:AE44"/>
+    <mergeCell ref="M45:M54"/>
+    <mergeCell ref="AO1:AO80"/>
+    <mergeCell ref="C58:AN58"/>
+    <mergeCell ref="C1:AN1"/>
+    <mergeCell ref="U15:U24"/>
+    <mergeCell ref="S15:S32"/>
+    <mergeCell ref="M15:M32"/>
+    <mergeCell ref="AE45:AE52"/>
+    <mergeCell ref="AA45:AA52"/>
+    <mergeCell ref="Y45:Y54"/>
+    <mergeCell ref="L2:L57"/>
+    <mergeCell ref="AH11:AM13"/>
+    <mergeCell ref="AI17:AI20"/>
+    <mergeCell ref="AH21:AM21"/>
+    <mergeCell ref="AH25:AM27"/>
+    <mergeCell ref="U44:Y44"/>
     <mergeCell ref="AG5:AN7"/>
     <mergeCell ref="B1:B58"/>
     <mergeCell ref="AH29:AH34"/>
@@ -6633,68 +6691,6 @@
     <mergeCell ref="U55:Y55"/>
     <mergeCell ref="AA53:AE53"/>
     <mergeCell ref="S45:S54"/>
-    <mergeCell ref="M45:M54"/>
-    <mergeCell ref="AO1:AO80"/>
-    <mergeCell ref="C58:AN58"/>
-    <mergeCell ref="C1:AN1"/>
-    <mergeCell ref="U15:U24"/>
-    <mergeCell ref="S15:S32"/>
-    <mergeCell ref="M15:M32"/>
-    <mergeCell ref="AE45:AE52"/>
-    <mergeCell ref="AA45:AA52"/>
-    <mergeCell ref="Y45:Y54"/>
-    <mergeCell ref="L2:L57"/>
-    <mergeCell ref="AH11:AM13"/>
-    <mergeCell ref="AI17:AI20"/>
-    <mergeCell ref="AH21:AM21"/>
-    <mergeCell ref="AH25:AM27"/>
-    <mergeCell ref="U44:Y44"/>
-    <mergeCell ref="M55:S55"/>
-    <mergeCell ref="M36:AE38"/>
-    <mergeCell ref="U41:Y43"/>
-    <mergeCell ref="W45:X45"/>
-    <mergeCell ref="V47:V50"/>
-    <mergeCell ref="V51:V54"/>
-    <mergeCell ref="AA41:AE43"/>
-    <mergeCell ref="AC45:AD45"/>
-    <mergeCell ref="M44:S44"/>
-    <mergeCell ref="P47:P50"/>
-    <mergeCell ref="P51:P54"/>
-    <mergeCell ref="M41:S43"/>
-    <mergeCell ref="U45:U54"/>
-    <mergeCell ref="AB47:AB49"/>
-    <mergeCell ref="AB50:AB52"/>
-    <mergeCell ref="AA44:AE44"/>
-    <mergeCell ref="M5:AE7"/>
-    <mergeCell ref="AA11:AE13"/>
-    <mergeCell ref="AC15:AD15"/>
-    <mergeCell ref="AB17:AB20"/>
-    <mergeCell ref="M33:S33"/>
-    <mergeCell ref="U25:Y25"/>
-    <mergeCell ref="AA21:AE21"/>
-    <mergeCell ref="AA14:AE14"/>
-    <mergeCell ref="U14:Y14"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="C8:K8"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="H13:J14"/>
-    <mergeCell ref="D13:E14"/>
-    <mergeCell ref="AJ15:AL15"/>
-    <mergeCell ref="AJ29:AL29"/>
-    <mergeCell ref="AF2:AF57"/>
-    <mergeCell ref="P17:P20"/>
-    <mergeCell ref="P21:P24"/>
-    <mergeCell ref="P25:P28"/>
-    <mergeCell ref="P29:P32"/>
-    <mergeCell ref="U11:Y13"/>
-    <mergeCell ref="W15:X15"/>
-    <mergeCell ref="V17:V20"/>
-    <mergeCell ref="V21:V24"/>
-    <mergeCell ref="M11:S13"/>
-    <mergeCell ref="Q15:R15"/>
-    <mergeCell ref="C2:K6"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="Q47">

</xml_diff>

<commit_message>
[FIX] - bracket auto loading put unknow player at last instead of first
</commit_message>
<xml_diff>
--- a/resources/template/rififi_bracket_solo_16.xlsx
+++ b/resources/template/rififi_bracket_solo_16.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hugor\GitHub\Asso\AssetsGenerator\resources\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71B8F226-4FFF-4343-82C4-8948BF67118F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85FF75EB-A9EB-4690-B1D0-5E7F1FC9031C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="5250" windowWidth="29040" windowHeight="16440" xr2:uid="{2F0D60C5-63AA-4767-A59B-0FBF4FA7B0CE}"/>
+    <workbookView xWindow="42075" yWindow="7530" windowWidth="21600" windowHeight="11835" xr2:uid="{2F0D60C5-63AA-4767-A59B-0FBF4FA7B0CE}"/>
   </bookViews>
   <sheets>
     <sheet name="Solo 16" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
[ADD] - Duo Top 8 generation from challonge website | [FIX] - Solo/Duo for Top 8 architecture
</commit_message>
<xml_diff>
--- a/resources/template/rififi_bracket_solo_16.xlsx
+++ b/resources/template/rififi_bracket_solo_16.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hugor\GitHub\Asso\AssetsGenerator\resources\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85FF75EB-A9EB-4690-B1D0-5E7F1FC9031C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{179F735B-543D-4481-AFFB-DC6FAFEBD35C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="42075" yWindow="7530" windowWidth="21600" windowHeight="11835" xr2:uid="{2F0D60C5-63AA-4767-A59B-0FBF4FA7B0CE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{2F0D60C5-63AA-4767-A59B-0FBF4FA7B0CE}"/>
   </bookViews>
   <sheets>
     <sheet name="Solo 16" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="167">
   <si>
     <t>RIFIFI sur le circuit #00</t>
   </si>
@@ -1339,6 +1339,240 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="15" fillId="4" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1372,242 +1606,8 @@
     <xf numFmtId="0" fontId="3" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="15" fillId="4" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2309,8 +2309,8 @@
     <col min="11" max="11" width="13.28515625" style="1" customWidth="1"/>
     <col min="12" max="12" width="10.7109375" style="1" customWidth="1"/>
     <col min="13" max="13" width="4.7109375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="29.28515625" style="1" hidden="1" customWidth="1"/>
-    <col min="15" max="15" width="36.5703125" style="1" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="16.42578125" style="1" hidden="1" customWidth="1"/>
+    <col min="15" max="15" width="18" style="1" hidden="1" customWidth="1"/>
     <col min="16" max="16" width="4.7109375" style="1" customWidth="1"/>
     <col min="17" max="18" width="30.7109375" style="1" customWidth="1"/>
     <col min="19" max="19" width="4.7109375" style="1" customWidth="1"/>
@@ -2337,64 +2337,64 @@
       <c r="A1" s="84" t="s">
         <v>133</v>
       </c>
-      <c r="B1" s="94"/>
-      <c r="C1" s="116"/>
-      <c r="D1" s="116"/>
-      <c r="E1" s="116"/>
-      <c r="F1" s="116"/>
-      <c r="G1" s="116"/>
-      <c r="H1" s="116"/>
-      <c r="I1" s="116"/>
-      <c r="J1" s="116"/>
-      <c r="K1" s="116"/>
-      <c r="L1" s="116"/>
-      <c r="M1" s="116"/>
-      <c r="N1" s="116"/>
-      <c r="O1" s="116"/>
-      <c r="P1" s="116"/>
-      <c r="Q1" s="116"/>
-      <c r="R1" s="116"/>
-      <c r="S1" s="116"/>
-      <c r="T1" s="116"/>
-      <c r="U1" s="116"/>
-      <c r="V1" s="116"/>
-      <c r="W1" s="116"/>
-      <c r="X1" s="116"/>
-      <c r="Y1" s="116"/>
-      <c r="Z1" s="116"/>
-      <c r="AA1" s="116"/>
-      <c r="AB1" s="116"/>
-      <c r="AC1" s="116"/>
-      <c r="AD1" s="116"/>
-      <c r="AE1" s="116"/>
-      <c r="AF1" s="116"/>
-      <c r="AG1" s="116"/>
-      <c r="AH1" s="116"/>
-      <c r="AI1" s="116"/>
-      <c r="AJ1" s="116"/>
-      <c r="AK1" s="116"/>
-      <c r="AL1" s="116"/>
-      <c r="AM1" s="116"/>
-      <c r="AN1" s="116"/>
-      <c r="AO1" s="112"/>
+      <c r="B1" s="172"/>
+      <c r="C1" s="155"/>
+      <c r="D1" s="155"/>
+      <c r="E1" s="155"/>
+      <c r="F1" s="155"/>
+      <c r="G1" s="155"/>
+      <c r="H1" s="155"/>
+      <c r="I1" s="155"/>
+      <c r="J1" s="155"/>
+      <c r="K1" s="155"/>
+      <c r="L1" s="155"/>
+      <c r="M1" s="155"/>
+      <c r="N1" s="155"/>
+      <c r="O1" s="155"/>
+      <c r="P1" s="155"/>
+      <c r="Q1" s="155"/>
+      <c r="R1" s="155"/>
+      <c r="S1" s="155"/>
+      <c r="T1" s="155"/>
+      <c r="U1" s="155"/>
+      <c r="V1" s="155"/>
+      <c r="W1" s="155"/>
+      <c r="X1" s="155"/>
+      <c r="Y1" s="155"/>
+      <c r="Z1" s="155"/>
+      <c r="AA1" s="155"/>
+      <c r="AB1" s="155"/>
+      <c r="AC1" s="155"/>
+      <c r="AD1" s="155"/>
+      <c r="AE1" s="155"/>
+      <c r="AF1" s="155"/>
+      <c r="AG1" s="155"/>
+      <c r="AH1" s="155"/>
+      <c r="AI1" s="155"/>
+      <c r="AJ1" s="155"/>
+      <c r="AK1" s="155"/>
+      <c r="AL1" s="155"/>
+      <c r="AM1" s="155"/>
+      <c r="AN1" s="155"/>
+      <c r="AO1" s="151"/>
     </row>
     <row r="2" spans="1:41" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="84" t="s">
         <v>134</v>
       </c>
-      <c r="B2" s="95"/>
-      <c r="C2" s="169" t="s">
+      <c r="B2" s="173"/>
+      <c r="C2" s="110" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="170"/>
-      <c r="E2" s="170"/>
-      <c r="F2" s="170"/>
-      <c r="G2" s="170"/>
-      <c r="H2" s="170"/>
-      <c r="I2" s="170"/>
-      <c r="J2" s="170"/>
-      <c r="K2" s="170"/>
-      <c r="L2" s="117"/>
+      <c r="D2" s="111"/>
+      <c r="E2" s="111"/>
+      <c r="F2" s="111"/>
+      <c r="G2" s="111"/>
+      <c r="H2" s="111"/>
+      <c r="I2" s="111"/>
+      <c r="J2" s="111"/>
+      <c r="K2" s="111"/>
+      <c r="L2" s="159"/>
       <c r="M2" s="37"/>
       <c r="N2" s="37"/>
       <c r="O2" s="37"/>
@@ -2414,7 +2414,7 @@
       <c r="AC2" s="38"/>
       <c r="AD2" s="38"/>
       <c r="AE2" s="38"/>
-      <c r="AF2" s="166"/>
+      <c r="AF2" s="95"/>
       <c r="AG2" s="38"/>
       <c r="AH2" s="38"/>
       <c r="AI2" s="38"/>
@@ -2423,23 +2423,23 @@
       <c r="AL2" s="38"/>
       <c r="AM2" s="38"/>
       <c r="AN2" s="39"/>
-      <c r="AO2" s="113"/>
+      <c r="AO2" s="152"/>
     </row>
     <row r="3" spans="1:41" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="84" t="s">
         <v>131</v>
       </c>
-      <c r="B3" s="95"/>
-      <c r="C3" s="171"/>
-      <c r="D3" s="172"/>
-      <c r="E3" s="172"/>
-      <c r="F3" s="172"/>
-      <c r="G3" s="172"/>
-      <c r="H3" s="172"/>
-      <c r="I3" s="172"/>
-      <c r="J3" s="172"/>
-      <c r="K3" s="172"/>
-      <c r="L3" s="118"/>
+      <c r="B3" s="173"/>
+      <c r="C3" s="112"/>
+      <c r="D3" s="113"/>
+      <c r="E3" s="113"/>
+      <c r="F3" s="113"/>
+      <c r="G3" s="113"/>
+      <c r="H3" s="113"/>
+      <c r="I3" s="113"/>
+      <c r="J3" s="113"/>
+      <c r="K3" s="113"/>
+      <c r="L3" s="160"/>
       <c r="M3" s="70"/>
       <c r="N3" s="70"/>
       <c r="O3" s="70"/>
@@ -2459,7 +2459,7 @@
       <c r="AC3" s="71"/>
       <c r="AD3" s="71"/>
       <c r="AE3" s="71"/>
-      <c r="AF3" s="167"/>
+      <c r="AF3" s="96"/>
       <c r="AG3" s="71"/>
       <c r="AH3" s="71"/>
       <c r="AI3" s="71"/>
@@ -2468,23 +2468,23 @@
       <c r="AL3" s="71"/>
       <c r="AM3" s="71"/>
       <c r="AN3" s="40"/>
-      <c r="AO3" s="113"/>
+      <c r="AO3" s="152"/>
     </row>
     <row r="4" spans="1:41" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="84" t="s">
         <v>130</v>
       </c>
-      <c r="B4" s="95"/>
-      <c r="C4" s="171"/>
-      <c r="D4" s="172"/>
-      <c r="E4" s="172"/>
-      <c r="F4" s="172"/>
-      <c r="G4" s="172"/>
-      <c r="H4" s="172"/>
-      <c r="I4" s="172"/>
-      <c r="J4" s="172"/>
-      <c r="K4" s="172"/>
-      <c r="L4" s="118"/>
+      <c r="B4" s="173"/>
+      <c r="C4" s="112"/>
+      <c r="D4" s="113"/>
+      <c r="E4" s="113"/>
+      <c r="F4" s="113"/>
+      <c r="G4" s="113"/>
+      <c r="H4" s="113"/>
+      <c r="I4" s="113"/>
+      <c r="J4" s="113"/>
+      <c r="K4" s="113"/>
+      <c r="L4" s="160"/>
       <c r="M4" s="71"/>
       <c r="N4" s="71"/>
       <c r="O4" s="71"/>
@@ -2504,7 +2504,7 @@
       <c r="AC4" s="71"/>
       <c r="AD4" s="71"/>
       <c r="AE4" s="71"/>
-      <c r="AF4" s="167"/>
+      <c r="AF4" s="96"/>
       <c r="AG4" s="71"/>
       <c r="AH4" s="71"/>
       <c r="AI4" s="71"/>
@@ -2513,166 +2513,166 @@
       <c r="AL4" s="71"/>
       <c r="AM4" s="71"/>
       <c r="AN4" s="40"/>
-      <c r="AO4" s="113"/>
+      <c r="AO4" s="152"/>
     </row>
     <row r="5" spans="1:41" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="84" t="s">
         <v>132</v>
       </c>
-      <c r="B5" s="95"/>
-      <c r="C5" s="171"/>
-      <c r="D5" s="172"/>
-      <c r="E5" s="172"/>
-      <c r="F5" s="172"/>
-      <c r="G5" s="172"/>
-      <c r="H5" s="172"/>
-      <c r="I5" s="172"/>
-      <c r="J5" s="172"/>
-      <c r="K5" s="172"/>
-      <c r="L5" s="118"/>
-      <c r="M5" s="143" t="s">
+      <c r="B5" s="173"/>
+      <c r="C5" s="112"/>
+      <c r="D5" s="113"/>
+      <c r="E5" s="113"/>
+      <c r="F5" s="113"/>
+      <c r="G5" s="113"/>
+      <c r="H5" s="113"/>
+      <c r="I5" s="113"/>
+      <c r="J5" s="113"/>
+      <c r="K5" s="113"/>
+      <c r="L5" s="160"/>
+      <c r="M5" s="121" t="s">
         <v>42</v>
       </c>
-      <c r="N5" s="144"/>
-      <c r="O5" s="144"/>
-      <c r="P5" s="144"/>
-      <c r="Q5" s="144"/>
-      <c r="R5" s="144"/>
-      <c r="S5" s="144"/>
-      <c r="T5" s="144"/>
-      <c r="U5" s="144"/>
-      <c r="V5" s="144"/>
-      <c r="W5" s="144"/>
-      <c r="X5" s="144"/>
-      <c r="Y5" s="144"/>
-      <c r="Z5" s="144"/>
-      <c r="AA5" s="144"/>
-      <c r="AB5" s="144"/>
-      <c r="AC5" s="144"/>
-      <c r="AD5" s="144"/>
-      <c r="AE5" s="145"/>
-      <c r="AF5" s="167"/>
-      <c r="AG5" s="85" t="s">
+      <c r="N5" s="122"/>
+      <c r="O5" s="122"/>
+      <c r="P5" s="122"/>
+      <c r="Q5" s="122"/>
+      <c r="R5" s="122"/>
+      <c r="S5" s="122"/>
+      <c r="T5" s="122"/>
+      <c r="U5" s="122"/>
+      <c r="V5" s="122"/>
+      <c r="W5" s="122"/>
+      <c r="X5" s="122"/>
+      <c r="Y5" s="122"/>
+      <c r="Z5" s="122"/>
+      <c r="AA5" s="122"/>
+      <c r="AB5" s="122"/>
+      <c r="AC5" s="122"/>
+      <c r="AD5" s="122"/>
+      <c r="AE5" s="123"/>
+      <c r="AF5" s="96"/>
+      <c r="AG5" s="163" t="s">
         <v>140</v>
       </c>
-      <c r="AH5" s="86"/>
-      <c r="AI5" s="86"/>
-      <c r="AJ5" s="86"/>
-      <c r="AK5" s="86"/>
-      <c r="AL5" s="86"/>
-      <c r="AM5" s="86"/>
-      <c r="AN5" s="87"/>
-      <c r="AO5" s="113"/>
+      <c r="AH5" s="164"/>
+      <c r="AI5" s="164"/>
+      <c r="AJ5" s="164"/>
+      <c r="AK5" s="164"/>
+      <c r="AL5" s="164"/>
+      <c r="AM5" s="164"/>
+      <c r="AN5" s="165"/>
+      <c r="AO5" s="152"/>
     </row>
     <row r="6" spans="1:41" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="84" t="s">
         <v>162</v>
       </c>
-      <c r="B6" s="95"/>
-      <c r="C6" s="173"/>
-      <c r="D6" s="174"/>
-      <c r="E6" s="174"/>
-      <c r="F6" s="174"/>
-      <c r="G6" s="174"/>
-      <c r="H6" s="174"/>
-      <c r="I6" s="174"/>
-      <c r="J6" s="174"/>
-      <c r="K6" s="174"/>
-      <c r="L6" s="118"/>
-      <c r="M6" s="146"/>
-      <c r="N6" s="147"/>
-      <c r="O6" s="147"/>
-      <c r="P6" s="147"/>
-      <c r="Q6" s="147"/>
-      <c r="R6" s="147"/>
-      <c r="S6" s="147"/>
-      <c r="T6" s="147"/>
-      <c r="U6" s="147"/>
-      <c r="V6" s="147"/>
-      <c r="W6" s="147"/>
-      <c r="X6" s="147"/>
-      <c r="Y6" s="147"/>
-      <c r="Z6" s="147"/>
-      <c r="AA6" s="147"/>
-      <c r="AB6" s="147"/>
-      <c r="AC6" s="147"/>
-      <c r="AD6" s="147"/>
-      <c r="AE6" s="148"/>
-      <c r="AF6" s="167"/>
-      <c r="AG6" s="88"/>
-      <c r="AH6" s="89"/>
-      <c r="AI6" s="89"/>
-      <c r="AJ6" s="89"/>
-      <c r="AK6" s="89"/>
-      <c r="AL6" s="89"/>
-      <c r="AM6" s="89"/>
-      <c r="AN6" s="90"/>
-      <c r="AO6" s="113"/>
+      <c r="B6" s="173"/>
+      <c r="C6" s="114"/>
+      <c r="D6" s="115"/>
+      <c r="E6" s="115"/>
+      <c r="F6" s="115"/>
+      <c r="G6" s="115"/>
+      <c r="H6" s="115"/>
+      <c r="I6" s="115"/>
+      <c r="J6" s="115"/>
+      <c r="K6" s="115"/>
+      <c r="L6" s="160"/>
+      <c r="M6" s="124"/>
+      <c r="N6" s="125"/>
+      <c r="O6" s="125"/>
+      <c r="P6" s="125"/>
+      <c r="Q6" s="125"/>
+      <c r="R6" s="125"/>
+      <c r="S6" s="125"/>
+      <c r="T6" s="125"/>
+      <c r="U6" s="125"/>
+      <c r="V6" s="125"/>
+      <c r="W6" s="125"/>
+      <c r="X6" s="125"/>
+      <c r="Y6" s="125"/>
+      <c r="Z6" s="125"/>
+      <c r="AA6" s="125"/>
+      <c r="AB6" s="125"/>
+      <c r="AC6" s="125"/>
+      <c r="AD6" s="125"/>
+      <c r="AE6" s="126"/>
+      <c r="AF6" s="96"/>
+      <c r="AG6" s="166"/>
+      <c r="AH6" s="167"/>
+      <c r="AI6" s="167"/>
+      <c r="AJ6" s="167"/>
+      <c r="AK6" s="167"/>
+      <c r="AL6" s="167"/>
+      <c r="AM6" s="167"/>
+      <c r="AN6" s="168"/>
+      <c r="AO6" s="152"/>
     </row>
     <row r="7" spans="1:41" ht="39.950000000000003" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="84" t="s">
         <v>112</v>
       </c>
-      <c r="B7" s="95"/>
+      <c r="B7" s="173"/>
       <c r="C7" s="68"/>
-      <c r="D7" s="156" t="s">
+      <c r="D7" s="120" t="s">
         <v>141</v>
       </c>
-      <c r="E7" s="156"/>
-      <c r="F7" s="156"/>
-      <c r="G7" s="156"/>
-      <c r="H7" s="156"/>
-      <c r="I7" s="155">
+      <c r="E7" s="120"/>
+      <c r="F7" s="120"/>
+      <c r="G7" s="120"/>
+      <c r="H7" s="120"/>
+      <c r="I7" s="119">
         <v>45658</v>
       </c>
-      <c r="J7" s="155"/>
+      <c r="J7" s="119"/>
       <c r="K7" s="69"/>
-      <c r="L7" s="118"/>
-      <c r="M7" s="149"/>
-      <c r="N7" s="150"/>
-      <c r="O7" s="150"/>
-      <c r="P7" s="150"/>
-      <c r="Q7" s="150"/>
-      <c r="R7" s="150"/>
-      <c r="S7" s="150"/>
-      <c r="T7" s="150"/>
-      <c r="U7" s="150"/>
-      <c r="V7" s="150"/>
-      <c r="W7" s="150"/>
-      <c r="X7" s="150"/>
-      <c r="Y7" s="150"/>
-      <c r="Z7" s="150"/>
-      <c r="AA7" s="150"/>
-      <c r="AB7" s="150"/>
-      <c r="AC7" s="150"/>
-      <c r="AD7" s="150"/>
-      <c r="AE7" s="151"/>
-      <c r="AF7" s="167"/>
-      <c r="AG7" s="91"/>
-      <c r="AH7" s="92"/>
-      <c r="AI7" s="92"/>
-      <c r="AJ7" s="92"/>
-      <c r="AK7" s="92"/>
-      <c r="AL7" s="92"/>
-      <c r="AM7" s="92"/>
-      <c r="AN7" s="93"/>
-      <c r="AO7" s="113"/>
+      <c r="L7" s="160"/>
+      <c r="M7" s="127"/>
+      <c r="N7" s="128"/>
+      <c r="O7" s="128"/>
+      <c r="P7" s="128"/>
+      <c r="Q7" s="128"/>
+      <c r="R7" s="128"/>
+      <c r="S7" s="128"/>
+      <c r="T7" s="128"/>
+      <c r="U7" s="128"/>
+      <c r="V7" s="128"/>
+      <c r="W7" s="128"/>
+      <c r="X7" s="128"/>
+      <c r="Y7" s="128"/>
+      <c r="Z7" s="128"/>
+      <c r="AA7" s="128"/>
+      <c r="AB7" s="128"/>
+      <c r="AC7" s="128"/>
+      <c r="AD7" s="128"/>
+      <c r="AE7" s="129"/>
+      <c r="AF7" s="96"/>
+      <c r="AG7" s="169"/>
+      <c r="AH7" s="170"/>
+      <c r="AI7" s="170"/>
+      <c r="AJ7" s="170"/>
+      <c r="AK7" s="170"/>
+      <c r="AL7" s="170"/>
+      <c r="AM7" s="170"/>
+      <c r="AN7" s="171"/>
+      <c r="AO7" s="152"/>
     </row>
     <row r="8" spans="1:41" ht="5.0999999999999996" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A8" s="84" t="s">
         <v>119</v>
       </c>
-      <c r="B8" s="95"/>
-      <c r="C8" s="153"/>
-      <c r="D8" s="154"/>
-      <c r="E8" s="154"/>
-      <c r="F8" s="154"/>
-      <c r="G8" s="154"/>
-      <c r="H8" s="154"/>
-      <c r="I8" s="154"/>
-      <c r="J8" s="154"/>
-      <c r="K8" s="154"/>
-      <c r="L8" s="118"/>
+      <c r="B8" s="173"/>
+      <c r="C8" s="117"/>
+      <c r="D8" s="118"/>
+      <c r="E8" s="118"/>
+      <c r="F8" s="118"/>
+      <c r="G8" s="118"/>
+      <c r="H8" s="118"/>
+      <c r="I8" s="118"/>
+      <c r="J8" s="118"/>
+      <c r="K8" s="118"/>
+      <c r="L8" s="160"/>
       <c r="M8" s="71"/>
       <c r="N8" s="71"/>
       <c r="O8" s="71"/>
@@ -2692,7 +2692,7 @@
       <c r="AC8" s="71"/>
       <c r="AD8" s="71"/>
       <c r="AE8" s="71"/>
-      <c r="AF8" s="167"/>
+      <c r="AF8" s="96"/>
       <c r="AG8" s="71"/>
       <c r="AH8" s="71"/>
       <c r="AI8" s="71"/>
@@ -2701,23 +2701,23 @@
       <c r="AL8" s="71"/>
       <c r="AM8" s="71"/>
       <c r="AN8" s="40"/>
-      <c r="AO8" s="113"/>
+      <c r="AO8" s="152"/>
     </row>
     <row r="9" spans="1:41" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="84" t="s">
         <v>115</v>
       </c>
-      <c r="B9" s="95"/>
+      <c r="B9" s="173"/>
       <c r="C9" s="41"/>
-      <c r="D9" s="152"/>
-      <c r="E9" s="152"/>
+      <c r="D9" s="116"/>
+      <c r="E9" s="116"/>
       <c r="F9" s="72"/>
       <c r="G9" s="73"/>
-      <c r="H9" s="152"/>
-      <c r="I9" s="152"/>
-      <c r="J9" s="152"/>
+      <c r="H9" s="116"/>
+      <c r="I9" s="116"/>
+      <c r="J9" s="116"/>
       <c r="K9" s="71"/>
-      <c r="L9" s="118"/>
+      <c r="L9" s="160"/>
       <c r="M9" s="71"/>
       <c r="N9" s="71"/>
       <c r="O9" s="71"/>
@@ -2737,7 +2737,7 @@
       <c r="AC9" s="71"/>
       <c r="AD9" s="71"/>
       <c r="AE9" s="71"/>
-      <c r="AF9" s="167"/>
+      <c r="AF9" s="96"/>
       <c r="AG9" s="71"/>
       <c r="AH9" s="71"/>
       <c r="AI9" s="71"/>
@@ -2746,13 +2746,13 @@
       <c r="AL9" s="71"/>
       <c r="AM9" s="71"/>
       <c r="AN9" s="40"/>
-      <c r="AO9" s="113"/>
+      <c r="AO9" s="152"/>
     </row>
     <row r="10" spans="1:41" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="84" t="s">
         <v>114</v>
       </c>
-      <c r="B10" s="95"/>
+      <c r="B10" s="173"/>
       <c r="C10" s="41"/>
       <c r="D10" s="71"/>
       <c r="E10" s="73"/>
@@ -2762,7 +2762,7 @@
       <c r="I10" s="71"/>
       <c r="J10" s="71"/>
       <c r="K10" s="71"/>
-      <c r="L10" s="118"/>
+      <c r="L10" s="160"/>
       <c r="M10" s="71"/>
       <c r="N10" s="71"/>
       <c r="O10" s="71"/>
@@ -2782,7 +2782,7 @@
       <c r="AC10" s="71"/>
       <c r="AD10" s="71"/>
       <c r="AE10" s="71"/>
-      <c r="AF10" s="167"/>
+      <c r="AF10" s="96"/>
       <c r="AG10" s="71"/>
       <c r="AH10" s="71"/>
       <c r="AI10" s="71"/>
@@ -2791,13 +2791,13 @@
       <c r="AL10" s="71"/>
       <c r="AM10" s="71"/>
       <c r="AN10" s="40"/>
-      <c r="AO10" s="113"/>
+      <c r="AO10" s="152"/>
     </row>
     <row r="11" spans="1:41" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="84" t="s">
         <v>116</v>
       </c>
-      <c r="B11" s="95"/>
+      <c r="B11" s="173"/>
       <c r="C11" s="41"/>
       <c r="D11" s="71"/>
       <c r="E11" s="73"/>
@@ -2807,50 +2807,50 @@
       <c r="I11" s="71"/>
       <c r="J11" s="71"/>
       <c r="K11" s="71"/>
-      <c r="L11" s="118"/>
-      <c r="M11" s="121" t="s">
+      <c r="L11" s="160"/>
+      <c r="M11" s="102" t="s">
         <v>38</v>
       </c>
-      <c r="N11" s="121"/>
-      <c r="O11" s="121"/>
-      <c r="P11" s="121"/>
-      <c r="Q11" s="121"/>
-      <c r="R11" s="121"/>
-      <c r="S11" s="122"/>
+      <c r="N11" s="102"/>
+      <c r="O11" s="102"/>
+      <c r="P11" s="102"/>
+      <c r="Q11" s="102"/>
+      <c r="R11" s="102"/>
+      <c r="S11" s="103"/>
       <c r="T11" s="71"/>
-      <c r="U11" s="120" t="s">
+      <c r="U11" s="101" t="s">
         <v>45</v>
       </c>
-      <c r="V11" s="121"/>
-      <c r="W11" s="121"/>
-      <c r="X11" s="121"/>
-      <c r="Y11" s="122"/>
+      <c r="V11" s="102"/>
+      <c r="W11" s="102"/>
+      <c r="X11" s="102"/>
+      <c r="Y11" s="103"/>
       <c r="Z11" s="71"/>
-      <c r="AA11" s="120" t="s">
+      <c r="AA11" s="101" t="s">
         <v>41</v>
       </c>
-      <c r="AB11" s="121"/>
-      <c r="AC11" s="121"/>
-      <c r="AD11" s="121"/>
-      <c r="AE11" s="121"/>
-      <c r="AF11" s="167"/>
+      <c r="AB11" s="102"/>
+      <c r="AC11" s="102"/>
+      <c r="AD11" s="102"/>
+      <c r="AE11" s="102"/>
+      <c r="AF11" s="96"/>
       <c r="AG11" s="71"/>
-      <c r="AH11" s="120" t="s">
+      <c r="AH11" s="101" t="s">
         <v>54</v>
       </c>
-      <c r="AI11" s="121"/>
-      <c r="AJ11" s="121"/>
-      <c r="AK11" s="121"/>
-      <c r="AL11" s="121"/>
-      <c r="AM11" s="122"/>
+      <c r="AI11" s="102"/>
+      <c r="AJ11" s="102"/>
+      <c r="AK11" s="102"/>
+      <c r="AL11" s="102"/>
+      <c r="AM11" s="103"/>
       <c r="AN11" s="40"/>
-      <c r="AO11" s="113"/>
+      <c r="AO11" s="152"/>
     </row>
     <row r="12" spans="1:41" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="84" t="s">
         <v>118</v>
       </c>
-      <c r="B12" s="95"/>
+      <c r="B12" s="173"/>
       <c r="C12" s="41"/>
       <c r="D12" s="71"/>
       <c r="E12" s="73"/>
@@ -2860,101 +2860,101 @@
       <c r="I12" s="71"/>
       <c r="J12" s="71"/>
       <c r="K12" s="71"/>
-      <c r="L12" s="118"/>
-      <c r="M12" s="124"/>
-      <c r="N12" s="124"/>
-      <c r="O12" s="124"/>
-      <c r="P12" s="124"/>
-      <c r="Q12" s="124"/>
-      <c r="R12" s="124"/>
-      <c r="S12" s="125"/>
+      <c r="L12" s="160"/>
+      <c r="M12" s="105"/>
+      <c r="N12" s="105"/>
+      <c r="O12" s="105"/>
+      <c r="P12" s="105"/>
+      <c r="Q12" s="105"/>
+      <c r="R12" s="105"/>
+      <c r="S12" s="106"/>
       <c r="T12" s="71"/>
-      <c r="U12" s="123"/>
-      <c r="V12" s="124"/>
-      <c r="W12" s="124"/>
-      <c r="X12" s="124"/>
-      <c r="Y12" s="125"/>
+      <c r="U12" s="104"/>
+      <c r="V12" s="105"/>
+      <c r="W12" s="105"/>
+      <c r="X12" s="105"/>
+      <c r="Y12" s="106"/>
       <c r="Z12" s="71"/>
-      <c r="AA12" s="123"/>
-      <c r="AB12" s="124"/>
-      <c r="AC12" s="124"/>
-      <c r="AD12" s="124"/>
-      <c r="AE12" s="124"/>
-      <c r="AF12" s="167"/>
+      <c r="AA12" s="104"/>
+      <c r="AB12" s="105"/>
+      <c r="AC12" s="105"/>
+      <c r="AD12" s="105"/>
+      <c r="AE12" s="105"/>
+      <c r="AF12" s="96"/>
       <c r="AG12" s="71"/>
-      <c r="AH12" s="123"/>
-      <c r="AI12" s="124"/>
-      <c r="AJ12" s="124"/>
-      <c r="AK12" s="124"/>
-      <c r="AL12" s="124"/>
-      <c r="AM12" s="125"/>
+      <c r="AH12" s="104"/>
+      <c r="AI12" s="105"/>
+      <c r="AJ12" s="105"/>
+      <c r="AK12" s="105"/>
+      <c r="AL12" s="105"/>
+      <c r="AM12" s="106"/>
       <c r="AN12" s="40"/>
-      <c r="AO12" s="113"/>
+      <c r="AO12" s="152"/>
     </row>
     <row r="13" spans="1:41" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="84" t="s">
         <v>120</v>
       </c>
-      <c r="B13" s="95"/>
+      <c r="B13" s="173"/>
       <c r="C13" s="41"/>
-      <c r="D13" s="157" t="s">
+      <c r="D13" s="85" t="s">
         <v>2</v>
       </c>
-      <c r="E13" s="159"/>
+      <c r="E13" s="87"/>
       <c r="F13" s="72"/>
       <c r="G13" s="73"/>
-      <c r="H13" s="157" t="s">
+      <c r="H13" s="85" t="s">
         <v>139</v>
       </c>
-      <c r="I13" s="158"/>
-      <c r="J13" s="159"/>
+      <c r="I13" s="86"/>
+      <c r="J13" s="87"/>
       <c r="K13" s="71"/>
-      <c r="L13" s="118"/>
-      <c r="M13" s="127"/>
-      <c r="N13" s="127"/>
-      <c r="O13" s="127"/>
-      <c r="P13" s="127"/>
-      <c r="Q13" s="127"/>
-      <c r="R13" s="127"/>
-      <c r="S13" s="128"/>
+      <c r="L13" s="160"/>
+      <c r="M13" s="108"/>
+      <c r="N13" s="108"/>
+      <c r="O13" s="108"/>
+      <c r="P13" s="108"/>
+      <c r="Q13" s="108"/>
+      <c r="R13" s="108"/>
+      <c r="S13" s="109"/>
       <c r="T13" s="71"/>
-      <c r="U13" s="126"/>
-      <c r="V13" s="127"/>
-      <c r="W13" s="127"/>
-      <c r="X13" s="127"/>
-      <c r="Y13" s="128"/>
+      <c r="U13" s="107"/>
+      <c r="V13" s="108"/>
+      <c r="W13" s="108"/>
+      <c r="X13" s="108"/>
+      <c r="Y13" s="109"/>
       <c r="Z13" s="71"/>
-      <c r="AA13" s="126"/>
-      <c r="AB13" s="127"/>
-      <c r="AC13" s="127"/>
-      <c r="AD13" s="127"/>
-      <c r="AE13" s="127"/>
-      <c r="AF13" s="167"/>
+      <c r="AA13" s="107"/>
+      <c r="AB13" s="108"/>
+      <c r="AC13" s="108"/>
+      <c r="AD13" s="108"/>
+      <c r="AE13" s="108"/>
+      <c r="AF13" s="96"/>
       <c r="AG13" s="71"/>
-      <c r="AH13" s="126"/>
-      <c r="AI13" s="127"/>
-      <c r="AJ13" s="127"/>
-      <c r="AK13" s="127"/>
-      <c r="AL13" s="127"/>
-      <c r="AM13" s="128"/>
+      <c r="AH13" s="107"/>
+      <c r="AI13" s="108"/>
+      <c r="AJ13" s="108"/>
+      <c r="AK13" s="108"/>
+      <c r="AL13" s="108"/>
+      <c r="AM13" s="109"/>
       <c r="AN13" s="40"/>
-      <c r="AO13" s="113"/>
+      <c r="AO13" s="152"/>
     </row>
     <row r="14" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="84" t="s">
         <v>113</v>
       </c>
-      <c r="B14" s="95"/>
+      <c r="B14" s="173"/>
       <c r="C14" s="41"/>
-      <c r="D14" s="160"/>
-      <c r="E14" s="163"/>
+      <c r="D14" s="88"/>
+      <c r="E14" s="90"/>
       <c r="F14" s="72"/>
       <c r="G14" s="73"/>
-      <c r="H14" s="160"/>
-      <c r="I14" s="161"/>
-      <c r="J14" s="162"/>
+      <c r="H14" s="88"/>
+      <c r="I14" s="89"/>
+      <c r="J14" s="90"/>
       <c r="K14" s="71"/>
-      <c r="L14" s="118"/>
+      <c r="L14" s="160"/>
       <c r="M14" s="74"/>
       <c r="N14" s="74"/>
       <c r="O14" s="74"/>
@@ -2963,33 +2963,33 @@
       <c r="R14" s="74"/>
       <c r="S14" s="3"/>
       <c r="T14" s="71"/>
-      <c r="U14" s="104"/>
-      <c r="V14" s="105"/>
-      <c r="W14" s="105"/>
-      <c r="X14" s="105"/>
-      <c r="Y14" s="107"/>
+      <c r="U14" s="132"/>
+      <c r="V14" s="130"/>
+      <c r="W14" s="130"/>
+      <c r="X14" s="130"/>
+      <c r="Y14" s="131"/>
       <c r="Z14" s="71"/>
-      <c r="AA14" s="104"/>
-      <c r="AB14" s="105"/>
-      <c r="AC14" s="105"/>
-      <c r="AD14" s="105"/>
-      <c r="AE14" s="105"/>
-      <c r="AF14" s="167"/>
+      <c r="AA14" s="132"/>
+      <c r="AB14" s="130"/>
+      <c r="AC14" s="130"/>
+      <c r="AD14" s="130"/>
+      <c r="AE14" s="130"/>
+      <c r="AF14" s="96"/>
       <c r="AG14" s="71"/>
-      <c r="AH14" s="104"/>
-      <c r="AI14" s="105"/>
-      <c r="AJ14" s="105"/>
-      <c r="AK14" s="105"/>
-      <c r="AL14" s="105"/>
-      <c r="AM14" s="107"/>
+      <c r="AH14" s="132"/>
+      <c r="AI14" s="130"/>
+      <c r="AJ14" s="130"/>
+      <c r="AK14" s="130"/>
+      <c r="AL14" s="130"/>
+      <c r="AM14" s="131"/>
       <c r="AN14" s="40"/>
-      <c r="AO14" s="113"/>
+      <c r="AO14" s="152"/>
     </row>
     <row r="15" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="84" t="s">
         <v>117</v>
       </c>
-      <c r="B15" s="95"/>
+      <c r="B15" s="173"/>
       <c r="C15" s="41"/>
       <c r="D15" s="65" t="s">
         <v>3</v>
@@ -3010,58 +3010,58 @@
         <v>19</v>
       </c>
       <c r="K15" s="71"/>
-      <c r="L15" s="118"/>
-      <c r="M15" s="111"/>
+      <c r="L15" s="160"/>
+      <c r="M15" s="148"/>
       <c r="N15" s="75"/>
       <c r="O15" s="75"/>
       <c r="P15" s="5">
         <v>4</v>
       </c>
-      <c r="Q15" s="138" t="s">
+      <c r="Q15" s="93" t="s">
         <v>31</v>
       </c>
-      <c r="R15" s="139"/>
-      <c r="S15" s="96"/>
+      <c r="R15" s="94"/>
+      <c r="S15" s="145"/>
       <c r="T15" s="71"/>
-      <c r="U15" s="96"/>
+      <c r="U15" s="145"/>
       <c r="V15" s="5">
         <v>4</v>
       </c>
-      <c r="W15" s="138" t="s">
+      <c r="W15" s="93" t="s">
         <v>31</v>
       </c>
-      <c r="X15" s="139"/>
-      <c r="Y15" s="96"/>
+      <c r="X15" s="94"/>
+      <c r="Y15" s="145"/>
       <c r="Z15" s="71"/>
-      <c r="AA15" s="96"/>
+      <c r="AA15" s="145"/>
       <c r="AB15" s="5">
         <v>6</v>
       </c>
-      <c r="AC15" s="138" t="s">
+      <c r="AC15" s="93" t="s">
         <v>31</v>
       </c>
-      <c r="AD15" s="139"/>
-      <c r="AE15" s="108"/>
-      <c r="AF15" s="167"/>
+      <c r="AD15" s="94"/>
+      <c r="AE15" s="156"/>
+      <c r="AF15" s="96"/>
       <c r="AG15" s="71"/>
-      <c r="AH15" s="96"/>
+      <c r="AH15" s="145"/>
       <c r="AI15" s="5">
         <v>8</v>
       </c>
-      <c r="AJ15" s="164" t="s">
+      <c r="AJ15" s="91" t="s">
         <v>31</v>
       </c>
-      <c r="AK15" s="164"/>
-      <c r="AL15" s="165"/>
-      <c r="AM15" s="96"/>
+      <c r="AK15" s="91"/>
+      <c r="AL15" s="92"/>
+      <c r="AM15" s="145"/>
       <c r="AN15" s="40"/>
-      <c r="AO15" s="113"/>
+      <c r="AO15" s="152"/>
     </row>
     <row r="16" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="84" t="s">
         <v>163</v>
       </c>
-      <c r="B16" s="95"/>
+      <c r="B16" s="173"/>
       <c r="C16" s="41"/>
       <c r="D16" s="66" t="s">
         <v>4</v>
@@ -3082,8 +3082,8 @@
         <v>20</v>
       </c>
       <c r="K16" s="71"/>
-      <c r="L16" s="118"/>
-      <c r="M16" s="99"/>
+      <c r="L16" s="160"/>
+      <c r="M16" s="149"/>
       <c r="N16" s="75"/>
       <c r="O16" s="75">
         <f>ROW()</f>
@@ -3098,9 +3098,9 @@
       <c r="R16" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="S16" s="97"/>
+      <c r="S16" s="146"/>
       <c r="T16" s="71"/>
-      <c r="U16" s="97"/>
+      <c r="U16" s="146"/>
       <c r="V16" s="4" t="s">
         <v>32</v>
       </c>
@@ -3110,9 +3110,9 @@
       <c r="X16" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="Y16" s="97"/>
+      <c r="Y16" s="146"/>
       <c r="Z16" s="71"/>
-      <c r="AA16" s="97"/>
+      <c r="AA16" s="146"/>
       <c r="AB16" s="4" t="s">
         <v>32</v>
       </c>
@@ -3122,10 +3122,10 @@
       <c r="AD16" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="AE16" s="109"/>
-      <c r="AF16" s="167"/>
+      <c r="AE16" s="157"/>
+      <c r="AF16" s="96"/>
       <c r="AG16" s="71"/>
-      <c r="AH16" s="97"/>
+      <c r="AH16" s="146"/>
       <c r="AI16" s="4" t="s">
         <v>32</v>
       </c>
@@ -3138,15 +3138,15 @@
       <c r="AL16" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="AM16" s="97"/>
+      <c r="AM16" s="146"/>
       <c r="AN16" s="40"/>
-      <c r="AO16" s="113"/>
+      <c r="AO16" s="152"/>
     </row>
     <row r="17" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="84" t="s">
         <v>91</v>
       </c>
-      <c r="B17" s="95"/>
+      <c r="B17" s="173"/>
       <c r="C17" s="41"/>
       <c r="D17" s="66" t="s">
         <v>5</v>
@@ -3167,8 +3167,8 @@
         <v>21</v>
       </c>
       <c r="K17" s="71"/>
-      <c r="L17" s="118"/>
-      <c r="M17" s="99"/>
+      <c r="L17" s="160"/>
+      <c r="M17" s="149"/>
       <c r="N17" s="75" t="str">
         <f t="shared" ref="N17:N32" si="1">IF(E15=2,D15 &amp; "  [DQ]",D15)</f>
         <v>Participant #01</v>
@@ -3177,7 +3177,7 @@
         <f t="shared" ref="O17:O32" si="2">IF(E15&gt;=1,ROW()-$O$16,"")</f>
         <v/>
       </c>
-      <c r="P17" s="101" t="s">
+      <c r="P17" s="174" t="s">
         <v>34</v>
       </c>
       <c r="Q17" s="11" t="str" cm="1">
@@ -3185,10 +3185,10 @@
         <v>-</v>
       </c>
       <c r="R17" s="9"/>
-      <c r="S17" s="97"/>
+      <c r="S17" s="146"/>
       <c r="T17" s="71"/>
-      <c r="U17" s="97"/>
-      <c r="V17" s="101" t="s">
+      <c r="U17" s="146"/>
+      <c r="V17" s="98" t="s">
         <v>39</v>
       </c>
       <c r="W17" s="11" t="str">
@@ -3196,10 +3196,10 @@
         <v>A1</v>
       </c>
       <c r="X17" s="6"/>
-      <c r="Y17" s="97"/>
+      <c r="Y17" s="146"/>
       <c r="Z17" s="71"/>
-      <c r="AA17" s="97"/>
-      <c r="AB17" s="101" t="s">
+      <c r="AA17" s="146"/>
+      <c r="AB17" s="98" t="s">
         <v>52</v>
       </c>
       <c r="AC17" s="11" t="str">
@@ -3207,11 +3207,11 @@
         <v>E1</v>
       </c>
       <c r="AD17" s="6"/>
-      <c r="AE17" s="109"/>
-      <c r="AF17" s="167"/>
+      <c r="AE17" s="157"/>
+      <c r="AF17" s="96"/>
       <c r="AG17" s="71"/>
-      <c r="AH17" s="97"/>
-      <c r="AI17" s="101" t="s">
+      <c r="AH17" s="146"/>
+      <c r="AI17" s="98" t="s">
         <v>55</v>
       </c>
       <c r="AJ17" s="21" t="str">
@@ -3222,15 +3222,15 @@
       <c r="AL17" s="47">
         <v>0</v>
       </c>
-      <c r="AM17" s="99"/>
+      <c r="AM17" s="149"/>
       <c r="AN17" s="40"/>
-      <c r="AO17" s="113"/>
+      <c r="AO17" s="152"/>
     </row>
     <row r="18" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="84" t="s">
         <v>164</v>
       </c>
-      <c r="B18" s="95"/>
+      <c r="B18" s="173"/>
       <c r="C18" s="42"/>
       <c r="D18" s="66" t="s">
         <v>6</v>
@@ -3251,8 +3251,8 @@
         <v>22</v>
       </c>
       <c r="K18" s="71"/>
-      <c r="L18" s="118"/>
-      <c r="M18" s="99"/>
+      <c r="L18" s="160"/>
+      <c r="M18" s="149"/>
       <c r="N18" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #02</v>
@@ -3261,35 +3261,35 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P18" s="102"/>
+      <c r="P18" s="174"/>
       <c r="Q18" s="12" t="str" cm="1">
         <f t="array" ref="Q18">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B5))),"-")</f>
         <v>-</v>
       </c>
       <c r="R18" s="10"/>
-      <c r="S18" s="97"/>
+      <c r="S18" s="146"/>
       <c r="T18" s="71"/>
-      <c r="U18" s="97"/>
-      <c r="V18" s="102"/>
+      <c r="U18" s="146"/>
+      <c r="V18" s="99"/>
       <c r="W18" s="12" t="str">
         <f>IF(ISBLANK($R$25),"C1",$R$25)</f>
         <v>C1</v>
       </c>
       <c r="X18" s="14"/>
-      <c r="Y18" s="97"/>
+      <c r="Y18" s="146"/>
       <c r="Z18" s="71"/>
-      <c r="AA18" s="97"/>
-      <c r="AB18" s="102"/>
+      <c r="AA18" s="146"/>
+      <c r="AB18" s="99"/>
       <c r="AC18" s="12" t="str">
         <f>IF(ISBLANK($X$21),"F1",$X$21)</f>
         <v>F1</v>
       </c>
       <c r="AD18" s="14"/>
-      <c r="AE18" s="109"/>
-      <c r="AF18" s="167"/>
+      <c r="AE18" s="157"/>
+      <c r="AF18" s="96"/>
       <c r="AG18" s="71"/>
-      <c r="AH18" s="97"/>
-      <c r="AI18" s="102"/>
+      <c r="AH18" s="146"/>
+      <c r="AI18" s="99"/>
       <c r="AJ18" s="22" t="str">
         <f>IF(ISBLANK($AD$18),"WF2",$AD$18)</f>
         <v>WF2</v>
@@ -3298,15 +3298,15 @@
       <c r="AL18" s="48">
         <v>0</v>
       </c>
-      <c r="AM18" s="99"/>
+      <c r="AM18" s="149"/>
       <c r="AN18" s="40"/>
-      <c r="AO18" s="113"/>
+      <c r="AO18" s="152"/>
     </row>
     <row r="19" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="84" t="s">
         <v>93</v>
       </c>
-      <c r="B19" s="95"/>
+      <c r="B19" s="173"/>
       <c r="C19" s="42"/>
       <c r="D19" s="66" t="s">
         <v>7</v>
@@ -3327,8 +3327,8 @@
         <v>23</v>
       </c>
       <c r="K19" s="71"/>
-      <c r="L19" s="118"/>
-      <c r="M19" s="99"/>
+      <c r="L19" s="160"/>
+      <c r="M19" s="149"/>
       <c r="N19" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #03</v>
@@ -3337,35 +3337,37 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P19" s="102"/>
+      <c r="P19" s="174" t="s">
+        <v>35</v>
+      </c>
       <c r="Q19" s="12" t="str" cm="1">
         <f t="array" ref="Q19">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B9))),"-")</f>
         <v>-</v>
       </c>
       <c r="R19" s="7"/>
-      <c r="S19" s="97"/>
+      <c r="S19" s="146"/>
       <c r="T19" s="71"/>
-      <c r="U19" s="97"/>
-      <c r="V19" s="102"/>
+      <c r="U19" s="146"/>
+      <c r="V19" s="99"/>
       <c r="W19" s="12" t="str">
         <f>IF(ISBLANK($R$22),"B2",$R$22)</f>
         <v>B2</v>
       </c>
       <c r="X19" s="7"/>
-      <c r="Y19" s="97"/>
+      <c r="Y19" s="146"/>
       <c r="Z19" s="71"/>
-      <c r="AA19" s="97"/>
-      <c r="AB19" s="102"/>
+      <c r="AA19" s="146"/>
+      <c r="AB19" s="99"/>
       <c r="AC19" s="12" t="str">
         <f>IF(ISBLANK($X$18),"E2",$X$18)</f>
         <v>E2</v>
       </c>
       <c r="AD19" s="7"/>
-      <c r="AE19" s="109"/>
-      <c r="AF19" s="167"/>
+      <c r="AE19" s="157"/>
+      <c r="AF19" s="96"/>
       <c r="AG19" s="71"/>
-      <c r="AH19" s="97"/>
-      <c r="AI19" s="102"/>
+      <c r="AH19" s="146"/>
+      <c r="AI19" s="99"/>
       <c r="AJ19" s="22" t="str">
         <f>IF(ISBLANK($AD$47),"K1",$AD$47)</f>
         <v>K1</v>
@@ -3374,15 +3376,15 @@
       <c r="AL19" s="49">
         <v>0</v>
       </c>
-      <c r="AM19" s="99"/>
+      <c r="AM19" s="149"/>
       <c r="AN19" s="40"/>
-      <c r="AO19" s="113"/>
+      <c r="AO19" s="152"/>
     </row>
     <row r="20" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="84" t="s">
         <v>142</v>
       </c>
-      <c r="B20" s="95"/>
+      <c r="B20" s="173"/>
       <c r="C20" s="42"/>
       <c r="D20" s="66" t="s">
         <v>8</v>
@@ -3403,8 +3405,8 @@
         <v>24</v>
       </c>
       <c r="K20" s="71"/>
-      <c r="L20" s="118"/>
-      <c r="M20" s="99"/>
+      <c r="L20" s="160"/>
+      <c r="M20" s="149"/>
       <c r="N20" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #04</v>
@@ -3413,35 +3415,35 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P20" s="103"/>
+      <c r="P20" s="174"/>
       <c r="Q20" s="13" t="str" cm="1">
         <f t="array" ref="Q20">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B13))),"-")</f>
         <v>-</v>
       </c>
       <c r="R20" s="8"/>
-      <c r="S20" s="97"/>
+      <c r="S20" s="146"/>
       <c r="T20" s="71"/>
-      <c r="U20" s="97"/>
-      <c r="V20" s="103"/>
+      <c r="U20" s="146"/>
+      <c r="V20" s="100"/>
       <c r="W20" s="13" t="str">
         <f>IF(ISBLANK($R$30),"D2",$R$30)</f>
         <v>D2</v>
       </c>
       <c r="X20" s="8"/>
-      <c r="Y20" s="97"/>
+      <c r="Y20" s="146"/>
       <c r="Z20" s="71"/>
-      <c r="AA20" s="98"/>
-      <c r="AB20" s="103"/>
+      <c r="AA20" s="147"/>
+      <c r="AB20" s="100"/>
       <c r="AC20" s="13" t="str">
         <f>IF(ISBLANK($X$22),"F2",$X$22)</f>
         <v>F2</v>
       </c>
       <c r="AD20" s="8"/>
-      <c r="AE20" s="110"/>
-      <c r="AF20" s="167"/>
+      <c r="AE20" s="158"/>
+      <c r="AF20" s="96"/>
       <c r="AG20" s="71"/>
-      <c r="AH20" s="98"/>
-      <c r="AI20" s="103"/>
+      <c r="AH20" s="147"/>
+      <c r="AI20" s="100"/>
       <c r="AJ20" s="23" t="str">
         <f>IF(ISBLANK($AD$50),"L1",$AD$50)</f>
         <v>L1</v>
@@ -3450,15 +3452,15 @@
       <c r="AL20" s="14">
         <v>0</v>
       </c>
-      <c r="AM20" s="100"/>
+      <c r="AM20" s="150"/>
       <c r="AN20" s="40"/>
-      <c r="AO20" s="113"/>
+      <c r="AO20" s="152"/>
     </row>
     <row r="21" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="84" t="s">
         <v>143</v>
       </c>
-      <c r="B21" s="95"/>
+      <c r="B21" s="173"/>
       <c r="C21" s="42"/>
       <c r="D21" s="66" t="s">
         <v>9</v>
@@ -3479,8 +3481,8 @@
         <v>25</v>
       </c>
       <c r="K21" s="71"/>
-      <c r="L21" s="118"/>
-      <c r="M21" s="99"/>
+      <c r="L21" s="160"/>
+      <c r="M21" s="149"/>
       <c r="N21" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #05</v>
@@ -3489,18 +3491,18 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P21" s="101" t="s">
-        <v>35</v>
+      <c r="P21" s="174" t="s">
+        <v>36</v>
       </c>
       <c r="Q21" s="11" t="str" cm="1">
         <f t="array" ref="Q21">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B2))),"-")</f>
         <v>-</v>
       </c>
       <c r="R21" s="9"/>
-      <c r="S21" s="97"/>
+      <c r="S21" s="146"/>
       <c r="T21" s="71"/>
-      <c r="U21" s="97"/>
-      <c r="V21" s="101" t="s">
+      <c r="U21" s="146"/>
+      <c r="V21" s="98" t="s">
         <v>40</v>
       </c>
       <c r="W21" s="12" t="str">
@@ -3508,29 +3510,29 @@
         <v>B1</v>
       </c>
       <c r="X21" s="6"/>
-      <c r="Y21" s="97"/>
+      <c r="Y21" s="146"/>
       <c r="Z21" s="71"/>
-      <c r="AA21" s="104"/>
-      <c r="AB21" s="105"/>
-      <c r="AC21" s="105"/>
-      <c r="AD21" s="105"/>
-      <c r="AE21" s="105"/>
-      <c r="AF21" s="167"/>
+      <c r="AA21" s="132"/>
+      <c r="AB21" s="130"/>
+      <c r="AC21" s="130"/>
+      <c r="AD21" s="130"/>
+      <c r="AE21" s="130"/>
+      <c r="AF21" s="96"/>
       <c r="AG21" s="71"/>
-      <c r="AH21" s="104"/>
-      <c r="AI21" s="105"/>
-      <c r="AJ21" s="106"/>
-      <c r="AK21" s="106"/>
-      <c r="AL21" s="106"/>
-      <c r="AM21" s="107"/>
+      <c r="AH21" s="132"/>
+      <c r="AI21" s="130"/>
+      <c r="AJ21" s="162"/>
+      <c r="AK21" s="162"/>
+      <c r="AL21" s="162"/>
+      <c r="AM21" s="131"/>
       <c r="AN21" s="40"/>
-      <c r="AO21" s="113"/>
+      <c r="AO21" s="152"/>
     </row>
     <row r="22" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="84" t="s">
         <v>144</v>
       </c>
-      <c r="B22" s="95"/>
+      <c r="B22" s="173"/>
       <c r="C22" s="42"/>
       <c r="D22" s="66" t="s">
         <v>10</v>
@@ -3551,8 +3553,8 @@
         <v>26</v>
       </c>
       <c r="K22" s="71"/>
-      <c r="L22" s="118"/>
-      <c r="M22" s="99"/>
+      <c r="L22" s="160"/>
+      <c r="M22" s="149"/>
       <c r="N22" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #06</v>
@@ -3561,29 +3563,29 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P22" s="102"/>
+      <c r="P22" s="174"/>
       <c r="Q22" s="12" t="str" cm="1">
         <f t="array" ref="Q22">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B6))),"-")</f>
         <v>-</v>
       </c>
       <c r="R22" s="10"/>
-      <c r="S22" s="97"/>
+      <c r="S22" s="146"/>
       <c r="T22" s="71"/>
-      <c r="U22" s="97"/>
-      <c r="V22" s="102"/>
+      <c r="U22" s="146"/>
+      <c r="V22" s="99"/>
       <c r="W22" s="12" t="str">
         <f>IF(ISBLANK($R$29),"D1",$R$29)</f>
         <v>D1</v>
       </c>
       <c r="X22" s="14"/>
-      <c r="Y22" s="97"/>
+      <c r="Y22" s="146"/>
       <c r="Z22" s="71"/>
       <c r="AA22" s="71"/>
       <c r="AB22" s="76"/>
       <c r="AC22" s="77"/>
       <c r="AD22" s="78"/>
       <c r="AE22" s="71"/>
-      <c r="AF22" s="167"/>
+      <c r="AF22" s="96"/>
       <c r="AG22" s="71"/>
       <c r="AH22" s="71"/>
       <c r="AI22" s="71"/>
@@ -3592,13 +3594,13 @@
       <c r="AL22" s="71"/>
       <c r="AM22" s="71"/>
       <c r="AN22" s="40"/>
-      <c r="AO22" s="113"/>
+      <c r="AO22" s="152"/>
     </row>
     <row r="23" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="84" t="s">
         <v>165</v>
       </c>
-      <c r="B23" s="95"/>
+      <c r="B23" s="173"/>
       <c r="C23" s="42"/>
       <c r="D23" s="66" t="s">
         <v>11</v>
@@ -3619,8 +3621,8 @@
         <v>27</v>
       </c>
       <c r="K23" s="71"/>
-      <c r="L23" s="118"/>
-      <c r="M23" s="99"/>
+      <c r="L23" s="160"/>
+      <c r="M23" s="149"/>
       <c r="N23" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #07</v>
@@ -3629,29 +3631,31 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P23" s="102"/>
+      <c r="P23" s="174" t="s">
+        <v>37</v>
+      </c>
       <c r="Q23" s="12" t="str" cm="1">
         <f t="array" ref="Q23">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B10))),"-")</f>
         <v>-</v>
       </c>
       <c r="R23" s="7"/>
-      <c r="S23" s="97"/>
+      <c r="S23" s="146"/>
       <c r="T23" s="71"/>
-      <c r="U23" s="97"/>
-      <c r="V23" s="102"/>
+      <c r="U23" s="146"/>
+      <c r="V23" s="99"/>
       <c r="W23" s="12" t="str">
         <f>IF(ISBLANK($R$18),"A2",$R$18)</f>
         <v>A2</v>
       </c>
       <c r="X23" s="7"/>
-      <c r="Y23" s="97"/>
+      <c r="Y23" s="146"/>
       <c r="Z23" s="71"/>
       <c r="AA23" s="71"/>
       <c r="AB23" s="76"/>
       <c r="AC23" s="77"/>
       <c r="AD23" s="78"/>
       <c r="AE23" s="71"/>
-      <c r="AF23" s="167"/>
+      <c r="AF23" s="96"/>
       <c r="AG23" s="71"/>
       <c r="AH23" s="71"/>
       <c r="AI23" s="71"/>
@@ -3660,13 +3664,13 @@
       <c r="AL23" s="71"/>
       <c r="AM23" s="71"/>
       <c r="AN23" s="40"/>
-      <c r="AO23" s="113"/>
+      <c r="AO23" s="152"/>
     </row>
     <row r="24" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="84" t="s">
         <v>145</v>
       </c>
-      <c r="B24" s="95"/>
+      <c r="B24" s="173"/>
       <c r="C24" s="42"/>
       <c r="D24" s="66" t="s">
         <v>12</v>
@@ -3687,8 +3691,8 @@
         <v>27</v>
       </c>
       <c r="K24" s="71"/>
-      <c r="L24" s="118"/>
-      <c r="M24" s="99"/>
+      <c r="L24" s="160"/>
+      <c r="M24" s="149"/>
       <c r="N24" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #08</v>
@@ -3697,29 +3701,29 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P24" s="103"/>
+      <c r="P24" s="174"/>
       <c r="Q24" s="13" t="str" cm="1">
         <f t="array" ref="Q24">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B14))),"-")</f>
         <v>-</v>
       </c>
       <c r="R24" s="8"/>
-      <c r="S24" s="97"/>
+      <c r="S24" s="146"/>
       <c r="T24" s="71"/>
-      <c r="U24" s="98"/>
-      <c r="V24" s="103"/>
+      <c r="U24" s="147"/>
+      <c r="V24" s="100"/>
       <c r="W24" s="13" t="str">
         <f>IF(ISBLANK($R$26),"C2",$R$26)</f>
         <v>C2</v>
       </c>
       <c r="X24" s="8"/>
-      <c r="Y24" s="98"/>
+      <c r="Y24" s="147"/>
       <c r="Z24" s="71"/>
       <c r="AA24" s="71"/>
       <c r="AB24" s="76"/>
       <c r="AC24" s="77"/>
       <c r="AD24" s="78"/>
       <c r="AE24" s="71"/>
-      <c r="AF24" s="167"/>
+      <c r="AF24" s="96"/>
       <c r="AG24" s="71"/>
       <c r="AH24" s="71"/>
       <c r="AI24" s="71"/>
@@ -3728,13 +3732,13 @@
       <c r="AL24" s="71"/>
       <c r="AM24" s="71"/>
       <c r="AN24" s="40"/>
-      <c r="AO24" s="113"/>
+      <c r="AO24" s="152"/>
     </row>
     <row r="25" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="84" t="s">
         <v>63</v>
       </c>
-      <c r="B25" s="95"/>
+      <c r="B25" s="173"/>
       <c r="C25" s="42"/>
       <c r="D25" s="66" t="s">
         <v>13</v>
@@ -3755,8 +3759,8 @@
         <v>28</v>
       </c>
       <c r="K25" s="71"/>
-      <c r="L25" s="118"/>
-      <c r="M25" s="99"/>
+      <c r="L25" s="160"/>
+      <c r="M25" s="149"/>
       <c r="N25" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #09</v>
@@ -3765,45 +3769,45 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P25" s="101" t="s">
-        <v>36</v>
+      <c r="P25" s="174" t="s">
+        <v>39</v>
       </c>
       <c r="Q25" s="11" t="str" cm="1">
         <f t="array" ref="Q25">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B3))),"-")</f>
         <v>-</v>
       </c>
       <c r="R25" s="9"/>
-      <c r="S25" s="97"/>
+      <c r="S25" s="146"/>
       <c r="T25" s="71"/>
-      <c r="U25" s="104"/>
-      <c r="V25" s="105"/>
-      <c r="W25" s="105"/>
-      <c r="X25" s="105"/>
-      <c r="Y25" s="107"/>
+      <c r="U25" s="132"/>
+      <c r="V25" s="130"/>
+      <c r="W25" s="130"/>
+      <c r="X25" s="130"/>
+      <c r="Y25" s="131"/>
       <c r="Z25" s="71"/>
       <c r="AA25" s="71"/>
       <c r="AB25" s="71"/>
       <c r="AC25" s="71"/>
       <c r="AD25" s="71"/>
       <c r="AE25" s="71"/>
-      <c r="AF25" s="167"/>
+      <c r="AF25" s="96"/>
       <c r="AG25" s="71"/>
-      <c r="AH25" s="120" t="s">
+      <c r="AH25" s="101" t="s">
         <v>53</v>
       </c>
-      <c r="AI25" s="121"/>
-      <c r="AJ25" s="121"/>
-      <c r="AK25" s="121"/>
-      <c r="AL25" s="121"/>
-      <c r="AM25" s="122"/>
+      <c r="AI25" s="102"/>
+      <c r="AJ25" s="102"/>
+      <c r="AK25" s="102"/>
+      <c r="AL25" s="102"/>
+      <c r="AM25" s="103"/>
       <c r="AN25" s="40"/>
-      <c r="AO25" s="113"/>
+      <c r="AO25" s="152"/>
     </row>
     <row r="26" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="84" t="s">
         <v>146</v>
       </c>
-      <c r="B26" s="95"/>
+      <c r="B26" s="173"/>
       <c r="C26" s="42"/>
       <c r="D26" s="66" t="s">
         <v>14</v>
@@ -3824,8 +3828,8 @@
         <v>28</v>
       </c>
       <c r="K26" s="71"/>
-      <c r="L26" s="118"/>
-      <c r="M26" s="99"/>
+      <c r="L26" s="160"/>
+      <c r="M26" s="149"/>
       <c r="N26" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #10</v>
@@ -3834,13 +3838,13 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P26" s="102"/>
+      <c r="P26" s="174"/>
       <c r="Q26" s="12" t="str" cm="1">
         <f t="array" ref="Q26">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B7))),"-")</f>
         <v>-</v>
       </c>
       <c r="R26" s="10"/>
-      <c r="S26" s="97"/>
+      <c r="S26" s="146"/>
       <c r="T26" s="71"/>
       <c r="U26" s="71"/>
       <c r="V26" s="76"/>
@@ -3853,22 +3857,22 @@
       <c r="AC26" s="71"/>
       <c r="AD26" s="71"/>
       <c r="AE26" s="71"/>
-      <c r="AF26" s="167"/>
+      <c r="AF26" s="96"/>
       <c r="AG26" s="71"/>
-      <c r="AH26" s="123"/>
-      <c r="AI26" s="124"/>
-      <c r="AJ26" s="124"/>
-      <c r="AK26" s="124"/>
-      <c r="AL26" s="124"/>
-      <c r="AM26" s="125"/>
+      <c r="AH26" s="104"/>
+      <c r="AI26" s="105"/>
+      <c r="AJ26" s="105"/>
+      <c r="AK26" s="105"/>
+      <c r="AL26" s="105"/>
+      <c r="AM26" s="106"/>
       <c r="AN26" s="40"/>
-      <c r="AO26" s="113"/>
+      <c r="AO26" s="152"/>
     </row>
     <row r="27" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="84" t="s">
         <v>124</v>
       </c>
-      <c r="B27" s="95"/>
+      <c r="B27" s="173"/>
       <c r="C27" s="42"/>
       <c r="D27" s="66" t="s">
         <v>15</v>
@@ -3889,8 +3893,8 @@
         <v>29</v>
       </c>
       <c r="K27" s="71"/>
-      <c r="L27" s="118"/>
-      <c r="M27" s="99"/>
+      <c r="L27" s="160"/>
+      <c r="M27" s="149"/>
       <c r="N27" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #11</v>
@@ -3899,13 +3903,15 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P27" s="102"/>
+      <c r="P27" s="174" t="s">
+        <v>40</v>
+      </c>
       <c r="Q27" s="12" t="str" cm="1">
         <f t="array" ref="Q27">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B11))),"-")</f>
         <v>-</v>
       </c>
       <c r="R27" s="7"/>
-      <c r="S27" s="97"/>
+      <c r="S27" s="146"/>
       <c r="T27" s="71"/>
       <c r="U27" s="71"/>
       <c r="V27" s="76"/>
@@ -3918,22 +3924,22 @@
       <c r="AC27" s="71"/>
       <c r="AD27" s="71"/>
       <c r="AE27" s="71"/>
-      <c r="AF27" s="167"/>
+      <c r="AF27" s="96"/>
       <c r="AG27" s="71"/>
-      <c r="AH27" s="126"/>
-      <c r="AI27" s="127"/>
-      <c r="AJ27" s="127"/>
-      <c r="AK27" s="127"/>
-      <c r="AL27" s="127"/>
-      <c r="AM27" s="128"/>
+      <c r="AH27" s="107"/>
+      <c r="AI27" s="108"/>
+      <c r="AJ27" s="108"/>
+      <c r="AK27" s="108"/>
+      <c r="AL27" s="108"/>
+      <c r="AM27" s="109"/>
       <c r="AN27" s="40"/>
-      <c r="AO27" s="113"/>
+      <c r="AO27" s="152"/>
     </row>
     <row r="28" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="84" t="s">
         <v>90</v>
       </c>
-      <c r="B28" s="95"/>
+      <c r="B28" s="173"/>
       <c r="C28" s="42"/>
       <c r="D28" s="66" t="s">
         <v>16</v>
@@ -3954,8 +3960,8 @@
         <v>29</v>
       </c>
       <c r="K28" s="71"/>
-      <c r="L28" s="118"/>
-      <c r="M28" s="99"/>
+      <c r="L28" s="160"/>
+      <c r="M28" s="149"/>
       <c r="N28" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #12</v>
@@ -3964,13 +3970,13 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P28" s="103"/>
+      <c r="P28" s="174"/>
       <c r="Q28" s="13" t="str" cm="1">
         <f t="array" ref="Q28">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B15))),"-")</f>
         <v>-</v>
       </c>
       <c r="R28" s="8"/>
-      <c r="S28" s="97"/>
+      <c r="S28" s="146"/>
       <c r="T28" s="71"/>
       <c r="U28" s="71"/>
       <c r="V28" s="76"/>
@@ -3983,22 +3989,22 @@
       <c r="AC28" s="71"/>
       <c r="AD28" s="71"/>
       <c r="AE28" s="71"/>
-      <c r="AF28" s="167"/>
+      <c r="AF28" s="96"/>
       <c r="AG28" s="71"/>
-      <c r="AH28" s="104"/>
-      <c r="AI28" s="105"/>
-      <c r="AJ28" s="105"/>
-      <c r="AK28" s="105"/>
-      <c r="AL28" s="105"/>
-      <c r="AM28" s="107"/>
+      <c r="AH28" s="132"/>
+      <c r="AI28" s="130"/>
+      <c r="AJ28" s="130"/>
+      <c r="AK28" s="130"/>
+      <c r="AL28" s="130"/>
+      <c r="AM28" s="131"/>
       <c r="AN28" s="40"/>
-      <c r="AO28" s="113"/>
+      <c r="AO28" s="152"/>
     </row>
     <row r="29" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="84" t="s">
         <v>138</v>
       </c>
-      <c r="B29" s="95"/>
+      <c r="B29" s="173"/>
       <c r="C29" s="42"/>
       <c r="D29" s="66" t="s">
         <v>17</v>
@@ -4019,8 +4025,8 @@
         <v>30</v>
       </c>
       <c r="K29" s="71"/>
-      <c r="L29" s="118"/>
-      <c r="M29" s="99"/>
+      <c r="L29" s="160"/>
+      <c r="M29" s="149"/>
       <c r="N29" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #13</v>
@@ -4029,15 +4035,15 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P29" s="101" t="s">
-        <v>37</v>
+      <c r="P29" s="174" t="s">
+        <v>46</v>
       </c>
       <c r="Q29" s="11" t="str" cm="1">
         <f t="array" ref="Q29">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B4))),"-")</f>
         <v>-</v>
       </c>
       <c r="R29" s="9"/>
-      <c r="S29" s="97"/>
+      <c r="S29" s="146"/>
       <c r="T29" s="71"/>
       <c r="U29" s="71"/>
       <c r="V29" s="76"/>
@@ -4050,26 +4056,26 @@
       <c r="AC29" s="71"/>
       <c r="AD29" s="71"/>
       <c r="AE29" s="71"/>
-      <c r="AF29" s="167"/>
+      <c r="AF29" s="96"/>
       <c r="AG29" s="71"/>
-      <c r="AH29" s="96"/>
+      <c r="AH29" s="145"/>
       <c r="AI29" s="5">
         <v>8</v>
       </c>
-      <c r="AJ29" s="138" t="s">
+      <c r="AJ29" s="93" t="s">
         <v>31</v>
       </c>
-      <c r="AK29" s="138"/>
-      <c r="AL29" s="139"/>
-      <c r="AM29" s="96"/>
+      <c r="AK29" s="93"/>
+      <c r="AL29" s="94"/>
+      <c r="AM29" s="145"/>
       <c r="AN29" s="40"/>
-      <c r="AO29" s="113"/>
+      <c r="AO29" s="152"/>
     </row>
     <row r="30" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="84" t="s">
         <v>166</v>
       </c>
-      <c r="B30" s="95"/>
+      <c r="B30" s="173"/>
       <c r="C30" s="42"/>
       <c r="D30" s="67" t="s">
         <v>18</v>
@@ -4090,8 +4096,8 @@
         <v>30</v>
       </c>
       <c r="K30" s="71"/>
-      <c r="L30" s="118"/>
-      <c r="M30" s="99"/>
+      <c r="L30" s="160"/>
+      <c r="M30" s="149"/>
       <c r="N30" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #14</v>
@@ -4100,13 +4106,13 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P30" s="102"/>
+      <c r="P30" s="174"/>
       <c r="Q30" s="12" t="str" cm="1">
         <f t="array" ref="Q30">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B8))),"-")</f>
         <v>-</v>
       </c>
       <c r="R30" s="10"/>
-      <c r="S30" s="97"/>
+      <c r="S30" s="146"/>
       <c r="T30" s="71"/>
       <c r="U30" s="71"/>
       <c r="V30" s="76"/>
@@ -4119,9 +4125,9 @@
       <c r="AC30" s="71"/>
       <c r="AD30" s="71"/>
       <c r="AE30" s="71"/>
-      <c r="AF30" s="167"/>
+      <c r="AF30" s="96"/>
       <c r="AG30" s="71"/>
-      <c r="AH30" s="97"/>
+      <c r="AH30" s="146"/>
       <c r="AI30" s="4" t="s">
         <v>32</v>
       </c>
@@ -4134,15 +4140,15 @@
       <c r="AL30" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="AM30" s="97"/>
+      <c r="AM30" s="146"/>
       <c r="AN30" s="40"/>
-      <c r="AO30" s="113"/>
+      <c r="AO30" s="152"/>
     </row>
     <row r="31" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="84" t="s">
         <v>125</v>
       </c>
-      <c r="B31" s="95"/>
+      <c r="B31" s="173"/>
       <c r="C31" s="42"/>
       <c r="D31" s="79"/>
       <c r="E31" s="72"/>
@@ -4152,8 +4158,8 @@
       <c r="I31" s="72"/>
       <c r="J31" s="72"/>
       <c r="K31" s="80"/>
-      <c r="L31" s="118"/>
-      <c r="M31" s="99"/>
+      <c r="L31" s="160"/>
+      <c r="M31" s="149"/>
       <c r="N31" s="75" t="str">
         <f t="shared" si="1"/>
         <v>Participant #15</v>
@@ -4162,13 +4168,15 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P31" s="102"/>
+      <c r="P31" s="174" t="s">
+        <v>47</v>
+      </c>
       <c r="Q31" s="12" t="str" cm="1">
         <f t="array" ref="Q31">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B12))),"-")</f>
         <v>-</v>
       </c>
       <c r="R31" s="7"/>
-      <c r="S31" s="97"/>
+      <c r="S31" s="146"/>
       <c r="T31" s="71"/>
       <c r="U31" s="71"/>
       <c r="V31" s="76"/>
@@ -4181,10 +4189,10 @@
       <c r="AC31" s="71"/>
       <c r="AD31" s="71"/>
       <c r="AE31" s="71"/>
-      <c r="AF31" s="167"/>
+      <c r="AF31" s="96"/>
       <c r="AG31" s="71"/>
-      <c r="AH31" s="97"/>
-      <c r="AI31" s="101" t="s">
+      <c r="AH31" s="146"/>
+      <c r="AI31" s="98" t="s">
         <v>56</v>
       </c>
       <c r="AJ31" s="21" t="str">
@@ -4195,15 +4203,15 @@
       <c r="AL31" s="47">
         <v>0</v>
       </c>
-      <c r="AM31" s="99"/>
+      <c r="AM31" s="149"/>
       <c r="AN31" s="40"/>
-      <c r="AO31" s="113"/>
+      <c r="AO31" s="152"/>
     </row>
     <row r="32" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="84" t="s">
         <v>147</v>
       </c>
-      <c r="B32" s="95"/>
+      <c r="B32" s="173"/>
       <c r="C32" s="42"/>
       <c r="D32" s="79"/>
       <c r="E32" s="72"/>
@@ -4213,8 +4221,8 @@
       <c r="I32" s="72"/>
       <c r="J32" s="72"/>
       <c r="K32" s="80"/>
-      <c r="L32" s="118"/>
-      <c r="M32" s="100"/>
+      <c r="L32" s="160"/>
+      <c r="M32" s="150"/>
       <c r="N32" s="60" t="str">
         <f t="shared" si="1"/>
         <v>Participant #16</v>
@@ -4223,13 +4231,13 @@
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="P32" s="103"/>
+      <c r="P32" s="174"/>
       <c r="Q32" s="13" t="str" cm="1">
         <f t="array" ref="Q32">IFERROR(INDEX($N$17:$N$32,SMALL($O$17:$O$32,ROW(B16))),"-")</f>
         <v>-</v>
       </c>
       <c r="R32" s="8"/>
-      <c r="S32" s="98"/>
+      <c r="S32" s="147"/>
       <c r="T32" s="71"/>
       <c r="U32" s="71"/>
       <c r="V32" s="76"/>
@@ -4242,10 +4250,10 @@
       <c r="AC32" s="71"/>
       <c r="AD32" s="71"/>
       <c r="AE32" s="71"/>
-      <c r="AF32" s="167"/>
+      <c r="AF32" s="96"/>
       <c r="AG32" s="71"/>
-      <c r="AH32" s="97"/>
-      <c r="AI32" s="102"/>
+      <c r="AH32" s="146"/>
+      <c r="AI32" s="99"/>
       <c r="AJ32" s="22" t="str">
         <f>IF(ISBLANK($AD$51),"L2",$AD$51)</f>
         <v>L2</v>
@@ -4254,15 +4262,15 @@
       <c r="AL32" s="48">
         <v>0</v>
       </c>
-      <c r="AM32" s="99"/>
+      <c r="AM32" s="149"/>
       <c r="AN32" s="40"/>
-      <c r="AO32" s="113"/>
+      <c r="AO32" s="152"/>
     </row>
     <row r="33" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="84" t="s">
         <v>64</v>
       </c>
-      <c r="B33" s="95"/>
+      <c r="B33" s="173"/>
       <c r="C33" s="42"/>
       <c r="D33" s="79"/>
       <c r="E33" s="72"/>
@@ -4272,17 +4280,17 @@
       <c r="I33" s="72"/>
       <c r="J33" s="72"/>
       <c r="K33" s="80"/>
-      <c r="L33" s="118"/>
-      <c r="M33" s="105" t="str">
+      <c r="L33" s="160"/>
+      <c r="M33" s="130" t="str">
         <f>IF(E31&gt;=1,ROW()-$O$16,"")</f>
         <v/>
       </c>
-      <c r="N33" s="105"/>
-      <c r="O33" s="105"/>
-      <c r="P33" s="105"/>
-      <c r="Q33" s="105"/>
-      <c r="R33" s="105"/>
-      <c r="S33" s="107"/>
+      <c r="N33" s="130"/>
+      <c r="O33" s="130"/>
+      <c r="P33" s="130"/>
+      <c r="Q33" s="130"/>
+      <c r="R33" s="130"/>
+      <c r="S33" s="131"/>
       <c r="T33" s="71"/>
       <c r="U33" s="71"/>
       <c r="V33" s="71"/>
@@ -4295,10 +4303,10 @@
       <c r="AC33" s="71"/>
       <c r="AD33" s="71"/>
       <c r="AE33" s="71"/>
-      <c r="AF33" s="167"/>
+      <c r="AF33" s="96"/>
       <c r="AG33" s="71"/>
-      <c r="AH33" s="97"/>
-      <c r="AI33" s="102"/>
+      <c r="AH33" s="146"/>
+      <c r="AI33" s="99"/>
       <c r="AJ33" s="22" t="str">
         <f>IF(ISBLANK($AD$49),"K3",$AD$49)</f>
         <v>K3</v>
@@ -4307,15 +4315,15 @@
       <c r="AL33" s="49">
         <v>0</v>
       </c>
-      <c r="AM33" s="99"/>
+      <c r="AM33" s="149"/>
       <c r="AN33" s="40"/>
-      <c r="AO33" s="113"/>
+      <c r="AO33" s="152"/>
     </row>
     <row r="34" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="84" t="s">
         <v>98</v>
       </c>
-      <c r="B34" s="95"/>
+      <c r="B34" s="173"/>
       <c r="C34" s="42"/>
       <c r="D34" s="79"/>
       <c r="E34" s="72"/>
@@ -4325,7 +4333,7 @@
       <c r="I34" s="72"/>
       <c r="J34" s="72"/>
       <c r="K34" s="80"/>
-      <c r="L34" s="118"/>
+      <c r="L34" s="160"/>
       <c r="M34" s="71"/>
       <c r="N34" s="71"/>
       <c r="O34" s="71" t="str">
@@ -4348,10 +4356,10 @@
       <c r="AC34" s="71"/>
       <c r="AD34" s="71"/>
       <c r="AE34" s="71"/>
-      <c r="AF34" s="167"/>
+      <c r="AF34" s="96"/>
       <c r="AG34" s="71"/>
-      <c r="AH34" s="98"/>
-      <c r="AI34" s="103"/>
+      <c r="AH34" s="147"/>
+      <c r="AI34" s="100"/>
       <c r="AJ34" s="23" t="str">
         <f>IF(ISBLANK($AD$52),"L3",$AD$52)</f>
         <v>L3</v>
@@ -4360,15 +4368,15 @@
       <c r="AL34" s="14">
         <v>0</v>
       </c>
-      <c r="AM34" s="100"/>
+      <c r="AM34" s="150"/>
       <c r="AN34" s="40"/>
-      <c r="AO34" s="113"/>
+      <c r="AO34" s="152"/>
     </row>
     <row r="35" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="84" t="s">
         <v>104</v>
       </c>
-      <c r="B35" s="95"/>
+      <c r="B35" s="173"/>
       <c r="C35" s="42"/>
       <c r="D35" s="79"/>
       <c r="E35" s="72"/>
@@ -4378,7 +4386,7 @@
       <c r="I35" s="72"/>
       <c r="J35" s="72"/>
       <c r="K35" s="80"/>
-      <c r="L35" s="118"/>
+      <c r="L35" s="160"/>
       <c r="M35" s="71"/>
       <c r="N35" s="82"/>
       <c r="O35" s="82"/>
@@ -4398,22 +4406,22 @@
       <c r="AC35" s="82"/>
       <c r="AD35" s="82"/>
       <c r="AE35" s="82"/>
-      <c r="AF35" s="167"/>
+      <c r="AF35" s="96"/>
       <c r="AG35" s="71"/>
-      <c r="AH35" s="104"/>
-      <c r="AI35" s="105"/>
-      <c r="AJ35" s="106"/>
-      <c r="AK35" s="106"/>
-      <c r="AL35" s="106"/>
-      <c r="AM35" s="107"/>
+      <c r="AH35" s="132"/>
+      <c r="AI35" s="130"/>
+      <c r="AJ35" s="162"/>
+      <c r="AK35" s="162"/>
+      <c r="AL35" s="162"/>
+      <c r="AM35" s="131"/>
       <c r="AN35" s="40"/>
-      <c r="AO35" s="113"/>
+      <c r="AO35" s="152"/>
     </row>
     <row r="36" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="84" t="s">
         <v>106</v>
       </c>
-      <c r="B36" s="95"/>
+      <c r="B36" s="173"/>
       <c r="C36" s="42"/>
       <c r="D36" s="79"/>
       <c r="E36" s="72"/>
@@ -4423,29 +4431,29 @@
       <c r="I36" s="72"/>
       <c r="J36" s="72"/>
       <c r="K36" s="80"/>
-      <c r="L36" s="118"/>
-      <c r="M36" s="129" t="s">
+      <c r="L36" s="160"/>
+      <c r="M36" s="133" t="s">
         <v>43</v>
       </c>
-      <c r="N36" s="130"/>
-      <c r="O36" s="130"/>
-      <c r="P36" s="130"/>
-      <c r="Q36" s="130"/>
-      <c r="R36" s="130"/>
-      <c r="S36" s="130"/>
-      <c r="T36" s="130"/>
-      <c r="U36" s="130"/>
-      <c r="V36" s="130"/>
-      <c r="W36" s="130"/>
-      <c r="X36" s="130"/>
-      <c r="Y36" s="130"/>
-      <c r="Z36" s="130"/>
-      <c r="AA36" s="130"/>
-      <c r="AB36" s="130"/>
-      <c r="AC36" s="130"/>
-      <c r="AD36" s="130"/>
-      <c r="AE36" s="131"/>
-      <c r="AF36" s="167"/>
+      <c r="N36" s="134"/>
+      <c r="O36" s="134"/>
+      <c r="P36" s="134"/>
+      <c r="Q36" s="134"/>
+      <c r="R36" s="134"/>
+      <c r="S36" s="134"/>
+      <c r="T36" s="134"/>
+      <c r="U36" s="134"/>
+      <c r="V36" s="134"/>
+      <c r="W36" s="134"/>
+      <c r="X36" s="134"/>
+      <c r="Y36" s="134"/>
+      <c r="Z36" s="134"/>
+      <c r="AA36" s="134"/>
+      <c r="AB36" s="134"/>
+      <c r="AC36" s="134"/>
+      <c r="AD36" s="134"/>
+      <c r="AE36" s="135"/>
+      <c r="AF36" s="96"/>
       <c r="AG36" s="71"/>
       <c r="AH36" s="71"/>
       <c r="AI36" s="71"/>
@@ -4454,13 +4462,13 @@
       <c r="AL36" s="71"/>
       <c r="AM36" s="71"/>
       <c r="AN36" s="40"/>
-      <c r="AO36" s="113"/>
+      <c r="AO36" s="152"/>
     </row>
     <row r="37" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="84" t="s">
         <v>105</v>
       </c>
-      <c r="B37" s="95"/>
+      <c r="B37" s="173"/>
       <c r="C37" s="42"/>
       <c r="D37" s="79"/>
       <c r="E37" s="72"/>
@@ -4470,27 +4478,27 @@
       <c r="I37" s="72"/>
       <c r="J37" s="72"/>
       <c r="K37" s="80"/>
-      <c r="L37" s="118"/>
-      <c r="M37" s="132"/>
-      <c r="N37" s="133"/>
-      <c r="O37" s="133"/>
-      <c r="P37" s="133"/>
-      <c r="Q37" s="133"/>
-      <c r="R37" s="133"/>
-      <c r="S37" s="133"/>
-      <c r="T37" s="133"/>
-      <c r="U37" s="133"/>
-      <c r="V37" s="133"/>
-      <c r="W37" s="133"/>
-      <c r="X37" s="133"/>
-      <c r="Y37" s="133"/>
-      <c r="Z37" s="133"/>
-      <c r="AA37" s="133"/>
-      <c r="AB37" s="133"/>
-      <c r="AC37" s="133"/>
-      <c r="AD37" s="133"/>
-      <c r="AE37" s="134"/>
-      <c r="AF37" s="167"/>
+      <c r="L37" s="160"/>
+      <c r="M37" s="136"/>
+      <c r="N37" s="137"/>
+      <c r="O37" s="137"/>
+      <c r="P37" s="137"/>
+      <c r="Q37" s="137"/>
+      <c r="R37" s="137"/>
+      <c r="S37" s="137"/>
+      <c r="T37" s="137"/>
+      <c r="U37" s="137"/>
+      <c r="V37" s="137"/>
+      <c r="W37" s="137"/>
+      <c r="X37" s="137"/>
+      <c r="Y37" s="137"/>
+      <c r="Z37" s="137"/>
+      <c r="AA37" s="137"/>
+      <c r="AB37" s="137"/>
+      <c r="AC37" s="137"/>
+      <c r="AD37" s="137"/>
+      <c r="AE37" s="138"/>
+      <c r="AF37" s="96"/>
       <c r="AG37" s="71"/>
       <c r="AH37" s="71"/>
       <c r="AI37" s="71"/>
@@ -4499,13 +4507,13 @@
       <c r="AL37" s="71"/>
       <c r="AM37" s="71"/>
       <c r="AN37" s="40"/>
-      <c r="AO37" s="113"/>
+      <c r="AO37" s="152"/>
     </row>
     <row r="38" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="84" t="s">
         <v>101</v>
       </c>
-      <c r="B38" s="95"/>
+      <c r="B38" s="173"/>
       <c r="C38" s="42"/>
       <c r="D38" s="79"/>
       <c r="E38" s="72"/>
@@ -4515,27 +4523,27 @@
       <c r="I38" s="72"/>
       <c r="J38" s="72"/>
       <c r="K38" s="80"/>
-      <c r="L38" s="118"/>
-      <c r="M38" s="135"/>
-      <c r="N38" s="136"/>
-      <c r="O38" s="136"/>
-      <c r="P38" s="136"/>
-      <c r="Q38" s="136"/>
-      <c r="R38" s="136"/>
-      <c r="S38" s="136"/>
-      <c r="T38" s="136"/>
-      <c r="U38" s="136"/>
-      <c r="V38" s="136"/>
-      <c r="W38" s="136"/>
-      <c r="X38" s="136"/>
-      <c r="Y38" s="136"/>
-      <c r="Z38" s="136"/>
-      <c r="AA38" s="136"/>
-      <c r="AB38" s="136"/>
-      <c r="AC38" s="136"/>
-      <c r="AD38" s="136"/>
-      <c r="AE38" s="137"/>
-      <c r="AF38" s="167"/>
+      <c r="L38" s="160"/>
+      <c r="M38" s="139"/>
+      <c r="N38" s="140"/>
+      <c r="O38" s="140"/>
+      <c r="P38" s="140"/>
+      <c r="Q38" s="140"/>
+      <c r="R38" s="140"/>
+      <c r="S38" s="140"/>
+      <c r="T38" s="140"/>
+      <c r="U38" s="140"/>
+      <c r="V38" s="140"/>
+      <c r="W38" s="140"/>
+      <c r="X38" s="140"/>
+      <c r="Y38" s="140"/>
+      <c r="Z38" s="140"/>
+      <c r="AA38" s="140"/>
+      <c r="AB38" s="140"/>
+      <c r="AC38" s="140"/>
+      <c r="AD38" s="140"/>
+      <c r="AE38" s="141"/>
+      <c r="AF38" s="96"/>
       <c r="AG38" s="71"/>
       <c r="AH38" s="71"/>
       <c r="AI38" s="71"/>
@@ -4544,13 +4552,13 @@
       <c r="AL38" s="71"/>
       <c r="AM38" s="71"/>
       <c r="AN38" s="40"/>
-      <c r="AO38" s="113"/>
+      <c r="AO38" s="152"/>
     </row>
     <row r="39" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="84" t="s">
         <v>103</v>
       </c>
-      <c r="B39" s="95"/>
+      <c r="B39" s="173"/>
       <c r="C39" s="42"/>
       <c r="D39" s="79"/>
       <c r="E39" s="72"/>
@@ -4560,7 +4568,7 @@
       <c r="I39" s="72"/>
       <c r="J39" s="72"/>
       <c r="K39" s="80"/>
-      <c r="L39" s="118"/>
+      <c r="L39" s="160"/>
       <c r="M39" s="71"/>
       <c r="N39" s="71"/>
       <c r="O39" s="71"/>
@@ -4580,7 +4588,7 @@
       <c r="AC39" s="71"/>
       <c r="AD39" s="71"/>
       <c r="AE39" s="71"/>
-      <c r="AF39" s="167"/>
+      <c r="AF39" s="96"/>
       <c r="AG39" s="71"/>
       <c r="AH39" s="71"/>
       <c r="AI39" s="71"/>
@@ -4589,13 +4597,13 @@
       <c r="AL39" s="71"/>
       <c r="AM39" s="71"/>
       <c r="AN39" s="40"/>
-      <c r="AO39" s="113"/>
+      <c r="AO39" s="152"/>
     </row>
     <row r="40" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="84" t="s">
         <v>102</v>
       </c>
-      <c r="B40" s="95"/>
+      <c r="B40" s="173"/>
       <c r="C40" s="42"/>
       <c r="D40" s="79"/>
       <c r="E40" s="72"/>
@@ -4605,7 +4613,7 @@
       <c r="I40" s="72"/>
       <c r="J40" s="72"/>
       <c r="K40" s="80"/>
-      <c r="L40" s="118"/>
+      <c r="L40" s="160"/>
       <c r="M40" s="71"/>
       <c r="N40" s="71"/>
       <c r="O40" s="71"/>
@@ -4625,7 +4633,7 @@
       <c r="AC40" s="71"/>
       <c r="AD40" s="71"/>
       <c r="AE40" s="71"/>
-      <c r="AF40" s="167"/>
+      <c r="AF40" s="96"/>
       <c r="AG40" s="71"/>
       <c r="AH40" s="71"/>
       <c r="AI40" s="71"/>
@@ -4634,13 +4642,13 @@
       <c r="AL40" s="71"/>
       <c r="AM40" s="71"/>
       <c r="AN40" s="40"/>
-      <c r="AO40" s="113"/>
+      <c r="AO40" s="152"/>
     </row>
     <row r="41" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="84" t="s">
         <v>122</v>
       </c>
-      <c r="B41" s="95"/>
+      <c r="B41" s="173"/>
       <c r="C41" s="42"/>
       <c r="D41" s="79"/>
       <c r="E41" s="72"/>
@@ -4650,33 +4658,33 @@
       <c r="I41" s="72"/>
       <c r="J41" s="72"/>
       <c r="K41" s="80"/>
-      <c r="L41" s="118"/>
-      <c r="M41" s="121" t="s">
+      <c r="L41" s="160"/>
+      <c r="M41" s="102" t="s">
         <v>44</v>
       </c>
-      <c r="N41" s="121"/>
-      <c r="O41" s="121"/>
-      <c r="P41" s="121"/>
-      <c r="Q41" s="121"/>
-      <c r="R41" s="121"/>
-      <c r="S41" s="122"/>
+      <c r="N41" s="102"/>
+      <c r="O41" s="102"/>
+      <c r="P41" s="102"/>
+      <c r="Q41" s="102"/>
+      <c r="R41" s="102"/>
+      <c r="S41" s="103"/>
       <c r="T41" s="70"/>
-      <c r="U41" s="120" t="s">
+      <c r="U41" s="101" t="s">
         <v>48</v>
       </c>
-      <c r="V41" s="121"/>
-      <c r="W41" s="121"/>
-      <c r="X41" s="121"/>
-      <c r="Y41" s="122"/>
+      <c r="V41" s="102"/>
+      <c r="W41" s="102"/>
+      <c r="X41" s="102"/>
+      <c r="Y41" s="103"/>
       <c r="Z41" s="70"/>
-      <c r="AA41" s="120" t="s">
+      <c r="AA41" s="101" t="s">
         <v>51</v>
       </c>
-      <c r="AB41" s="121"/>
-      <c r="AC41" s="121"/>
-      <c r="AD41" s="121"/>
-      <c r="AE41" s="121"/>
-      <c r="AF41" s="167"/>
+      <c r="AB41" s="102"/>
+      <c r="AC41" s="102"/>
+      <c r="AD41" s="102"/>
+      <c r="AE41" s="102"/>
+      <c r="AF41" s="96"/>
       <c r="AG41" s="71"/>
       <c r="AH41" s="71"/>
       <c r="AI41" s="71"/>
@@ -4685,13 +4693,13 @@
       <c r="AL41" s="71"/>
       <c r="AM41" s="71"/>
       <c r="AN41" s="40"/>
-      <c r="AO41" s="113"/>
+      <c r="AO41" s="152"/>
     </row>
     <row r="42" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="84" t="s">
         <v>77</v>
       </c>
-      <c r="B42" s="95"/>
+      <c r="B42" s="173"/>
       <c r="C42" s="42"/>
       <c r="D42" s="79"/>
       <c r="E42" s="72"/>
@@ -4701,27 +4709,27 @@
       <c r="I42" s="72"/>
       <c r="J42" s="72"/>
       <c r="K42" s="80"/>
-      <c r="L42" s="118"/>
-      <c r="M42" s="124"/>
-      <c r="N42" s="124"/>
-      <c r="O42" s="124"/>
-      <c r="P42" s="124"/>
-      <c r="Q42" s="124"/>
-      <c r="R42" s="124"/>
-      <c r="S42" s="125"/>
+      <c r="L42" s="160"/>
+      <c r="M42" s="105"/>
+      <c r="N42" s="105"/>
+      <c r="O42" s="105"/>
+      <c r="P42" s="105"/>
+      <c r="Q42" s="105"/>
+      <c r="R42" s="105"/>
+      <c r="S42" s="106"/>
       <c r="T42" s="70"/>
-      <c r="U42" s="123"/>
-      <c r="V42" s="124"/>
-      <c r="W42" s="124"/>
-      <c r="X42" s="124"/>
-      <c r="Y42" s="125"/>
+      <c r="U42" s="104"/>
+      <c r="V42" s="105"/>
+      <c r="W42" s="105"/>
+      <c r="X42" s="105"/>
+      <c r="Y42" s="106"/>
       <c r="Z42" s="70"/>
-      <c r="AA42" s="123"/>
-      <c r="AB42" s="124"/>
-      <c r="AC42" s="124"/>
-      <c r="AD42" s="124"/>
-      <c r="AE42" s="124"/>
-      <c r="AF42" s="167"/>
+      <c r="AA42" s="104"/>
+      <c r="AB42" s="105"/>
+      <c r="AC42" s="105"/>
+      <c r="AD42" s="105"/>
+      <c r="AE42" s="105"/>
+      <c r="AF42" s="96"/>
       <c r="AG42" s="71"/>
       <c r="AH42" s="71"/>
       <c r="AI42" s="71"/>
@@ -4730,13 +4738,13 @@
       <c r="AL42" s="71"/>
       <c r="AM42" s="71"/>
       <c r="AN42" s="40"/>
-      <c r="AO42" s="113"/>
+      <c r="AO42" s="152"/>
     </row>
     <row r="43" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="84" t="s">
         <v>86</v>
       </c>
-      <c r="B43" s="95"/>
+      <c r="B43" s="173"/>
       <c r="C43" s="42"/>
       <c r="D43" s="79"/>
       <c r="E43" s="72"/>
@@ -4746,27 +4754,27 @@
       <c r="I43" s="72"/>
       <c r="J43" s="72"/>
       <c r="K43" s="80"/>
-      <c r="L43" s="118"/>
-      <c r="M43" s="127"/>
-      <c r="N43" s="127"/>
-      <c r="O43" s="127"/>
-      <c r="P43" s="127"/>
-      <c r="Q43" s="127"/>
-      <c r="R43" s="127"/>
-      <c r="S43" s="128"/>
+      <c r="L43" s="160"/>
+      <c r="M43" s="108"/>
+      <c r="N43" s="108"/>
+      <c r="O43" s="108"/>
+      <c r="P43" s="108"/>
+      <c r="Q43" s="108"/>
+      <c r="R43" s="108"/>
+      <c r="S43" s="109"/>
       <c r="T43" s="70"/>
-      <c r="U43" s="126"/>
-      <c r="V43" s="127"/>
-      <c r="W43" s="127"/>
-      <c r="X43" s="127"/>
-      <c r="Y43" s="128"/>
+      <c r="U43" s="107"/>
+      <c r="V43" s="108"/>
+      <c r="W43" s="108"/>
+      <c r="X43" s="108"/>
+      <c r="Y43" s="109"/>
       <c r="Z43" s="70"/>
-      <c r="AA43" s="126"/>
-      <c r="AB43" s="127"/>
-      <c r="AC43" s="127"/>
-      <c r="AD43" s="127"/>
-      <c r="AE43" s="127"/>
-      <c r="AF43" s="167"/>
+      <c r="AA43" s="107"/>
+      <c r="AB43" s="108"/>
+      <c r="AC43" s="108"/>
+      <c r="AD43" s="108"/>
+      <c r="AE43" s="108"/>
+      <c r="AF43" s="96"/>
       <c r="AG43" s="71"/>
       <c r="AH43" s="71"/>
       <c r="AI43" s="71"/>
@@ -4775,13 +4783,13 @@
       <c r="AL43" s="71"/>
       <c r="AM43" s="71"/>
       <c r="AN43" s="40"/>
-      <c r="AO43" s="113"/>
+      <c r="AO43" s="152"/>
     </row>
     <row r="44" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="84" t="s">
         <v>95</v>
       </c>
-      <c r="B44" s="95"/>
+      <c r="B44" s="173"/>
       <c r="C44" s="42"/>
       <c r="D44" s="79"/>
       <c r="E44" s="72"/>
@@ -4791,27 +4799,27 @@
       <c r="I44" s="72"/>
       <c r="J44" s="72"/>
       <c r="K44" s="80"/>
-      <c r="L44" s="118"/>
-      <c r="M44" s="105"/>
-      <c r="N44" s="105"/>
-      <c r="O44" s="105"/>
-      <c r="P44" s="105"/>
-      <c r="Q44" s="105"/>
-      <c r="R44" s="105"/>
-      <c r="S44" s="107"/>
+      <c r="L44" s="160"/>
+      <c r="M44" s="130"/>
+      <c r="N44" s="130"/>
+      <c r="O44" s="130"/>
+      <c r="P44" s="130"/>
+      <c r="Q44" s="130"/>
+      <c r="R44" s="130"/>
+      <c r="S44" s="131"/>
       <c r="T44" s="71"/>
-      <c r="U44" s="104"/>
-      <c r="V44" s="105"/>
-      <c r="W44" s="105"/>
-      <c r="X44" s="105"/>
-      <c r="Y44" s="107"/>
+      <c r="U44" s="132"/>
+      <c r="V44" s="130"/>
+      <c r="W44" s="130"/>
+      <c r="X44" s="130"/>
+      <c r="Y44" s="131"/>
       <c r="Z44" s="71"/>
-      <c r="AA44" s="104"/>
-      <c r="AB44" s="105"/>
-      <c r="AC44" s="105"/>
-      <c r="AD44" s="105"/>
-      <c r="AE44" s="105"/>
-      <c r="AF44" s="167"/>
+      <c r="AA44" s="132"/>
+      <c r="AB44" s="130"/>
+      <c r="AC44" s="130"/>
+      <c r="AD44" s="130"/>
+      <c r="AE44" s="130"/>
+      <c r="AF44" s="96"/>
       <c r="AG44" s="71"/>
       <c r="AH44" s="71"/>
       <c r="AI44" s="71"/>
@@ -4820,13 +4828,13 @@
       <c r="AL44" s="71"/>
       <c r="AM44" s="71"/>
       <c r="AN44" s="40"/>
-      <c r="AO44" s="113"/>
+      <c r="AO44" s="152"/>
     </row>
     <row r="45" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="84" t="s">
         <v>94</v>
       </c>
-      <c r="B45" s="95"/>
+      <c r="B45" s="173"/>
       <c r="C45" s="42"/>
       <c r="D45" s="79"/>
       <c r="E45" s="72"/>
@@ -4836,8 +4844,8 @@
       <c r="I45" s="72"/>
       <c r="J45" s="72"/>
       <c r="K45" s="80"/>
-      <c r="L45" s="118"/>
-      <c r="M45" s="111"/>
+      <c r="L45" s="160"/>
+      <c r="M45" s="148"/>
       <c r="P45" s="18">
         <v>4</v>
       </c>
@@ -4845,28 +4853,28 @@
         <v>31</v>
       </c>
       <c r="R45" s="20"/>
-      <c r="S45" s="96"/>
+      <c r="S45" s="145"/>
       <c r="T45" s="71"/>
-      <c r="U45" s="96"/>
+      <c r="U45" s="145"/>
       <c r="V45" s="5">
         <v>4</v>
       </c>
-      <c r="W45" s="138" t="s">
+      <c r="W45" s="93" t="s">
         <v>31</v>
       </c>
-      <c r="X45" s="139"/>
-      <c r="Y45" s="96"/>
+      <c r="X45" s="94"/>
+      <c r="Y45" s="145"/>
       <c r="Z45" s="83"/>
-      <c r="AA45" s="96"/>
+      <c r="AA45" s="145"/>
       <c r="AB45" s="5">
         <v>6</v>
       </c>
-      <c r="AC45" s="138" t="s">
+      <c r="AC45" s="93" t="s">
         <v>31</v>
       </c>
-      <c r="AD45" s="139"/>
-      <c r="AE45" s="108"/>
-      <c r="AF45" s="167"/>
+      <c r="AD45" s="94"/>
+      <c r="AE45" s="156"/>
+      <c r="AF45" s="96"/>
       <c r="AG45" s="71"/>
       <c r="AH45" s="71"/>
       <c r="AI45" s="71"/>
@@ -4875,13 +4883,13 @@
       <c r="AL45" s="71"/>
       <c r="AM45" s="71"/>
       <c r="AN45" s="40"/>
-      <c r="AO45" s="113"/>
+      <c r="AO45" s="152"/>
     </row>
     <row r="46" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="84" t="s">
         <v>107</v>
       </c>
-      <c r="B46" s="95"/>
+      <c r="B46" s="173"/>
       <c r="C46" s="42"/>
       <c r="D46" s="79"/>
       <c r="E46" s="72"/>
@@ -4891,8 +4899,8 @@
       <c r="I46" s="72"/>
       <c r="J46" s="72"/>
       <c r="K46" s="80"/>
-      <c r="L46" s="118"/>
-      <c r="M46" s="99"/>
+      <c r="L46" s="160"/>
+      <c r="M46" s="149"/>
       <c r="P46" s="4" t="s">
         <v>32</v>
       </c>
@@ -4902,9 +4910,9 @@
       <c r="R46" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="S46" s="97"/>
+      <c r="S46" s="146"/>
       <c r="T46" s="71"/>
-      <c r="U46" s="97"/>
+      <c r="U46" s="146"/>
       <c r="V46" s="4" t="s">
         <v>32</v>
       </c>
@@ -4914,9 +4922,9 @@
       <c r="X46" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="Y46" s="97"/>
+      <c r="Y46" s="146"/>
       <c r="Z46" s="72"/>
-      <c r="AA46" s="97"/>
+      <c r="AA46" s="146"/>
       <c r="AB46" s="4" t="s">
         <v>32</v>
       </c>
@@ -4926,8 +4934,8 @@
       <c r="AD46" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="AE46" s="109"/>
-      <c r="AF46" s="167"/>
+      <c r="AE46" s="157"/>
+      <c r="AF46" s="96"/>
       <c r="AG46" s="71"/>
       <c r="AH46" s="71"/>
       <c r="AI46" s="71"/>
@@ -4936,13 +4944,13 @@
       <c r="AL46" s="71"/>
       <c r="AM46" s="71"/>
       <c r="AN46" s="40"/>
-      <c r="AO46" s="113"/>
+      <c r="AO46" s="152"/>
     </row>
     <row r="47" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="84" t="s">
         <v>108</v>
       </c>
-      <c r="B47" s="95"/>
+      <c r="B47" s="173"/>
       <c r="C47" s="42"/>
       <c r="D47" s="79"/>
       <c r="E47" s="72"/>
@@ -4952,9 +4960,9 @@
       <c r="I47" s="72"/>
       <c r="J47" s="72"/>
       <c r="K47" s="80"/>
-      <c r="L47" s="118"/>
-      <c r="M47" s="99"/>
-      <c r="P47" s="140" t="s">
+      <c r="L47" s="160"/>
+      <c r="M47" s="149"/>
+      <c r="P47" s="142" t="s">
         <v>46</v>
       </c>
       <c r="Q47" s="11" t="str">
@@ -4962,10 +4970,10 @@
         <v>A3</v>
       </c>
       <c r="R47" s="6"/>
-      <c r="S47" s="97"/>
+      <c r="S47" s="146"/>
       <c r="T47" s="71"/>
-      <c r="U47" s="97"/>
-      <c r="V47" s="101" t="s">
+      <c r="U47" s="146"/>
+      <c r="V47" s="98" t="s">
         <v>50</v>
       </c>
       <c r="W47" s="11" t="str">
@@ -4973,10 +4981,10 @@
         <v>G1</v>
       </c>
       <c r="X47" s="6"/>
-      <c r="Y47" s="97"/>
+      <c r="Y47" s="146"/>
       <c r="Z47" s="77"/>
-      <c r="AA47" s="97"/>
-      <c r="AB47" s="140" t="s">
+      <c r="AA47" s="146"/>
+      <c r="AB47" s="142" t="s">
         <v>57</v>
       </c>
       <c r="AC47" s="21" t="str">
@@ -4984,8 +4992,8 @@
         <v>WF3</v>
       </c>
       <c r="AD47" s="26"/>
-      <c r="AE47" s="109"/>
-      <c r="AF47" s="167"/>
+      <c r="AE47" s="157"/>
+      <c r="AF47" s="96"/>
       <c r="AG47" s="71"/>
       <c r="AH47" s="71"/>
       <c r="AI47" s="71"/>
@@ -4994,13 +5002,13 @@
       <c r="AL47" s="71"/>
       <c r="AM47" s="71"/>
       <c r="AN47" s="40"/>
-      <c r="AO47" s="113"/>
+      <c r="AO47" s="152"/>
     </row>
     <row r="48" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="84" t="s">
         <v>97</v>
       </c>
-      <c r="B48" s="95"/>
+      <c r="B48" s="173"/>
       <c r="C48" s="42"/>
       <c r="D48" s="79"/>
       <c r="E48" s="72"/>
@@ -5010,34 +5018,34 @@
       <c r="I48" s="72"/>
       <c r="J48" s="72"/>
       <c r="K48" s="80"/>
-      <c r="L48" s="118"/>
-      <c r="M48" s="99"/>
-      <c r="P48" s="141"/>
+      <c r="L48" s="160"/>
+      <c r="M48" s="149"/>
+      <c r="P48" s="143"/>
       <c r="Q48" s="12" t="str">
         <f>IF(ISBLANK($R$27),"C3",$R$27)</f>
         <v>C3</v>
       </c>
       <c r="R48" s="14"/>
-      <c r="S48" s="97"/>
+      <c r="S48" s="146"/>
       <c r="T48" s="71"/>
-      <c r="U48" s="97"/>
-      <c r="V48" s="102"/>
+      <c r="U48" s="146"/>
+      <c r="V48" s="99"/>
       <c r="W48" s="12" t="str">
         <f>IF(ISBLANK($R$52),"H2",$R$52)</f>
         <v>H2</v>
       </c>
       <c r="X48" s="14"/>
-      <c r="Y48" s="97"/>
+      <c r="Y48" s="146"/>
       <c r="Z48" s="77"/>
-      <c r="AA48" s="97"/>
-      <c r="AB48" s="141"/>
+      <c r="AA48" s="146"/>
+      <c r="AB48" s="143"/>
       <c r="AC48" s="22" t="str">
         <f>IF(ISBLANK($X$47),"I1",$X$47)</f>
         <v>I1</v>
       </c>
       <c r="AD48" s="25"/>
-      <c r="AE48" s="109"/>
-      <c r="AF48" s="167"/>
+      <c r="AE48" s="157"/>
+      <c r="AF48" s="96"/>
       <c r="AG48" s="71"/>
       <c r="AH48" s="71"/>
       <c r="AI48" s="71"/>
@@ -5046,13 +5054,13 @@
       <c r="AL48" s="71"/>
       <c r="AM48" s="71"/>
       <c r="AN48" s="40"/>
-      <c r="AO48" s="113"/>
+      <c r="AO48" s="152"/>
     </row>
     <row r="49" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="84" t="s">
         <v>61</v>
       </c>
-      <c r="B49" s="95"/>
+      <c r="B49" s="173"/>
       <c r="C49" s="42"/>
       <c r="D49" s="79"/>
       <c r="E49" s="72"/>
@@ -5062,34 +5070,34 @@
       <c r="I49" s="72"/>
       <c r="J49" s="72"/>
       <c r="K49" s="80"/>
-      <c r="L49" s="118"/>
-      <c r="M49" s="99"/>
-      <c r="P49" s="141"/>
+      <c r="L49" s="160"/>
+      <c r="M49" s="149"/>
+      <c r="P49" s="143"/>
       <c r="Q49" s="12" t="str">
         <f>IF(ISBLANK($R$24),"B4",$R$24)</f>
         <v>B4</v>
       </c>
       <c r="R49" s="7"/>
-      <c r="S49" s="97"/>
+      <c r="S49" s="146"/>
       <c r="T49" s="71"/>
-      <c r="U49" s="97"/>
-      <c r="V49" s="102"/>
+      <c r="U49" s="146"/>
+      <c r="V49" s="99"/>
       <c r="W49" s="12" t="str">
         <f>IF(ISBLANK($X$19),"E3",$X$19)</f>
         <v>E3</v>
       </c>
       <c r="X49" s="7"/>
-      <c r="Y49" s="97"/>
+      <c r="Y49" s="146"/>
       <c r="Z49" s="77"/>
-      <c r="AA49" s="97"/>
-      <c r="AB49" s="142"/>
+      <c r="AA49" s="146"/>
+      <c r="AB49" s="144"/>
       <c r="AC49" s="22" t="str">
         <f>IF(ISBLANK($X$52),"J2",$X$52)</f>
         <v>J2</v>
       </c>
       <c r="AD49" s="24"/>
-      <c r="AE49" s="109"/>
-      <c r="AF49" s="167"/>
+      <c r="AE49" s="157"/>
+      <c r="AF49" s="96"/>
       <c r="AG49" s="71"/>
       <c r="AH49" s="71"/>
       <c r="AI49" s="71"/>
@@ -5098,13 +5106,13 @@
       <c r="AL49" s="71"/>
       <c r="AM49" s="71"/>
       <c r="AN49" s="40"/>
-      <c r="AO49" s="113"/>
+      <c r="AO49" s="152"/>
     </row>
     <row r="50" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="84" t="s">
         <v>111</v>
       </c>
-      <c r="B50" s="95"/>
+      <c r="B50" s="173"/>
       <c r="C50" s="41"/>
       <c r="D50" s="71"/>
       <c r="E50" s="73"/>
@@ -5114,27 +5122,27 @@
       <c r="I50" s="72"/>
       <c r="J50" s="72"/>
       <c r="K50" s="71"/>
-      <c r="L50" s="118"/>
-      <c r="M50" s="99"/>
-      <c r="P50" s="142"/>
+      <c r="L50" s="160"/>
+      <c r="M50" s="149"/>
+      <c r="P50" s="144"/>
       <c r="Q50" s="12" t="str">
         <f>IF(ISBLANK($R$32),"D4",$R$32)</f>
         <v>D4</v>
       </c>
       <c r="R50" s="8"/>
-      <c r="S50" s="97"/>
+      <c r="S50" s="146"/>
       <c r="T50" s="71"/>
-      <c r="U50" s="97"/>
-      <c r="V50" s="103"/>
+      <c r="U50" s="146"/>
+      <c r="V50" s="100"/>
       <c r="W50" s="12" t="str">
         <f>IF(ISBLANK($X$24),"F4",$X$24)</f>
         <v>F4</v>
       </c>
       <c r="X50" s="8"/>
-      <c r="Y50" s="97"/>
+      <c r="Y50" s="146"/>
       <c r="Z50" s="77"/>
-      <c r="AA50" s="97"/>
-      <c r="AB50" s="102" t="s">
+      <c r="AA50" s="146"/>
+      <c r="AB50" s="99" t="s">
         <v>58</v>
       </c>
       <c r="AC50" s="21" t="str">
@@ -5142,8 +5150,8 @@
         <v>WF4</v>
       </c>
       <c r="AD50" s="26"/>
-      <c r="AE50" s="109"/>
-      <c r="AF50" s="167"/>
+      <c r="AE50" s="157"/>
+      <c r="AF50" s="96"/>
       <c r="AG50" s="71"/>
       <c r="AH50" s="71"/>
       <c r="AI50" s="71"/>
@@ -5152,13 +5160,13 @@
       <c r="AL50" s="71"/>
       <c r="AM50" s="71"/>
       <c r="AN50" s="40"/>
-      <c r="AO50" s="113"/>
+      <c r="AO50" s="152"/>
     </row>
     <row r="51" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="84" t="s">
         <v>60</v>
       </c>
-      <c r="B51" s="95"/>
+      <c r="B51" s="173"/>
       <c r="C51" s="41"/>
       <c r="D51" s="71"/>
       <c r="E51" s="73"/>
@@ -5168,9 +5176,9 @@
       <c r="I51" s="72"/>
       <c r="J51" s="72"/>
       <c r="K51" s="71"/>
-      <c r="L51" s="118"/>
-      <c r="M51" s="99"/>
-      <c r="P51" s="140" t="s">
+      <c r="L51" s="160"/>
+      <c r="M51" s="149"/>
+      <c r="P51" s="142" t="s">
         <v>47</v>
       </c>
       <c r="Q51" s="11" t="str">
@@ -5178,10 +5186,10 @@
         <v>B3</v>
       </c>
       <c r="R51" s="6"/>
-      <c r="S51" s="97"/>
+      <c r="S51" s="146"/>
       <c r="T51" s="71"/>
-      <c r="U51" s="97"/>
-      <c r="V51" s="101" t="s">
+      <c r="U51" s="146"/>
+      <c r="V51" s="98" t="s">
         <v>49</v>
       </c>
       <c r="W51" s="11" t="str">
@@ -5189,17 +5197,17 @@
         <v>H1</v>
       </c>
       <c r="X51" s="6"/>
-      <c r="Y51" s="97"/>
+      <c r="Y51" s="146"/>
       <c r="Z51" s="77"/>
-      <c r="AA51" s="97"/>
-      <c r="AB51" s="102"/>
+      <c r="AA51" s="146"/>
+      <c r="AB51" s="99"/>
       <c r="AC51" s="22" t="str">
         <f>IF(ISBLANK($X$51),"J1",$X$51)</f>
         <v>J1</v>
       </c>
       <c r="AD51" s="25"/>
-      <c r="AE51" s="109"/>
-      <c r="AF51" s="167"/>
+      <c r="AE51" s="157"/>
+      <c r="AF51" s="96"/>
       <c r="AG51" s="71"/>
       <c r="AH51" s="71"/>
       <c r="AI51" s="71"/>
@@ -5208,13 +5216,13 @@
       <c r="AL51" s="71"/>
       <c r="AM51" s="71"/>
       <c r="AN51" s="40"/>
-      <c r="AO51" s="113"/>
+      <c r="AO51" s="152"/>
     </row>
     <row r="52" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="84" t="s">
         <v>136</v>
       </c>
-      <c r="B52" s="95"/>
+      <c r="B52" s="173"/>
       <c r="C52" s="41"/>
       <c r="D52" s="71"/>
       <c r="E52" s="73"/>
@@ -5224,34 +5232,34 @@
       <c r="I52" s="72"/>
       <c r="J52" s="72"/>
       <c r="K52" s="71"/>
-      <c r="L52" s="118"/>
-      <c r="M52" s="99"/>
-      <c r="P52" s="141"/>
+      <c r="L52" s="160"/>
+      <c r="M52" s="149"/>
+      <c r="P52" s="143"/>
       <c r="Q52" s="12" t="str">
         <f>IF(ISBLANK($R$31),"D3",$R$31)</f>
         <v>D3</v>
       </c>
       <c r="R52" s="14"/>
-      <c r="S52" s="97"/>
+      <c r="S52" s="146"/>
       <c r="T52" s="71"/>
-      <c r="U52" s="97"/>
-      <c r="V52" s="102"/>
+      <c r="U52" s="146"/>
+      <c r="V52" s="99"/>
       <c r="W52" s="12" t="str">
         <f>IF(ISBLANK($R$48),"G2",$R$48)</f>
         <v>G2</v>
       </c>
       <c r="X52" s="14"/>
-      <c r="Y52" s="97"/>
+      <c r="Y52" s="146"/>
       <c r="Z52" s="77"/>
-      <c r="AA52" s="98"/>
-      <c r="AB52" s="102"/>
+      <c r="AA52" s="147"/>
+      <c r="AB52" s="99"/>
       <c r="AC52" s="22" t="str">
         <f>IF(ISBLANK($X$48),"I2",$X$48)</f>
         <v>I2</v>
       </c>
       <c r="AD52" s="25"/>
-      <c r="AE52" s="110"/>
-      <c r="AF52" s="167"/>
+      <c r="AE52" s="158"/>
+      <c r="AF52" s="96"/>
       <c r="AG52" s="71"/>
       <c r="AH52" s="71"/>
       <c r="AI52" s="71"/>
@@ -5260,13 +5268,13 @@
       <c r="AL52" s="71"/>
       <c r="AM52" s="71"/>
       <c r="AN52" s="40"/>
-      <c r="AO52" s="113"/>
+      <c r="AO52" s="152"/>
     </row>
     <row r="53" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="84" t="s">
         <v>65</v>
       </c>
-      <c r="B53" s="95"/>
+      <c r="B53" s="173"/>
       <c r="C53" s="41"/>
       <c r="D53" s="71"/>
       <c r="E53" s="73"/>
@@ -5276,31 +5284,31 @@
       <c r="I53" s="72"/>
       <c r="J53" s="72"/>
       <c r="K53" s="71"/>
-      <c r="L53" s="118"/>
-      <c r="M53" s="99"/>
-      <c r="P53" s="141"/>
+      <c r="L53" s="160"/>
+      <c r="M53" s="149"/>
+      <c r="P53" s="143"/>
       <c r="Q53" s="12" t="str">
         <f>IF(ISBLANK($R$20),"A4",$R$20)</f>
         <v>A4</v>
       </c>
       <c r="R53" s="7"/>
-      <c r="S53" s="97"/>
+      <c r="S53" s="146"/>
       <c r="T53" s="71"/>
-      <c r="U53" s="97"/>
-      <c r="V53" s="102"/>
+      <c r="U53" s="146"/>
+      <c r="V53" s="99"/>
       <c r="W53" s="12" t="str">
         <f>IF(ISBLANK($X$23),"F3",$X$23)</f>
         <v>F3</v>
       </c>
       <c r="X53" s="7"/>
-      <c r="Y53" s="97"/>
+      <c r="Y53" s="146"/>
       <c r="Z53" s="77"/>
-      <c r="AA53" s="104"/>
-      <c r="AB53" s="105"/>
-      <c r="AC53" s="105"/>
-      <c r="AD53" s="105"/>
-      <c r="AE53" s="105"/>
-      <c r="AF53" s="167"/>
+      <c r="AA53" s="132"/>
+      <c r="AB53" s="130"/>
+      <c r="AC53" s="130"/>
+      <c r="AD53" s="130"/>
+      <c r="AE53" s="130"/>
+      <c r="AF53" s="96"/>
       <c r="AG53" s="71"/>
       <c r="AH53" s="71"/>
       <c r="AI53" s="71"/>
@@ -5309,13 +5317,13 @@
       <c r="AL53" s="71"/>
       <c r="AM53" s="71"/>
       <c r="AN53" s="40"/>
-      <c r="AO53" s="113"/>
+      <c r="AO53" s="152"/>
     </row>
     <row r="54" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="84" t="s">
         <v>78</v>
       </c>
-      <c r="B54" s="95"/>
+      <c r="B54" s="173"/>
       <c r="C54" s="41"/>
       <c r="D54" s="71"/>
       <c r="E54" s="73"/>
@@ -5325,31 +5333,31 @@
       <c r="I54" s="72"/>
       <c r="J54" s="72"/>
       <c r="K54" s="71"/>
-      <c r="L54" s="118"/>
-      <c r="M54" s="100"/>
-      <c r="P54" s="142"/>
+      <c r="L54" s="160"/>
+      <c r="M54" s="150"/>
+      <c r="P54" s="144"/>
       <c r="Q54" s="12" t="str">
         <f>IF(ISBLANK($R$28),"C4",$R$28)</f>
         <v>C4</v>
       </c>
       <c r="R54" s="7"/>
-      <c r="S54" s="98"/>
+      <c r="S54" s="147"/>
       <c r="T54" s="71"/>
-      <c r="U54" s="98"/>
-      <c r="V54" s="103"/>
+      <c r="U54" s="147"/>
+      <c r="V54" s="100"/>
       <c r="W54" s="13" t="str">
         <f>IF(ISBLANK($X$20),"E4",$X$20)</f>
         <v>E4</v>
       </c>
       <c r="X54" s="8"/>
-      <c r="Y54" s="98"/>
+      <c r="Y54" s="147"/>
       <c r="Z54" s="77"/>
       <c r="AA54" s="71"/>
       <c r="AB54" s="71"/>
       <c r="AC54" s="71"/>
       <c r="AD54" s="71"/>
       <c r="AE54" s="71"/>
-      <c r="AF54" s="167"/>
+      <c r="AF54" s="96"/>
       <c r="AG54" s="71"/>
       <c r="AH54" s="71"/>
       <c r="AI54" s="71"/>
@@ -5358,13 +5366,13 @@
       <c r="AL54" s="71"/>
       <c r="AM54" s="71"/>
       <c r="AN54" s="40"/>
-      <c r="AO54" s="113"/>
+      <c r="AO54" s="152"/>
     </row>
     <row r="55" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="84" t="s">
         <v>85</v>
       </c>
-      <c r="B55" s="95"/>
+      <c r="B55" s="173"/>
       <c r="C55" s="41"/>
       <c r="D55" s="71"/>
       <c r="E55" s="73"/>
@@ -5374,27 +5382,27 @@
       <c r="I55" s="72"/>
       <c r="J55" s="72"/>
       <c r="K55" s="71"/>
-      <c r="L55" s="118"/>
-      <c r="M55" s="105"/>
-      <c r="N55" s="105"/>
-      <c r="O55" s="105"/>
-      <c r="P55" s="105"/>
-      <c r="Q55" s="105"/>
-      <c r="R55" s="105"/>
-      <c r="S55" s="107"/>
+      <c r="L55" s="160"/>
+      <c r="M55" s="130"/>
+      <c r="N55" s="130"/>
+      <c r="O55" s="130"/>
+      <c r="P55" s="130"/>
+      <c r="Q55" s="130"/>
+      <c r="R55" s="130"/>
+      <c r="S55" s="131"/>
       <c r="T55" s="71"/>
-      <c r="U55" s="104"/>
-      <c r="V55" s="105"/>
-      <c r="W55" s="106"/>
-      <c r="X55" s="105"/>
-      <c r="Y55" s="107"/>
+      <c r="U55" s="132"/>
+      <c r="V55" s="130"/>
+      <c r="W55" s="162"/>
+      <c r="X55" s="130"/>
+      <c r="Y55" s="131"/>
       <c r="Z55" s="71"/>
       <c r="AA55" s="71"/>
       <c r="AB55" s="71"/>
       <c r="AC55" s="71"/>
       <c r="AD55" s="71"/>
       <c r="AE55" s="71"/>
-      <c r="AF55" s="167"/>
+      <c r="AF55" s="96"/>
       <c r="AG55" s="71"/>
       <c r="AH55" s="71"/>
       <c r="AI55" s="71"/>
@@ -5403,13 +5411,13 @@
       <c r="AL55" s="71"/>
       <c r="AM55" s="71"/>
       <c r="AN55" s="40"/>
-      <c r="AO55" s="113"/>
+      <c r="AO55" s="152"/>
     </row>
     <row r="56" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="84" t="s">
         <v>81</v>
       </c>
-      <c r="B56" s="95"/>
+      <c r="B56" s="173"/>
       <c r="C56" s="41"/>
       <c r="D56" s="71"/>
       <c r="E56" s="73"/>
@@ -5419,7 +5427,7 @@
       <c r="I56" s="72"/>
       <c r="J56" s="72"/>
       <c r="K56" s="71"/>
-      <c r="L56" s="118"/>
+      <c r="L56" s="160"/>
       <c r="M56" s="71"/>
       <c r="N56" s="71"/>
       <c r="O56" s="71"/>
@@ -5438,7 +5446,7 @@
       <c r="AB56" s="71"/>
       <c r="AD56" s="71"/>
       <c r="AE56" s="71"/>
-      <c r="AF56" s="167"/>
+      <c r="AF56" s="96"/>
       <c r="AG56" s="71"/>
       <c r="AH56" s="71"/>
       <c r="AI56" s="71"/>
@@ -5447,13 +5455,13 @@
       <c r="AL56" s="71"/>
       <c r="AM56" s="71"/>
       <c r="AN56" s="40"/>
-      <c r="AO56" s="113"/>
+      <c r="AO56" s="152"/>
     </row>
     <row r="57" spans="1:41" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A57" s="84" t="s">
         <v>80</v>
       </c>
-      <c r="B57" s="95"/>
+      <c r="B57" s="173"/>
       <c r="C57" s="43"/>
       <c r="D57" s="44"/>
       <c r="E57" s="45"/>
@@ -5463,7 +5471,7 @@
       <c r="I57" s="54"/>
       <c r="J57" s="54"/>
       <c r="K57" s="44"/>
-      <c r="L57" s="119"/>
+      <c r="L57" s="161"/>
       <c r="M57" s="44"/>
       <c r="N57" s="44"/>
       <c r="O57" s="44"/>
@@ -5483,7 +5491,7 @@
       <c r="AC57" s="44"/>
       <c r="AD57" s="44"/>
       <c r="AE57" s="44"/>
-      <c r="AF57" s="168"/>
+      <c r="AF57" s="97"/>
       <c r="AG57" s="44"/>
       <c r="AH57" s="44"/>
       <c r="AI57" s="44"/>
@@ -5492,52 +5500,52 @@
       <c r="AL57" s="44"/>
       <c r="AM57" s="44"/>
       <c r="AN57" s="46"/>
-      <c r="AO57" s="113"/>
+      <c r="AO57" s="152"/>
     </row>
     <row r="58" spans="1:41" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="84" t="s">
         <v>82</v>
       </c>
-      <c r="B58" s="95"/>
-      <c r="C58" s="115"/>
-      <c r="D58" s="115"/>
-      <c r="E58" s="115"/>
-      <c r="F58" s="115"/>
-      <c r="G58" s="115"/>
-      <c r="H58" s="115"/>
-      <c r="I58" s="115"/>
-      <c r="J58" s="115"/>
-      <c r="K58" s="115"/>
-      <c r="L58" s="115"/>
-      <c r="M58" s="115"/>
-      <c r="N58" s="115"/>
-      <c r="O58" s="115"/>
-      <c r="P58" s="115"/>
-      <c r="Q58" s="115"/>
-      <c r="R58" s="115"/>
-      <c r="S58" s="115"/>
-      <c r="T58" s="115"/>
-      <c r="U58" s="115"/>
-      <c r="V58" s="115"/>
-      <c r="W58" s="115"/>
-      <c r="X58" s="115"/>
-      <c r="Y58" s="115"/>
-      <c r="Z58" s="115"/>
-      <c r="AA58" s="115"/>
-      <c r="AB58" s="115"/>
-      <c r="AC58" s="115"/>
-      <c r="AD58" s="115"/>
-      <c r="AE58" s="115"/>
-      <c r="AF58" s="115"/>
-      <c r="AG58" s="115"/>
-      <c r="AH58" s="115"/>
-      <c r="AI58" s="115"/>
-      <c r="AJ58" s="115"/>
-      <c r="AK58" s="115"/>
-      <c r="AL58" s="115"/>
-      <c r="AM58" s="115"/>
-      <c r="AN58" s="115"/>
-      <c r="AO58" s="113"/>
+      <c r="B58" s="173"/>
+      <c r="C58" s="154"/>
+      <c r="D58" s="154"/>
+      <c r="E58" s="154"/>
+      <c r="F58" s="154"/>
+      <c r="G58" s="154"/>
+      <c r="H58" s="154"/>
+      <c r="I58" s="154"/>
+      <c r="J58" s="154"/>
+      <c r="K58" s="154"/>
+      <c r="L58" s="154"/>
+      <c r="M58" s="154"/>
+      <c r="N58" s="154"/>
+      <c r="O58" s="154"/>
+      <c r="P58" s="154"/>
+      <c r="Q58" s="154"/>
+      <c r="R58" s="154"/>
+      <c r="S58" s="154"/>
+      <c r="T58" s="154"/>
+      <c r="U58" s="154"/>
+      <c r="V58" s="154"/>
+      <c r="W58" s="154"/>
+      <c r="X58" s="154"/>
+      <c r="Y58" s="154"/>
+      <c r="Z58" s="154"/>
+      <c r="AA58" s="154"/>
+      <c r="AB58" s="154"/>
+      <c r="AC58" s="154"/>
+      <c r="AD58" s="154"/>
+      <c r="AE58" s="154"/>
+      <c r="AF58" s="154"/>
+      <c r="AG58" s="154"/>
+      <c r="AH58" s="154"/>
+      <c r="AI58" s="154"/>
+      <c r="AJ58" s="154"/>
+      <c r="AK58" s="154"/>
+      <c r="AL58" s="154"/>
+      <c r="AM58" s="154"/>
+      <c r="AN58" s="154"/>
+      <c r="AO58" s="152"/>
     </row>
     <row r="59" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="84" t="s">
@@ -5582,7 +5590,7 @@
       <c r="AL59" s="55"/>
       <c r="AM59" s="55"/>
       <c r="AN59" s="55"/>
-      <c r="AO59" s="113"/>
+      <c r="AO59" s="152"/>
     </row>
     <row r="60" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="84" t="s">
@@ -5627,7 +5635,7 @@
       <c r="AL60" s="55"/>
       <c r="AM60" s="55"/>
       <c r="AN60" s="55"/>
-      <c r="AO60" s="113"/>
+      <c r="AO60" s="152"/>
     </row>
     <row r="61" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="84" t="s">
@@ -5672,7 +5680,7 @@
       <c r="AL61" s="55"/>
       <c r="AM61" s="55"/>
       <c r="AN61" s="55"/>
-      <c r="AO61" s="113"/>
+      <c r="AO61" s="152"/>
     </row>
     <row r="62" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="84" t="s">
@@ -5717,7 +5725,7 @@
       <c r="AL62" s="55"/>
       <c r="AM62" s="55"/>
       <c r="AN62" s="55"/>
-      <c r="AO62" s="113"/>
+      <c r="AO62" s="152"/>
     </row>
     <row r="63" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="84" t="s">
@@ -5762,7 +5770,7 @@
       <c r="AL63" s="55"/>
       <c r="AM63" s="55"/>
       <c r="AN63" s="55"/>
-      <c r="AO63" s="113"/>
+      <c r="AO63" s="152"/>
     </row>
     <row r="64" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="84" t="s">
@@ -5807,7 +5815,7 @@
       <c r="AL64" s="55"/>
       <c r="AM64" s="55"/>
       <c r="AN64" s="55"/>
-      <c r="AO64" s="113"/>
+      <c r="AO64" s="152"/>
     </row>
     <row r="65" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="84" t="s">
@@ -5852,7 +5860,7 @@
       <c r="AL65" s="55"/>
       <c r="AM65" s="55"/>
       <c r="AN65" s="55"/>
-      <c r="AO65" s="113"/>
+      <c r="AO65" s="152"/>
     </row>
     <row r="66" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="84" t="s">
@@ -5897,7 +5905,7 @@
       <c r="AL66" s="55"/>
       <c r="AM66" s="55"/>
       <c r="AN66" s="55"/>
-      <c r="AO66" s="113"/>
+      <c r="AO66" s="152"/>
     </row>
     <row r="67" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="84" t="s">
@@ -5942,7 +5950,7 @@
       <c r="AL67" s="55"/>
       <c r="AM67" s="55"/>
       <c r="AN67" s="55"/>
-      <c r="AO67" s="113"/>
+      <c r="AO67" s="152"/>
     </row>
     <row r="68" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="84" t="s">
@@ -5987,7 +5995,7 @@
       <c r="AL68" s="55"/>
       <c r="AM68" s="55"/>
       <c r="AN68" s="55"/>
-      <c r="AO68" s="113"/>
+      <c r="AO68" s="152"/>
     </row>
     <row r="69" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="84" t="s">
@@ -6032,7 +6040,7 @@
       <c r="AL69" s="55"/>
       <c r="AM69" s="55"/>
       <c r="AN69" s="55"/>
-      <c r="AO69" s="113"/>
+      <c r="AO69" s="152"/>
     </row>
     <row r="70" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="84" t="s">
@@ -6077,7 +6085,7 @@
       <c r="AL70" s="55"/>
       <c r="AM70" s="55"/>
       <c r="AN70" s="55"/>
-      <c r="AO70" s="113"/>
+      <c r="AO70" s="152"/>
     </row>
     <row r="71" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="84" t="s">
@@ -6122,7 +6130,7 @@
       <c r="AL71" s="55"/>
       <c r="AM71" s="55"/>
       <c r="AN71" s="55"/>
-      <c r="AO71" s="113"/>
+      <c r="AO71" s="152"/>
     </row>
     <row r="72" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="84" t="s">
@@ -6167,7 +6175,7 @@
       <c r="AL72" s="55"/>
       <c r="AM72" s="55"/>
       <c r="AN72" s="55"/>
-      <c r="AO72" s="113"/>
+      <c r="AO72" s="152"/>
     </row>
     <row r="73" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="84" t="s">
@@ -6212,7 +6220,7 @@
       <c r="AL73" s="55"/>
       <c r="AM73" s="55"/>
       <c r="AN73" s="55"/>
-      <c r="AO73" s="113"/>
+      <c r="AO73" s="152"/>
     </row>
     <row r="74" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="84" t="s">
@@ -6257,7 +6265,7 @@
       <c r="AL74" s="55"/>
       <c r="AM74" s="55"/>
       <c r="AN74" s="55"/>
-      <c r="AO74" s="113"/>
+      <c r="AO74" s="152"/>
     </row>
     <row r="75" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="84" t="s">
@@ -6302,7 +6310,7 @@
       <c r="AL75" s="55"/>
       <c r="AM75" s="55"/>
       <c r="AN75" s="55"/>
-      <c r="AO75" s="113"/>
+      <c r="AO75" s="152"/>
     </row>
     <row r="76" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="84" t="s">
@@ -6347,7 +6355,7 @@
       <c r="AL76" s="55"/>
       <c r="AM76" s="55"/>
       <c r="AN76" s="55"/>
-      <c r="AO76" s="113"/>
+      <c r="AO76" s="152"/>
     </row>
     <row r="77" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="84" t="s">
@@ -6392,7 +6400,7 @@
       <c r="AL77" s="55"/>
       <c r="AM77" s="55"/>
       <c r="AN77" s="55"/>
-      <c r="AO77" s="113"/>
+      <c r="AO77" s="152"/>
     </row>
     <row r="78" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="84" t="s">
@@ -6437,7 +6445,7 @@
       <c r="AL78" s="55"/>
       <c r="AM78" s="55"/>
       <c r="AN78" s="55"/>
-      <c r="AO78" s="113"/>
+      <c r="AO78" s="152"/>
     </row>
     <row r="79" spans="1:41" ht="24.95" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="84" t="s">
@@ -6482,14 +6490,14 @@
       <c r="AL79" s="55"/>
       <c r="AM79" s="55"/>
       <c r="AN79" s="55"/>
-      <c r="AO79" s="113"/>
+      <c r="AO79" s="152"/>
     </row>
     <row r="80" spans="1:41" s="64" customFormat="1" ht="30" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A80" s="84" t="s">
         <v>99</v>
       </c>
       <c r="B80" s="63"/>
-      <c r="AO80" s="114"/>
+      <c r="AO80" s="153"/>
     </row>
     <row r="81" spans="1:1" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="84" t="s">
@@ -6612,37 +6620,40 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="78">
-    <mergeCell ref="H13:J14"/>
-    <mergeCell ref="D13:E14"/>
-    <mergeCell ref="AJ15:AL15"/>
-    <mergeCell ref="AJ29:AL29"/>
-    <mergeCell ref="AF2:AF57"/>
-    <mergeCell ref="P17:P20"/>
-    <mergeCell ref="P21:P24"/>
-    <mergeCell ref="P25:P28"/>
-    <mergeCell ref="P29:P32"/>
-    <mergeCell ref="U11:Y13"/>
-    <mergeCell ref="W15:X15"/>
-    <mergeCell ref="V17:V20"/>
-    <mergeCell ref="V21:V24"/>
-    <mergeCell ref="M11:S13"/>
-    <mergeCell ref="Q15:R15"/>
-    <mergeCell ref="C2:K6"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="C8:K8"/>
-    <mergeCell ref="I7:J7"/>
-    <mergeCell ref="D7:H7"/>
-    <mergeCell ref="M5:AE7"/>
-    <mergeCell ref="AA11:AE13"/>
-    <mergeCell ref="AC15:AD15"/>
-    <mergeCell ref="AB17:AB20"/>
-    <mergeCell ref="M33:S33"/>
-    <mergeCell ref="U25:Y25"/>
-    <mergeCell ref="AA21:AE21"/>
-    <mergeCell ref="AA14:AE14"/>
-    <mergeCell ref="U14:Y14"/>
+  <mergeCells count="82">
+    <mergeCell ref="P31:P32"/>
+    <mergeCell ref="AG5:AN7"/>
+    <mergeCell ref="B1:B58"/>
+    <mergeCell ref="AH29:AH34"/>
+    <mergeCell ref="AM29:AM34"/>
+    <mergeCell ref="AI31:AI34"/>
+    <mergeCell ref="AH35:AM35"/>
+    <mergeCell ref="AH28:AM28"/>
+    <mergeCell ref="AH14:AM14"/>
+    <mergeCell ref="AE15:AE20"/>
+    <mergeCell ref="AA15:AA20"/>
+    <mergeCell ref="Y15:Y24"/>
+    <mergeCell ref="AM15:AM20"/>
+    <mergeCell ref="AH15:AH20"/>
+    <mergeCell ref="U55:Y55"/>
+    <mergeCell ref="AA53:AE53"/>
+    <mergeCell ref="S45:S54"/>
+    <mergeCell ref="M45:M54"/>
+    <mergeCell ref="AO1:AO80"/>
+    <mergeCell ref="C58:AN58"/>
+    <mergeCell ref="C1:AN1"/>
+    <mergeCell ref="U15:U24"/>
+    <mergeCell ref="S15:S32"/>
+    <mergeCell ref="M15:M32"/>
+    <mergeCell ref="AE45:AE52"/>
+    <mergeCell ref="AA45:AA52"/>
+    <mergeCell ref="Y45:Y54"/>
+    <mergeCell ref="L2:L57"/>
+    <mergeCell ref="AH11:AM13"/>
+    <mergeCell ref="AI17:AI20"/>
+    <mergeCell ref="AH21:AM21"/>
+    <mergeCell ref="AH25:AM27"/>
+    <mergeCell ref="U44:Y44"/>
     <mergeCell ref="M55:S55"/>
     <mergeCell ref="M36:AE38"/>
     <mergeCell ref="U41:Y43"/>
@@ -6659,38 +6670,39 @@
     <mergeCell ref="AB47:AB49"/>
     <mergeCell ref="AB50:AB52"/>
     <mergeCell ref="AA44:AE44"/>
-    <mergeCell ref="M45:M54"/>
-    <mergeCell ref="AO1:AO80"/>
-    <mergeCell ref="C58:AN58"/>
-    <mergeCell ref="C1:AN1"/>
-    <mergeCell ref="U15:U24"/>
-    <mergeCell ref="S15:S32"/>
-    <mergeCell ref="M15:M32"/>
-    <mergeCell ref="AE45:AE52"/>
-    <mergeCell ref="AA45:AA52"/>
-    <mergeCell ref="Y45:Y54"/>
-    <mergeCell ref="L2:L57"/>
-    <mergeCell ref="AH11:AM13"/>
-    <mergeCell ref="AI17:AI20"/>
-    <mergeCell ref="AH21:AM21"/>
-    <mergeCell ref="AH25:AM27"/>
-    <mergeCell ref="U44:Y44"/>
-    <mergeCell ref="AG5:AN7"/>
-    <mergeCell ref="B1:B58"/>
-    <mergeCell ref="AH29:AH34"/>
-    <mergeCell ref="AM29:AM34"/>
-    <mergeCell ref="AI31:AI34"/>
-    <mergeCell ref="AH35:AM35"/>
-    <mergeCell ref="AH28:AM28"/>
-    <mergeCell ref="AH14:AM14"/>
-    <mergeCell ref="AE15:AE20"/>
-    <mergeCell ref="AA15:AA20"/>
-    <mergeCell ref="Y15:Y24"/>
-    <mergeCell ref="AM15:AM20"/>
-    <mergeCell ref="AH15:AH20"/>
-    <mergeCell ref="U55:Y55"/>
-    <mergeCell ref="AA53:AE53"/>
-    <mergeCell ref="S45:S54"/>
+    <mergeCell ref="M5:AE7"/>
+    <mergeCell ref="AA11:AE13"/>
+    <mergeCell ref="AC15:AD15"/>
+    <mergeCell ref="AB17:AB20"/>
+    <mergeCell ref="M33:S33"/>
+    <mergeCell ref="U25:Y25"/>
+    <mergeCell ref="AA21:AE21"/>
+    <mergeCell ref="AA14:AE14"/>
+    <mergeCell ref="U14:Y14"/>
+    <mergeCell ref="P17:P18"/>
+    <mergeCell ref="P19:P20"/>
+    <mergeCell ref="P21:P22"/>
+    <mergeCell ref="P23:P24"/>
+    <mergeCell ref="P25:P26"/>
+    <mergeCell ref="P27:P28"/>
+    <mergeCell ref="P29:P30"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="C8:K8"/>
+    <mergeCell ref="I7:J7"/>
+    <mergeCell ref="D7:H7"/>
+    <mergeCell ref="H13:J14"/>
+    <mergeCell ref="D13:E14"/>
+    <mergeCell ref="AJ15:AL15"/>
+    <mergeCell ref="AJ29:AL29"/>
+    <mergeCell ref="AF2:AF57"/>
+    <mergeCell ref="U11:Y13"/>
+    <mergeCell ref="W15:X15"/>
+    <mergeCell ref="V17:V20"/>
+    <mergeCell ref="V21:V24"/>
+    <mergeCell ref="M11:S13"/>
+    <mergeCell ref="Q15:R15"/>
+    <mergeCell ref="C2:K6"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="Q47">

</xml_diff>